<commit_message>
atualização fretes e aniversarios
</commit_message>
<xml_diff>
--- a/scripts/cargas.xlsx
+++ b/scripts/cargas.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projetos\tr.alienigenaV5-main\scripts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B92DF0D5-E987-4DFF-9AFB-84A78CFD1C3C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{B9BC6202-462C-40D9-9DDA-5E6030BF438D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" tabRatio="551" xr2:uid="{9E8F4E85-D2FF-4383-A72B-5CAFDCCC5644}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="993" uniqueCount="251">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="997" uniqueCount="234">
   <si>
     <t>Origem</t>
   </si>
@@ -80,9 +80,6 @@
     <t>Não</t>
   </si>
   <si>
-    <t>Carreta, Bitrem 7 eixos, Rodotrem</t>
-  </si>
-  <si>
     <t>Graneleiro, Caçamba</t>
   </si>
   <si>
@@ -149,18 +146,9 @@
     <t>Carreta LS, Rodotrem</t>
   </si>
   <si>
-    <t>Dias dÁvila - BA</t>
-  </si>
-  <si>
     <t>Laranjeiras - SE</t>
   </si>
   <si>
-    <t>88,00</t>
-  </si>
-  <si>
-    <t>PAGBEM</t>
-  </si>
-  <si>
     <t>São Gonçalo - RJ</t>
   </si>
   <si>
@@ -338,9 +326,6 @@
     <t>PARA CARREGAMENTO, NECESSÁRIO CHAPA E TER PALLETS, CINTA, LONA E EPI - POSSIVEIS DESTINOS DISPONIVEIS: Região de Gargalo, Vitória da Conquista e Ipiau</t>
   </si>
   <si>
-    <t>Carreta</t>
-  </si>
-  <si>
     <t>PARA CARREGAMENTO, NECESSÁRIO CHAPA E TER PALLETS, CINTA, LONA E EPI / Tem cargas todos os dias e não agregamos passantes.</t>
   </si>
   <si>
@@ -407,18 +392,6 @@
     <t>8.902,06</t>
   </si>
   <si>
-    <t>São João da Barra - RJ</t>
-  </si>
-  <si>
-    <t>Coque</t>
-  </si>
-  <si>
-    <t>13.630,00</t>
-  </si>
-  <si>
-    <t>VALOR PAGO NO CARTÃO PAGBEM / PEDÁGIO INCLUSO NO FRETE</t>
-  </si>
-  <si>
     <t>Itaguaí - RJ</t>
   </si>
   <si>
@@ -428,9 +401,6 @@
     <t>VALOR PAGO NO CARTÃO REPOM /</t>
   </si>
   <si>
-    <t>Vanderléia</t>
-  </si>
-  <si>
     <t>Trindade - PE</t>
   </si>
   <si>
@@ -449,9 +419,6 @@
     <t>Pitimbu - PB</t>
   </si>
   <si>
-    <t>Vanderléia, Bitrem 7 eixos, Rodotrem</t>
-  </si>
-  <si>
     <t>PAGBEM/REPOM</t>
   </si>
   <si>
@@ -479,15 +446,9 @@
     <t>Unaí - MG</t>
   </si>
   <si>
-    <t>Pará de Minas - MG</t>
-  </si>
-  <si>
     <t>SORGO</t>
   </si>
   <si>
-    <t>169,00</t>
-  </si>
-  <si>
     <t>Grajaú - MA</t>
   </si>
   <si>
@@ -512,9 +473,6 @@
     <t>CALCÁRIO</t>
   </si>
   <si>
-    <t>Calcario</t>
-  </si>
-  <si>
     <t>170,00</t>
   </si>
   <si>
@@ -536,9 +494,6 @@
     <t>Apenas 7 eixos acima 38 ton</t>
   </si>
   <si>
-    <t>Carreta 4º eixo</t>
-  </si>
-  <si>
     <t>130,00</t>
   </si>
   <si>
@@ -587,21 +542,9 @@
     <t>Hidrolândia - GO</t>
   </si>
   <si>
-    <t>55,00</t>
-  </si>
-  <si>
-    <t>Palmeiras de Goiás - GO</t>
-  </si>
-  <si>
     <t>Jataí - GO</t>
   </si>
   <si>
-    <t>Avelinópolis - GO</t>
-  </si>
-  <si>
-    <t>Edéia - GO</t>
-  </si>
-  <si>
     <t>Rio Verde - GO</t>
   </si>
   <si>
@@ -614,9 +557,6 @@
     <t>Montividiu - GO</t>
   </si>
   <si>
-    <t>65,00</t>
-  </si>
-  <si>
     <t>80,00</t>
   </si>
   <si>
@@ -635,18 +575,9 @@
     <t>157,00</t>
   </si>
   <si>
-    <t>Diversos</t>
-  </si>
-  <si>
     <t>Cajati - SP</t>
   </si>
   <si>
-    <t>Carreta LS, Vanderléia, Bitrem 7 eixos</t>
-  </si>
-  <si>
-    <t>Botucatu - SP</t>
-  </si>
-  <si>
     <t>Bitrem 7 eixos, Carreta 4º eixo, Rodotrem</t>
   </si>
   <si>
@@ -671,12 +602,6 @@
     <t>70,00</t>
   </si>
   <si>
-    <t>Cezarina - GO</t>
-  </si>
-  <si>
-    <t>30,00</t>
-  </si>
-  <si>
     <t>Rio Branco do Sul - PR</t>
   </si>
   <si>
@@ -713,24 +638,6 @@
     <t>115,00</t>
   </si>
   <si>
-    <t>Joinville - SC</t>
-  </si>
-  <si>
-    <t>São José - SC</t>
-  </si>
-  <si>
-    <t>Tubos e Conexões</t>
-  </si>
-  <si>
-    <t>Sider, Baú</t>
-  </si>
-  <si>
-    <t>1.150,00</t>
-  </si>
-  <si>
-    <t>precisa de MOPP ativo</t>
-  </si>
-  <si>
     <t>Castro - PR</t>
   </si>
   <si>
@@ -767,15 +674,6 @@
     <t>35,00</t>
   </si>
   <si>
-    <t>62,00</t>
-  </si>
-  <si>
-    <t>Penápolis - SP</t>
-  </si>
-  <si>
-    <t>Ureia granel</t>
-  </si>
-  <si>
     <t>Alfenas - MG</t>
   </si>
   <si>
@@ -795,6 +693,57 @@
   </si>
   <si>
     <t>Paranaíba - MS</t>
+  </si>
+  <si>
+    <t>Edealina - GO</t>
+  </si>
+  <si>
+    <t>4.670,00</t>
+  </si>
+  <si>
+    <t>Aldeias Altas - MA</t>
+  </si>
+  <si>
+    <t>190,00</t>
+  </si>
+  <si>
+    <t>Carreta LS, Carreta 4º eixo</t>
+  </si>
+  <si>
+    <t>Carreta LS, Bitrem 7 eixos, Carreta 4º eixo</t>
+  </si>
+  <si>
+    <t>Itápolis - SP</t>
+  </si>
+  <si>
+    <t>Carreta, Carreta LS</t>
+  </si>
+  <si>
+    <t>Vanderléia, Carreta 4º eixo</t>
+  </si>
+  <si>
+    <t>230,00</t>
+  </si>
+  <si>
+    <t>Cabeceira Grande - MG</t>
+  </si>
+  <si>
+    <t>Rio Pomba - MG</t>
+  </si>
+  <si>
+    <t>235,00</t>
+  </si>
+  <si>
+    <t>70,71</t>
+  </si>
+  <si>
+    <t>Bariri - SP</t>
+  </si>
+  <si>
+    <t>40,00</t>
+  </si>
+  <si>
+    <t>Caruaru - PE</t>
   </si>
 </sst>
 </file>
@@ -1197,7 +1146,7 @@
   <dimension ref="A1:J118"/>
   <sheetFormatPr defaultColWidth="12.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="24" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="25.5546875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="25.6640625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="18.44140625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="9.6640625" bestFit="1" customWidth="1"/>
@@ -1243,13 +1192,13 @@
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>149</v>
+        <v>144</v>
       </c>
       <c r="B2" t="s">
-        <v>232</v>
+        <v>217</v>
       </c>
       <c r="C2" t="s">
-        <v>108</v>
+        <v>145</v>
       </c>
       <c r="D2" t="s">
         <v>10</v>
@@ -1258,27 +1207,24 @@
         <v>11</v>
       </c>
       <c r="F2" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="G2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H2" t="s">
-        <v>233</v>
-      </c>
-      <c r="J2" s="3" t="s">
-        <v>21</v>
+        <v>218</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>149</v>
+        <v>124</v>
       </c>
       <c r="B3" t="s">
-        <v>152</v>
+        <v>25</v>
       </c>
       <c r="C3" t="s">
-        <v>108</v>
+        <v>161</v>
       </c>
       <c r="D3" t="s">
         <v>10</v>
@@ -1287,56 +1233,56 @@
         <v>11</v>
       </c>
       <c r="F3" t="s">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="G3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H3" t="s">
-        <v>215</v>
+        <v>95</v>
       </c>
       <c r="J3" s="3" t="s">
-        <v>21</v>
+        <v>125</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
+        <v>136</v>
+      </c>
+      <c r="B4" t="s">
         <v>219</v>
       </c>
-      <c r="B4" t="s">
+      <c r="C4" t="s">
+        <v>103</v>
+      </c>
+      <c r="D4" t="s">
+        <v>10</v>
+      </c>
+      <c r="E4" t="s">
+        <v>11</v>
+      </c>
+      <c r="F4" t="s">
+        <v>19</v>
+      </c>
+      <c r="G4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H4" t="s">
         <v>220</v>
       </c>
-      <c r="C4" t="s">
-        <v>221</v>
-      </c>
-      <c r="D4" t="s">
-        <v>10</v>
-      </c>
-      <c r="E4" t="s">
-        <v>11</v>
-      </c>
-      <c r="F4" t="s">
-        <v>17</v>
-      </c>
-      <c r="G4" t="s">
-        <v>14</v>
-      </c>
-      <c r="H4" t="s">
-        <v>222</v>
-      </c>
       <c r="J4" s="3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>198</v>
+        <v>136</v>
       </c>
       <c r="B5" t="s">
-        <v>216</v>
+        <v>201</v>
       </c>
       <c r="C5" t="s">
-        <v>150</v>
+        <v>103</v>
       </c>
       <c r="D5" t="s">
         <v>10</v>
@@ -1345,27 +1291,27 @@
         <v>11</v>
       </c>
       <c r="F5" t="s">
-        <v>164</v>
+        <v>19</v>
       </c>
       <c r="G5" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H5" t="s">
-        <v>217</v>
+        <v>202</v>
       </c>
       <c r="J5" s="3" t="s">
-        <v>115</v>
+        <v>20</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>198</v>
+        <v>194</v>
       </c>
       <c r="B6" t="s">
-        <v>216</v>
+        <v>195</v>
       </c>
       <c r="C6" t="s">
-        <v>150</v>
+        <v>196</v>
       </c>
       <c r="D6" t="s">
         <v>10</v>
@@ -1374,27 +1320,27 @@
         <v>11</v>
       </c>
       <c r="F6" t="s">
-        <v>199</v>
+        <v>16</v>
       </c>
       <c r="G6" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H6" t="s">
-        <v>217</v>
+        <v>197</v>
       </c>
       <c r="J6" s="3" t="s">
-        <v>115</v>
+        <v>20</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>198</v>
+        <v>177</v>
       </c>
       <c r="B7" t="s">
-        <v>211</v>
+        <v>191</v>
       </c>
       <c r="C7" t="s">
-        <v>150</v>
+        <v>137</v>
       </c>
       <c r="D7" t="s">
         <v>10</v>
@@ -1403,27 +1349,27 @@
         <v>11</v>
       </c>
       <c r="F7" t="s">
-        <v>212</v>
+        <v>221</v>
       </c>
       <c r="G7" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H7" t="s">
-        <v>213</v>
+        <v>192</v>
       </c>
       <c r="J7" s="3" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>198</v>
+        <v>177</v>
       </c>
       <c r="B8" t="s">
-        <v>211</v>
+        <v>191</v>
       </c>
       <c r="C8" t="s">
-        <v>150</v>
+        <v>137</v>
       </c>
       <c r="D8" t="s">
         <v>10</v>
@@ -1432,27 +1378,27 @@
         <v>11</v>
       </c>
       <c r="F8" t="s">
-        <v>201</v>
+        <v>187</v>
       </c>
       <c r="G8" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H8" t="s">
-        <v>213</v>
+        <v>192</v>
       </c>
       <c r="J8" s="3" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>198</v>
+        <v>177</v>
       </c>
       <c r="B9" t="s">
-        <v>214</v>
+        <v>186</v>
       </c>
       <c r="C9" t="s">
-        <v>150</v>
+        <v>137</v>
       </c>
       <c r="D9" t="s">
         <v>10</v>
@@ -1461,27 +1407,27 @@
         <v>11</v>
       </c>
       <c r="F9" t="s">
-        <v>201</v>
+        <v>187</v>
       </c>
       <c r="G9" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H9" t="s">
-        <v>213</v>
+        <v>188</v>
       </c>
       <c r="J9" s="3" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>106</v>
+        <v>177</v>
       </c>
       <c r="B10" t="s">
-        <v>200</v>
+        <v>186</v>
       </c>
       <c r="C10" t="s">
-        <v>108</v>
+        <v>137</v>
       </c>
       <c r="D10" t="s">
         <v>10</v>
@@ -1490,27 +1436,27 @@
         <v>11</v>
       </c>
       <c r="F10" t="s">
-        <v>201</v>
+        <v>222</v>
       </c>
       <c r="G10" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H10" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="J10" s="3" t="s">
-        <v>21</v>
+        <v>110</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>106</v>
+        <v>177</v>
       </c>
       <c r="B11" t="s">
-        <v>202</v>
+        <v>189</v>
       </c>
       <c r="C11" t="s">
-        <v>108</v>
+        <v>137</v>
       </c>
       <c r="D11" t="s">
         <v>10</v>
@@ -1519,27 +1465,27 @@
         <v>11</v>
       </c>
       <c r="F11" t="s">
-        <v>201</v>
+        <v>55</v>
       </c>
       <c r="G11" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H11" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="J11" s="3" t="s">
-        <v>21</v>
+        <v>110</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>106</v>
+        <v>101</v>
       </c>
       <c r="B12" t="s">
-        <v>107</v>
+        <v>223</v>
       </c>
       <c r="C12" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="D12" t="s">
         <v>10</v>
@@ -1548,27 +1494,27 @@
         <v>11</v>
       </c>
       <c r="F12" t="s">
-        <v>201</v>
+        <v>27</v>
       </c>
       <c r="G12" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H12" t="s">
-        <v>109</v>
+        <v>190</v>
       </c>
       <c r="J12" s="3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>36</v>
+        <v>101</v>
       </c>
       <c r="B13" t="s">
-        <v>26</v>
+        <v>179</v>
       </c>
       <c r="C13" t="s">
-        <v>24</v>
+        <v>103</v>
       </c>
       <c r="D13" t="s">
         <v>10</v>
@@ -1577,56 +1523,56 @@
         <v>11</v>
       </c>
       <c r="F13" t="s">
-        <v>16</v>
+        <v>27</v>
       </c>
       <c r="G13" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H13" t="s">
-        <v>110</v>
+        <v>171</v>
       </c>
       <c r="J13" s="3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>223</v>
+        <v>101</v>
       </c>
       <c r="B14" t="s">
-        <v>224</v>
+        <v>102</v>
       </c>
       <c r="C14" t="s">
-        <v>225</v>
+        <v>103</v>
       </c>
       <c r="D14" t="s">
-        <v>197</v>
+        <v>10</v>
       </c>
       <c r="E14" t="s">
         <v>11</v>
       </c>
       <c r="F14" t="s">
-        <v>18</v>
+        <v>27</v>
       </c>
       <c r="G14" t="s">
-        <v>226</v>
+        <v>13</v>
       </c>
       <c r="H14" t="s">
-        <v>227</v>
+        <v>104</v>
       </c>
       <c r="J14" s="3" t="s">
-        <v>228</v>
+        <v>20</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>111</v>
+        <v>34</v>
       </c>
       <c r="B15" t="s">
-        <v>112</v>
+        <v>25</v>
       </c>
       <c r="C15" t="s">
-        <v>113</v>
+        <v>23</v>
       </c>
       <c r="D15" t="s">
         <v>10</v>
@@ -1635,27 +1581,27 @@
         <v>11</v>
       </c>
       <c r="F15" t="s">
+        <v>55</v>
+      </c>
+      <c r="G15" t="s">
+        <v>13</v>
+      </c>
+      <c r="H15" t="s">
+        <v>105</v>
+      </c>
+      <c r="J15" s="3" t="s">
         <v>20</v>
-      </c>
-      <c r="G15" t="s">
-        <v>14</v>
-      </c>
-      <c r="H15" t="s">
-        <v>114</v>
-      </c>
-      <c r="J15" s="3" t="s">
-        <v>115</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>116</v>
+        <v>106</v>
       </c>
       <c r="B16" t="s">
-        <v>117</v>
+        <v>107</v>
       </c>
       <c r="C16" t="s">
-        <v>118</v>
+        <v>108</v>
       </c>
       <c r="D16" t="s">
         <v>10</v>
@@ -1664,16 +1610,16 @@
         <v>11</v>
       </c>
       <c r="F16" t="s">
-        <v>20</v>
+        <v>33</v>
       </c>
       <c r="G16" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H16" t="s">
-        <v>119</v>
+        <v>109</v>
       </c>
       <c r="J16" s="3" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.3">
@@ -1693,27 +1639,27 @@
         <v>11</v>
       </c>
       <c r="F17" t="s">
-        <v>22</v>
+        <v>33</v>
       </c>
       <c r="G17" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H17" t="s">
-        <v>120</v>
+        <v>114</v>
       </c>
       <c r="J17" s="3" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>125</v>
+        <v>106</v>
       </c>
       <c r="B18" t="s">
-        <v>126</v>
+        <v>107</v>
       </c>
       <c r="C18" t="s">
-        <v>23</v>
+        <v>108</v>
       </c>
       <c r="D18" t="s">
         <v>10</v>
@@ -1722,30 +1668,27 @@
         <v>11</v>
       </c>
       <c r="F18" t="s">
-        <v>164</v>
+        <v>55</v>
       </c>
       <c r="G18" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H18" t="s">
-        <v>165</v>
-      </c>
-      <c r="I18" s="3">
-        <v>28000</v>
+        <v>115</v>
       </c>
       <c r="J18" s="3" t="s">
-        <v>127</v>
+        <v>110</v>
       </c>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>125</v>
+        <v>116</v>
       </c>
       <c r="B19" t="s">
-        <v>105</v>
+        <v>117</v>
       </c>
       <c r="C19" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D19" t="s">
         <v>10</v>
@@ -1754,30 +1697,30 @@
         <v>11</v>
       </c>
       <c r="F19" t="s">
-        <v>164</v>
+        <v>221</v>
       </c>
       <c r="G19" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H19" t="s">
-        <v>165</v>
+        <v>150</v>
       </c>
       <c r="I19" s="3">
         <v>28000</v>
       </c>
       <c r="J19" s="3" t="s">
-        <v>127</v>
+        <v>118</v>
       </c>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>121</v>
+        <v>116</v>
       </c>
       <c r="B20" t="s">
-        <v>79</v>
+        <v>100</v>
       </c>
       <c r="C20" t="s">
-        <v>122</v>
+        <v>22</v>
       </c>
       <c r="D20" t="s">
         <v>10</v>
@@ -1786,27 +1729,30 @@
         <v>11</v>
       </c>
       <c r="F20" t="s">
-        <v>20</v>
+        <v>221</v>
       </c>
       <c r="G20" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H20" t="s">
-        <v>123</v>
+        <v>150</v>
+      </c>
+      <c r="I20" s="3">
+        <v>28000</v>
       </c>
       <c r="J20" s="3" t="s">
-        <v>124</v>
+        <v>118</v>
       </c>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>125</v>
+        <v>116</v>
       </c>
       <c r="B21" t="s">
-        <v>126</v>
+        <v>117</v>
       </c>
       <c r="C21" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D21" t="s">
         <v>10</v>
@@ -1815,30 +1761,30 @@
         <v>11</v>
       </c>
       <c r="F21" t="s">
-        <v>20</v>
+        <v>33</v>
       </c>
       <c r="G21" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H21" t="s">
-        <v>166</v>
+        <v>151</v>
       </c>
       <c r="I21" s="3">
         <v>28000</v>
       </c>
       <c r="J21" s="3" t="s">
-        <v>127</v>
+        <v>118</v>
       </c>
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>125</v>
+        <v>116</v>
       </c>
       <c r="B22" t="s">
-        <v>126</v>
+        <v>117</v>
       </c>
       <c r="C22" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D22" t="s">
         <v>10</v>
@@ -1847,30 +1793,30 @@
         <v>11</v>
       </c>
       <c r="F22" t="s">
-        <v>22</v>
+        <v>55</v>
       </c>
       <c r="G22" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H22" t="s">
-        <v>165</v>
+        <v>150</v>
       </c>
       <c r="I22" s="3">
         <v>28000</v>
       </c>
       <c r="J22" s="3" t="s">
-        <v>127</v>
+        <v>118</v>
       </c>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>125</v>
+        <v>116</v>
       </c>
       <c r="B23" t="s">
-        <v>105</v>
+        <v>100</v>
       </c>
       <c r="C23" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D23" t="s">
         <v>10</v>
@@ -1879,30 +1825,30 @@
         <v>11</v>
       </c>
       <c r="F23" t="s">
-        <v>20</v>
+        <v>33</v>
       </c>
       <c r="G23" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H23" t="s">
-        <v>166</v>
+        <v>151</v>
       </c>
       <c r="I23" s="3">
         <v>28000</v>
       </c>
       <c r="J23" s="3" t="s">
-        <v>127</v>
+        <v>118</v>
       </c>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>125</v>
+        <v>116</v>
       </c>
       <c r="B24" t="s">
-        <v>105</v>
+        <v>100</v>
       </c>
       <c r="C24" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D24" t="s">
         <v>10</v>
@@ -1911,30 +1857,30 @@
         <v>11</v>
       </c>
       <c r="F24" t="s">
-        <v>22</v>
+        <v>55</v>
       </c>
       <c r="G24" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H24" t="s">
-        <v>165</v>
+        <v>150</v>
       </c>
       <c r="I24" s="3">
         <v>28000</v>
       </c>
       <c r="J24" s="3" t="s">
-        <v>127</v>
+        <v>118</v>
       </c>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>129</v>
+        <v>119</v>
       </c>
       <c r="B25" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="C25" t="s">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="D25" t="s">
         <v>10</v>
@@ -1943,27 +1889,27 @@
         <v>11</v>
       </c>
       <c r="F25" t="s">
+        <v>33</v>
+      </c>
+      <c r="G25" t="s">
+        <v>13</v>
+      </c>
+      <c r="H25" t="s">
+        <v>152</v>
+      </c>
+      <c r="J25" s="3" t="s">
         <v>20</v>
-      </c>
-      <c r="G25" t="s">
-        <v>14</v>
-      </c>
-      <c r="H25" t="s">
-        <v>167</v>
-      </c>
-      <c r="J25" s="3" t="s">
-        <v>21</v>
       </c>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>129</v>
+        <v>119</v>
       </c>
       <c r="B26" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="C26" t="s">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="D26" t="s">
         <v>10</v>
@@ -1972,27 +1918,27 @@
         <v>11</v>
       </c>
       <c r="F26" t="s">
-        <v>164</v>
+        <v>221</v>
       </c>
       <c r="G26" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H26" t="s">
-        <v>168</v>
+        <v>153</v>
       </c>
       <c r="J26" s="3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>129</v>
+        <v>119</v>
       </c>
       <c r="B27" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="C27" t="s">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="D27" t="s">
         <v>10</v>
@@ -2001,27 +1947,27 @@
         <v>11</v>
       </c>
       <c r="F27" t="s">
-        <v>22</v>
+        <v>55</v>
       </c>
       <c r="G27" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H27" t="s">
-        <v>168</v>
+        <v>153</v>
       </c>
       <c r="J27" s="3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>129</v>
+        <v>119</v>
       </c>
       <c r="B28" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="C28" t="s">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="D28" t="s">
         <v>10</v>
@@ -2030,27 +1976,27 @@
         <v>11</v>
       </c>
       <c r="F28" t="s">
-        <v>128</v>
+        <v>187</v>
       </c>
       <c r="G28" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H28" t="s">
-        <v>169</v>
+        <v>154</v>
       </c>
       <c r="J28" s="3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>129</v>
+        <v>119</v>
       </c>
       <c r="B29" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="C29" t="s">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="D29" t="s">
         <v>10</v>
@@ -2059,27 +2005,27 @@
         <v>11</v>
       </c>
       <c r="F29" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="G29" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H29" t="s">
-        <v>169</v>
+        <v>154</v>
       </c>
       <c r="J29" s="3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>129</v>
+        <v>119</v>
       </c>
       <c r="B30" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="C30" t="s">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="D30" t="s">
         <v>10</v>
@@ -2088,56 +2034,56 @@
         <v>11</v>
       </c>
       <c r="F30" t="s">
-        <v>98</v>
+        <v>224</v>
       </c>
       <c r="G30" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H30" t="s">
-        <v>170</v>
+        <v>155</v>
       </c>
       <c r="J30" s="3" t="s">
-        <v>171</v>
+        <v>156</v>
       </c>
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>129</v>
+        <v>119</v>
       </c>
       <c r="B31" t="s">
+        <v>32</v>
+      </c>
+      <c r="C31" t="s">
+        <v>120</v>
+      </c>
+      <c r="D31" t="s">
+        <v>10</v>
+      </c>
+      <c r="E31" t="s">
+        <v>11</v>
+      </c>
+      <c r="F31" t="s">
         <v>33</v>
       </c>
-      <c r="C31" t="s">
-        <v>130</v>
-      </c>
-      <c r="D31" t="s">
-        <v>10</v>
-      </c>
-      <c r="E31" t="s">
-        <v>11</v>
-      </c>
-      <c r="F31" t="s">
+      <c r="G31" t="s">
+        <v>13</v>
+      </c>
+      <c r="H31" t="s">
+        <v>157</v>
+      </c>
+      <c r="J31" s="3" t="s">
         <v>20</v>
-      </c>
-      <c r="G31" t="s">
-        <v>14</v>
-      </c>
-      <c r="H31" t="s">
-        <v>172</v>
-      </c>
-      <c r="J31" s="3" t="s">
-        <v>21</v>
       </c>
     </row>
     <row r="32" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>129</v>
+        <v>119</v>
       </c>
       <c r="B32" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C32" t="s">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="D32" t="s">
         <v>10</v>
@@ -2146,27 +2092,27 @@
         <v>11</v>
       </c>
       <c r="F32" t="s">
-        <v>164</v>
+        <v>221</v>
       </c>
       <c r="G32" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H32" t="s">
-        <v>173</v>
+        <v>158</v>
       </c>
       <c r="J32" s="3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="33" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
-        <v>129</v>
+        <v>119</v>
       </c>
       <c r="B33" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C33" t="s">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="D33" t="s">
         <v>10</v>
@@ -2175,27 +2121,27 @@
         <v>11</v>
       </c>
       <c r="F33" t="s">
-        <v>22</v>
+        <v>55</v>
       </c>
       <c r="G33" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H33" t="s">
-        <v>173</v>
+        <v>158</v>
       </c>
       <c r="J33" s="3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="34" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>129</v>
+        <v>119</v>
       </c>
       <c r="B34" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C34" t="s">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="D34" t="s">
         <v>10</v>
@@ -2204,27 +2150,27 @@
         <v>11</v>
       </c>
       <c r="F34" t="s">
-        <v>128</v>
+        <v>187</v>
       </c>
       <c r="G34" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H34" t="s">
-        <v>174</v>
+        <v>159</v>
       </c>
       <c r="J34" s="3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="35" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
-        <v>129</v>
+        <v>119</v>
       </c>
       <c r="B35" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C35" t="s">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="D35" t="s">
         <v>10</v>
@@ -2233,27 +2179,27 @@
         <v>11</v>
       </c>
       <c r="F35" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="G35" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H35" t="s">
-        <v>174</v>
+        <v>159</v>
       </c>
       <c r="J35" s="3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="36" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>129</v>
+        <v>119</v>
       </c>
       <c r="B36" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C36" t="s">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="D36" t="s">
         <v>10</v>
@@ -2262,27 +2208,27 @@
         <v>11</v>
       </c>
       <c r="F36" t="s">
-        <v>98</v>
+        <v>224</v>
       </c>
       <c r="G36" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H36" t="s">
-        <v>175</v>
+        <v>160</v>
       </c>
       <c r="J36" s="3" t="s">
-        <v>171</v>
+        <v>156</v>
       </c>
     </row>
     <row r="37" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>131</v>
+        <v>121</v>
       </c>
       <c r="B37" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C37" t="s">
-        <v>132</v>
+        <v>122</v>
       </c>
       <c r="D37" t="s">
         <v>10</v>
@@ -2291,27 +2237,27 @@
         <v>11</v>
       </c>
       <c r="F37" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="G37" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="H37" t="s">
-        <v>133</v>
+        <v>123</v>
       </c>
       <c r="J37" s="3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="38" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>131</v>
+        <v>121</v>
       </c>
       <c r="B38" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="C38" t="s">
-        <v>132</v>
+        <v>122</v>
       </c>
       <c r="D38" t="s">
         <v>10</v>
@@ -2320,30 +2266,30 @@
         <v>11</v>
       </c>
       <c r="F38" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="G38" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H38" t="s">
-        <v>133</v>
+        <v>123</v>
       </c>
       <c r="I38" s="3">
         <v>52</v>
       </c>
       <c r="J38" s="3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="39" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>134</v>
+        <v>126</v>
       </c>
       <c r="B39" t="s">
-        <v>26</v>
+        <v>127</v>
       </c>
       <c r="C39" t="s">
-        <v>176</v>
+        <v>128</v>
       </c>
       <c r="D39" t="s">
         <v>10</v>
@@ -2352,27 +2298,27 @@
         <v>11</v>
       </c>
       <c r="F39" t="s">
-        <v>135</v>
+        <v>33</v>
       </c>
       <c r="G39" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H39" t="s">
-        <v>100</v>
+        <v>193</v>
       </c>
       <c r="J39" s="3" t="s">
-        <v>136</v>
+        <v>129</v>
       </c>
     </row>
     <row r="40" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>137</v>
+        <v>28</v>
       </c>
       <c r="B40" t="s">
-        <v>138</v>
+        <v>130</v>
       </c>
       <c r="C40" t="s">
-        <v>139</v>
+        <v>131</v>
       </c>
       <c r="D40" t="s">
         <v>10</v>
@@ -2381,27 +2327,27 @@
         <v>11</v>
       </c>
       <c r="F40" t="s">
-        <v>20</v>
+        <v>33</v>
       </c>
       <c r="G40" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H40" t="s">
-        <v>218</v>
+        <v>132</v>
       </c>
       <c r="J40" s="3" t="s">
-        <v>140</v>
+        <v>129</v>
       </c>
     </row>
     <row r="41" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
-        <v>29</v>
+        <v>227</v>
       </c>
       <c r="B41" t="s">
-        <v>141</v>
+        <v>228</v>
       </c>
       <c r="C41" t="s">
-        <v>142</v>
+        <v>134</v>
       </c>
       <c r="D41" t="s">
         <v>10</v>
@@ -2410,27 +2356,27 @@
         <v>11</v>
       </c>
       <c r="F41" t="s">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="G41" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="H41" t="s">
-        <v>143</v>
+        <v>229</v>
       </c>
       <c r="J41" s="3" t="s">
-        <v>140</v>
+        <v>125</v>
       </c>
     </row>
     <row r="42" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
-        <v>194</v>
+        <v>227</v>
       </c>
       <c r="B42" t="s">
-        <v>195</v>
+        <v>228</v>
       </c>
       <c r="C42" t="s">
-        <v>146</v>
+        <v>134</v>
       </c>
       <c r="D42" t="s">
         <v>10</v>
@@ -2439,27 +2385,27 @@
         <v>11</v>
       </c>
       <c r="F42" t="s">
+        <v>225</v>
+      </c>
+      <c r="G42" t="s">
         <v>12</v>
       </c>
-      <c r="G42" t="s">
-        <v>13</v>
-      </c>
       <c r="H42" t="s">
-        <v>196</v>
+        <v>229</v>
       </c>
       <c r="J42" s="3" t="s">
-        <v>136</v>
+        <v>125</v>
       </c>
     </row>
     <row r="43" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
-        <v>144</v>
+        <v>133</v>
       </c>
       <c r="B43" t="s">
-        <v>192</v>
+        <v>228</v>
       </c>
       <c r="C43" t="s">
-        <v>146</v>
+        <v>134</v>
       </c>
       <c r="D43" t="s">
         <v>10</v>
@@ -2468,27 +2414,27 @@
         <v>11</v>
       </c>
       <c r="F43" t="s">
+        <v>225</v>
+      </c>
+      <c r="G43" t="s">
         <v>12</v>
       </c>
-      <c r="G43" t="s">
-        <v>13</v>
-      </c>
       <c r="H43" t="s">
-        <v>193</v>
+        <v>226</v>
       </c>
       <c r="J43" s="3" t="s">
-        <v>136</v>
+        <v>125</v>
       </c>
     </row>
     <row r="44" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
-        <v>144</v>
+        <v>133</v>
       </c>
       <c r="B44" t="s">
-        <v>145</v>
+        <v>228</v>
       </c>
       <c r="C44" t="s">
-        <v>146</v>
+        <v>134</v>
       </c>
       <c r="D44" t="s">
         <v>10</v>
@@ -2497,85 +2443,85 @@
         <v>11</v>
       </c>
       <c r="F44" t="s">
+        <v>27</v>
+      </c>
+      <c r="G44" t="s">
         <v>12</v>
       </c>
-      <c r="G44" t="s">
-        <v>13</v>
-      </c>
       <c r="H44" t="s">
-        <v>147</v>
+        <v>226</v>
       </c>
       <c r="J44" s="3" t="s">
-        <v>136</v>
+        <v>125</v>
       </c>
     </row>
     <row r="45" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
-        <v>148</v>
+        <v>174</v>
       </c>
       <c r="B45" t="s">
-        <v>149</v>
+        <v>175</v>
       </c>
       <c r="C45" t="s">
-        <v>150</v>
+        <v>134</v>
       </c>
       <c r="D45" t="s">
-        <v>151</v>
+        <v>10</v>
       </c>
       <c r="E45" t="s">
         <v>11</v>
       </c>
       <c r="F45" t="s">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="G45" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="H45" t="s">
-        <v>203</v>
-      </c>
-      <c r="I45" s="3">
-        <v>49</v>
+        <v>176</v>
+      </c>
+      <c r="J45" s="3" t="s">
+        <v>125</v>
       </c>
     </row>
     <row r="46" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
-        <v>152</v>
+        <v>174</v>
       </c>
       <c r="B46" t="s">
-        <v>27</v>
+        <v>175</v>
       </c>
       <c r="C46" t="s">
-        <v>23</v>
+        <v>134</v>
       </c>
       <c r="D46" t="s">
-        <v>151</v>
+        <v>10</v>
       </c>
       <c r="E46" t="s">
         <v>11</v>
       </c>
       <c r="F46" t="s">
-        <v>28</v>
+        <v>225</v>
       </c>
       <c r="G46" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="H46" t="s">
-        <v>153</v>
-      </c>
-      <c r="I46" s="3">
-        <v>49</v>
+        <v>176</v>
+      </c>
+      <c r="J46" s="3" t="s">
+        <v>125</v>
       </c>
     </row>
     <row r="47" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
-        <v>158</v>
+        <v>133</v>
       </c>
       <c r="B47" t="s">
-        <v>105</v>
+        <v>172</v>
       </c>
       <c r="C47" t="s">
-        <v>159</v>
+        <v>134</v>
       </c>
       <c r="D47" t="s">
         <v>10</v>
@@ -2584,24 +2530,27 @@
         <v>11</v>
       </c>
       <c r="F47" t="s">
-        <v>20</v>
+        <v>225</v>
       </c>
       <c r="G47" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="H47" t="s">
-        <v>160</v>
+        <v>173</v>
+      </c>
+      <c r="J47" s="3" t="s">
+        <v>125</v>
       </c>
     </row>
     <row r="48" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
-        <v>158</v>
+        <v>133</v>
       </c>
       <c r="B48" t="s">
-        <v>105</v>
+        <v>172</v>
       </c>
       <c r="C48" t="s">
-        <v>159</v>
+        <v>134</v>
       </c>
       <c r="D48" t="s">
         <v>10</v>
@@ -2610,114 +2559,114 @@
         <v>11</v>
       </c>
       <c r="F48" t="s">
-        <v>161</v>
+        <v>27</v>
       </c>
       <c r="G48" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="H48" t="s">
-        <v>162</v>
+        <v>173</v>
       </c>
       <c r="J48" s="3" t="s">
-        <v>163</v>
+        <v>125</v>
       </c>
     </row>
     <row r="49" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
-        <v>32</v>
+        <v>139</v>
       </c>
       <c r="B49" t="s">
-        <v>27</v>
+        <v>136</v>
       </c>
       <c r="C49" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D49" t="s">
-        <v>10</v>
+        <v>138</v>
       </c>
       <c r="E49" t="s">
         <v>11</v>
       </c>
       <c r="F49" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="G49" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H49" t="s">
-        <v>234</v>
-      </c>
-      <c r="J49" s="3" t="s">
-        <v>235</v>
+        <v>171</v>
+      </c>
+      <c r="I49" s="3">
+        <v>49</v>
       </c>
     </row>
     <row r="50" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
-        <v>33</v>
+        <v>135</v>
       </c>
       <c r="B50" t="s">
-        <v>27</v>
+        <v>136</v>
       </c>
       <c r="C50" t="s">
-        <v>156</v>
+        <v>137</v>
       </c>
       <c r="D50" t="s">
-        <v>10</v>
+        <v>138</v>
       </c>
       <c r="E50" t="s">
         <v>11</v>
       </c>
       <c r="F50" t="s">
-        <v>34</v>
+        <v>19</v>
       </c>
       <c r="G50" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H50" t="s">
-        <v>157</v>
-      </c>
-      <c r="J50" s="3" t="s">
-        <v>21</v>
+        <v>180</v>
+      </c>
+      <c r="I50" s="3">
+        <v>49</v>
       </c>
     </row>
     <row r="51" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
-        <v>35</v>
+        <v>139</v>
       </c>
       <c r="B51" t="s">
-        <v>36</v>
+        <v>26</v>
       </c>
       <c r="C51" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D51" t="s">
-        <v>10</v>
+        <v>138</v>
       </c>
       <c r="E51" t="s">
         <v>11</v>
       </c>
       <c r="F51" t="s">
-        <v>16</v>
+        <v>27</v>
       </c>
       <c r="G51" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H51" t="s">
-        <v>37</v>
-      </c>
-      <c r="J51" s="3" t="s">
-        <v>38</v>
+        <v>140</v>
+      </c>
+      <c r="I51" s="3">
+        <v>49</v>
       </c>
     </row>
     <row r="52" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
-        <v>229</v>
+        <v>144</v>
       </c>
       <c r="B52" t="s">
-        <v>230</v>
+        <v>100</v>
       </c>
       <c r="C52" t="s">
-        <v>155</v>
+        <v>145</v>
       </c>
       <c r="D52" t="s">
         <v>10</v>
@@ -2726,21 +2675,24 @@
         <v>11</v>
       </c>
       <c r="F52" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="G52" t="s">
-        <v>14</v>
+        <v>13</v>
+      </c>
+      <c r="H52" t="s">
+        <v>146</v>
       </c>
     </row>
     <row r="53" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
-        <v>236</v>
+        <v>144</v>
       </c>
       <c r="B53" t="s">
-        <v>187</v>
+        <v>100</v>
       </c>
       <c r="C53" t="s">
-        <v>31</v>
+        <v>145</v>
       </c>
       <c r="D53" t="s">
         <v>10</v>
@@ -2749,24 +2701,27 @@
         <v>11</v>
       </c>
       <c r="F53" t="s">
-        <v>28</v>
+        <v>147</v>
       </c>
       <c r="G53" t="s">
         <v>13</v>
       </c>
       <c r="H53" t="s">
-        <v>237</v>
+        <v>148</v>
+      </c>
+      <c r="J53" s="3" t="s">
+        <v>149</v>
       </c>
     </row>
     <row r="54" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
-        <v>189</v>
+        <v>31</v>
       </c>
       <c r="B54" t="s">
-        <v>238</v>
+        <v>32</v>
       </c>
       <c r="C54" t="s">
-        <v>31</v>
+        <v>22</v>
       </c>
       <c r="D54" t="s">
         <v>10</v>
@@ -2775,24 +2730,27 @@
         <v>11</v>
       </c>
       <c r="F54" t="s">
-        <v>28</v>
+        <v>19</v>
       </c>
       <c r="G54" t="s">
         <v>13</v>
       </c>
       <c r="H54" t="s">
-        <v>239</v>
+        <v>230</v>
+      </c>
+      <c r="J54" s="3" t="s">
+        <v>204</v>
       </c>
     </row>
     <row r="55" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
-        <v>189</v>
+        <v>31</v>
       </c>
       <c r="B55" t="s">
-        <v>186</v>
+        <v>26</v>
       </c>
       <c r="C55" t="s">
-        <v>31</v>
+        <v>22</v>
       </c>
       <c r="D55" t="s">
         <v>10</v>
@@ -2801,24 +2759,27 @@
         <v>11</v>
       </c>
       <c r="F55" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="G55" t="s">
         <v>13</v>
       </c>
       <c r="H55" t="s">
-        <v>240</v>
+        <v>203</v>
+      </c>
+      <c r="J55" s="3" t="s">
+        <v>204</v>
       </c>
     </row>
     <row r="56" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
-        <v>177</v>
+        <v>198</v>
       </c>
       <c r="B56" t="s">
-        <v>178</v>
+        <v>199</v>
       </c>
       <c r="C56" t="s">
-        <v>179</v>
+        <v>142</v>
       </c>
       <c r="D56" t="s">
         <v>10</v>
@@ -2827,24 +2788,21 @@
         <v>11</v>
       </c>
       <c r="F56" t="s">
-        <v>28</v>
+        <v>19</v>
       </c>
       <c r="G56" t="s">
         <v>13</v>
-      </c>
-      <c r="H56" t="s">
-        <v>231</v>
       </c>
     </row>
     <row r="57" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
-        <v>207</v>
+        <v>199</v>
       </c>
       <c r="B57" t="s">
-        <v>180</v>
+        <v>231</v>
       </c>
       <c r="C57" t="s">
-        <v>179</v>
+        <v>30</v>
       </c>
       <c r="D57" t="s">
         <v>10</v>
@@ -2853,24 +2811,24 @@
         <v>11</v>
       </c>
       <c r="F57" t="s">
-        <v>28</v>
+        <v>19</v>
       </c>
       <c r="G57" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H57" t="s">
-        <v>208</v>
+        <v>143</v>
       </c>
     </row>
     <row r="58" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
-        <v>183</v>
+        <v>170</v>
       </c>
       <c r="B58" t="s">
-        <v>187</v>
+        <v>207</v>
       </c>
       <c r="C58" t="s">
-        <v>179</v>
+        <v>30</v>
       </c>
       <c r="D58" t="s">
         <v>10</v>
@@ -2879,24 +2837,24 @@
         <v>11</v>
       </c>
       <c r="F58" t="s">
-        <v>15</v>
+        <v>27</v>
       </c>
       <c r="G58" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="H58" t="s">
-        <v>190</v>
+        <v>208</v>
       </c>
     </row>
     <row r="59" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
-        <v>183</v>
+        <v>170</v>
       </c>
       <c r="B59" t="s">
-        <v>178</v>
+        <v>167</v>
       </c>
       <c r="C59" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D59" t="s">
         <v>10</v>
@@ -2905,24 +2863,24 @@
         <v>11</v>
       </c>
       <c r="F59" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="G59" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="H59" t="s">
-        <v>241</v>
+        <v>209</v>
       </c>
     </row>
     <row r="60" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
-        <v>209</v>
+        <v>162</v>
       </c>
       <c r="B60" t="s">
-        <v>182</v>
+        <v>163</v>
       </c>
       <c r="C60" t="s">
-        <v>31</v>
+        <v>164</v>
       </c>
       <c r="D60" t="s">
         <v>10</v>
@@ -2931,24 +2889,24 @@
         <v>11</v>
       </c>
       <c r="F60" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="G60" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="H60" t="s">
-        <v>210</v>
+        <v>200</v>
       </c>
     </row>
     <row r="61" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
-        <v>154</v>
+        <v>184</v>
       </c>
       <c r="B61" t="s">
-        <v>187</v>
+        <v>165</v>
       </c>
       <c r="C61" t="s">
-        <v>31</v>
+        <v>164</v>
       </c>
       <c r="D61" t="s">
         <v>10</v>
@@ -2957,24 +2915,24 @@
         <v>11</v>
       </c>
       <c r="F61" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="G61" t="s">
         <v>13</v>
       </c>
       <c r="H61" t="s">
-        <v>188</v>
+        <v>185</v>
       </c>
     </row>
     <row r="62" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
-        <v>184</v>
+        <v>166</v>
       </c>
       <c r="B62" t="s">
-        <v>185</v>
+        <v>167</v>
       </c>
       <c r="C62" t="s">
-        <v>31</v>
+        <v>164</v>
       </c>
       <c r="D62" t="s">
         <v>10</v>
@@ -2983,24 +2941,24 @@
         <v>11</v>
       </c>
       <c r="F62" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="G62" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="H62" t="s">
-        <v>181</v>
+        <v>232</v>
       </c>
     </row>
     <row r="63" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
-        <v>79</v>
+        <v>205</v>
       </c>
       <c r="B63" t="s">
-        <v>79</v>
+        <v>168</v>
       </c>
       <c r="C63" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D63" t="s">
         <v>10</v>
@@ -3009,24 +2967,24 @@
         <v>11</v>
       </c>
       <c r="F63" t="s">
+        <v>27</v>
+      </c>
+      <c r="G63" t="s">
         <v>12</v>
       </c>
-      <c r="G63" t="s">
-        <v>13</v>
-      </c>
       <c r="H63" t="s">
-        <v>181</v>
+        <v>206</v>
       </c>
     </row>
     <row r="64" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
-        <v>85</v>
+        <v>141</v>
       </c>
       <c r="B64" t="s">
-        <v>242</v>
+        <v>168</v>
       </c>
       <c r="C64" t="s">
-        <v>243</v>
+        <v>30</v>
       </c>
       <c r="D64" t="s">
         <v>10</v>
@@ -3035,1426 +2993,1432 @@
         <v>11</v>
       </c>
       <c r="F64" t="s">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="G64" t="s">
-        <v>13</v>
+        <v>12</v>
+      </c>
+      <c r="H64" t="s">
+        <v>169</v>
       </c>
     </row>
     <row r="65" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
-        <v>36</v>
+        <v>64</v>
       </c>
       <c r="B65" t="s">
-        <v>242</v>
+        <v>65</v>
       </c>
       <c r="C65" t="s">
-        <v>243</v>
+        <v>36</v>
       </c>
       <c r="D65" t="s">
-        <v>10</v>
+        <v>37</v>
       </c>
       <c r="E65" t="s">
         <v>11</v>
       </c>
       <c r="F65" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="G65" t="s">
-        <v>13</v>
+        <v>58</v>
+      </c>
+      <c r="J65" s="3" t="s">
+        <v>50</v>
       </c>
     </row>
     <row r="66" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="B66" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="C66" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="D66" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="E66" t="s">
         <v>11</v>
       </c>
       <c r="F66" t="s">
-        <v>18</v>
+        <v>66</v>
       </c>
       <c r="G66" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="J66" s="3" t="s">
-        <v>54</v>
+        <v>67</v>
       </c>
     </row>
     <row r="67" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="B67" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="C67" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="D67" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="E67" t="s">
         <v>11</v>
       </c>
       <c r="F67" t="s">
-        <v>70</v>
+        <v>61</v>
       </c>
       <c r="G67" t="s">
-        <v>67</v>
+        <v>58</v>
       </c>
       <c r="J67" s="3" t="s">
-        <v>71</v>
+        <v>50</v>
       </c>
     </row>
     <row r="68" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
+        <v>64</v>
+      </c>
+      <c r="B68" t="s">
+        <v>64</v>
+      </c>
+      <c r="C68" t="s">
+        <v>36</v>
+      </c>
+      <c r="D68" t="s">
+        <v>37</v>
+      </c>
+      <c r="E68" t="s">
+        <v>11</v>
+      </c>
+      <c r="F68" t="s">
+        <v>14</v>
+      </c>
+      <c r="G68" t="s">
+        <v>63</v>
+      </c>
+      <c r="J68" s="3" t="s">
         <v>68</v>
-      </c>
-      <c r="B68" t="s">
-        <v>68</v>
-      </c>
-      <c r="C68" t="s">
-        <v>40</v>
-      </c>
-      <c r="D68" t="s">
-        <v>41</v>
-      </c>
-      <c r="E68" t="s">
-        <v>11</v>
-      </c>
-      <c r="F68" t="s">
-        <v>65</v>
-      </c>
-      <c r="G68" t="s">
-        <v>62</v>
-      </c>
-      <c r="J68" s="3" t="s">
-        <v>54</v>
       </c>
     </row>
     <row r="69" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
-        <v>68</v>
+        <v>44</v>
       </c>
       <c r="B69" t="s">
-        <v>68</v>
+        <v>45</v>
       </c>
       <c r="C69" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="D69" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="E69" t="s">
         <v>11</v>
       </c>
       <c r="F69" t="s">
-        <v>15</v>
+        <v>46</v>
       </c>
       <c r="G69" t="s">
-        <v>67</v>
+        <v>38</v>
       </c>
       <c r="J69" s="3" t="s">
-        <v>72</v>
+        <v>47</v>
       </c>
     </row>
     <row r="70" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
+        <v>44</v>
+      </c>
+      <c r="B70" t="s">
         <v>48</v>
       </c>
-      <c r="B70" t="s">
-        <v>49</v>
-      </c>
       <c r="C70" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="D70" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="E70" t="s">
         <v>11</v>
       </c>
       <c r="F70" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="G70" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="J70" s="3" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
     </row>
     <row r="71" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="B71" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="C71" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="D71" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="E71" t="s">
         <v>11</v>
       </c>
       <c r="F71" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="G71" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="J71" s="3" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
     </row>
     <row r="72" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="B72" t="s">
-        <v>53</v>
+        <v>44</v>
       </c>
       <c r="C72" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="D72" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="E72" t="s">
         <v>11</v>
       </c>
       <c r="F72" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="G72" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="J72" s="3" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
     </row>
     <row r="73" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="B73" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="C73" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="D73" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="E73" t="s">
         <v>11</v>
       </c>
       <c r="F73" t="s">
+        <v>46</v>
+      </c>
+      <c r="G73" t="s">
+        <v>38</v>
+      </c>
+      <c r="J73" s="3" t="s">
         <v>50</v>
-      </c>
-      <c r="G73" t="s">
-        <v>42</v>
-      </c>
-      <c r="J73" s="3" t="s">
-        <v>51</v>
       </c>
     </row>
     <row r="74" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="B74" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="C74" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="D74" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="E74" t="s">
         <v>11</v>
       </c>
       <c r="F74" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="G74" t="s">
-        <v>42</v>
+        <v>58</v>
       </c>
       <c r="J74" s="3" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="75" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
-        <v>56</v>
+        <v>34</v>
       </c>
       <c r="B75" t="s">
-        <v>56</v>
+        <v>34</v>
       </c>
       <c r="C75" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="D75" t="s">
-        <v>41</v>
+        <v>54</v>
       </c>
       <c r="E75" t="s">
         <v>11</v>
       </c>
       <c r="F75" t="s">
+        <v>55</v>
+      </c>
+      <c r="G75" t="s">
+        <v>38</v>
+      </c>
+      <c r="J75" s="3" t="s">
         <v>50</v>
-      </c>
-      <c r="G75" t="s">
-        <v>62</v>
-      </c>
-      <c r="J75" s="3" t="s">
-        <v>57</v>
       </c>
     </row>
     <row r="76" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A76" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B76" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="C76" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="D76" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="E76" t="s">
         <v>11</v>
       </c>
       <c r="F76" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="G76" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="J76" s="3" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
     </row>
     <row r="77" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A77" t="s">
-        <v>36</v>
+        <v>57</v>
       </c>
       <c r="B77" t="s">
-        <v>36</v>
+        <v>57</v>
       </c>
       <c r="C77" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="D77" t="s">
+        <v>37</v>
+      </c>
+      <c r="E77" t="s">
+        <v>11</v>
+      </c>
+      <c r="F77" t="s">
+        <v>56</v>
+      </c>
+      <c r="G77" t="s">
         <v>58</v>
       </c>
-      <c r="E77" t="s">
-        <v>11</v>
-      </c>
-      <c r="F77" t="s">
-        <v>60</v>
-      </c>
-      <c r="G77" t="s">
-        <v>42</v>
-      </c>
       <c r="J77" s="3" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
     </row>
     <row r="78" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A78" t="s">
-        <v>61</v>
+        <v>35</v>
       </c>
       <c r="B78" t="s">
-        <v>61</v>
+        <v>35</v>
       </c>
       <c r="C78" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="D78" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="E78" t="s">
         <v>11</v>
       </c>
       <c r="F78" t="s">
-        <v>60</v>
+        <v>17</v>
       </c>
       <c r="G78" t="s">
-        <v>62</v>
+        <v>38</v>
       </c>
       <c r="J78" s="3" t="s">
-        <v>63</v>
+        <v>39</v>
       </c>
     </row>
     <row r="79" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A79" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B79" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C79" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="D79" t="s">
+        <v>37</v>
+      </c>
+      <c r="E79" t="s">
+        <v>11</v>
+      </c>
+      <c r="F79" t="s">
+        <v>17</v>
+      </c>
+      <c r="G79" t="s">
+        <v>38</v>
+      </c>
+      <c r="J79" s="3" t="s">
         <v>41</v>
-      </c>
-      <c r="E79" t="s">
-        <v>11</v>
-      </c>
-      <c r="F79" t="s">
-        <v>18</v>
-      </c>
-      <c r="G79" t="s">
-        <v>42</v>
-      </c>
-      <c r="J79" s="3" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="80" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A80" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="B80" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="C80" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="D80" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="E80" t="s">
         <v>11</v>
       </c>
       <c r="F80" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="G80" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="J80" s="3" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
     </row>
     <row r="81" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A81" t="s">
-        <v>44</v>
+        <v>181</v>
       </c>
       <c r="B81" t="s">
-        <v>44</v>
+        <v>181</v>
       </c>
       <c r="C81" t="s">
-        <v>46</v>
+        <v>36</v>
       </c>
       <c r="D81" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="E81" t="s">
         <v>11</v>
       </c>
       <c r="F81" t="s">
-        <v>18</v>
+        <v>178</v>
       </c>
       <c r="G81" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="J81" s="3" t="s">
-        <v>47</v>
+        <v>182</v>
       </c>
     </row>
     <row r="82" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A82" t="s">
-        <v>204</v>
+        <v>69</v>
       </c>
       <c r="B82" t="s">
-        <v>204</v>
+        <v>69</v>
       </c>
       <c r="C82" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="D82" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="E82" t="s">
         <v>11</v>
       </c>
       <c r="F82" t="s">
-        <v>201</v>
+        <v>183</v>
       </c>
       <c r="G82" t="s">
-        <v>42</v>
+        <v>63</v>
       </c>
       <c r="J82" s="3" t="s">
-        <v>205</v>
+        <v>50</v>
       </c>
     </row>
     <row r="83" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A83" t="s">
-        <v>73</v>
+        <v>25</v>
       </c>
       <c r="B83" t="s">
-        <v>73</v>
+        <v>25</v>
       </c>
       <c r="C83" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="D83" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="E83" t="s">
         <v>11</v>
       </c>
       <c r="F83" t="s">
-        <v>206</v>
+        <v>61</v>
       </c>
       <c r="G83" t="s">
-        <v>67</v>
+        <v>58</v>
       </c>
       <c r="J83" s="3" t="s">
-        <v>54</v>
+        <v>70</v>
       </c>
     </row>
     <row r="84" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A84" t="s">
-        <v>26</v>
+        <v>233</v>
       </c>
       <c r="B84" t="s">
-        <v>26</v>
+        <v>233</v>
       </c>
       <c r="C84" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="D84" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="E84" t="s">
         <v>11</v>
       </c>
       <c r="F84" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="G84" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="J84" s="3" t="s">
-        <v>74</v>
+        <v>50</v>
       </c>
     </row>
     <row r="85" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A85" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B85" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C85" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="D85" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="E85" t="s">
         <v>11</v>
       </c>
       <c r="F85" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="G85" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="J85" s="3" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
     </row>
     <row r="86" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A86" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B86" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C86" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="D86" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="E86" t="s">
         <v>11</v>
       </c>
       <c r="F86" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="G86" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="J86" s="3" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
     </row>
     <row r="87" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A87" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="B87" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="C87" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="D87" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="E87" t="s">
         <v>11</v>
       </c>
       <c r="F87" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="G87" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="J87" s="3" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
     </row>
     <row r="88" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A88" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B88" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C88" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="D88" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="E88" t="s">
         <v>11</v>
       </c>
       <c r="F88" t="s">
-        <v>201</v>
+        <v>178</v>
       </c>
       <c r="G88" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="J88" s="3" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
     </row>
     <row r="89" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A89" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B89" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C89" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="D89" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="E89" t="s">
         <v>11</v>
       </c>
       <c r="F89" t="s">
-        <v>212</v>
+        <v>187</v>
       </c>
       <c r="G89" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="J89" s="3" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
     </row>
     <row r="90" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A90" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B90" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C90" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="D90" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="E90" t="s">
         <v>11</v>
       </c>
       <c r="F90" t="s">
+        <v>56</v>
+      </c>
+      <c r="G90" t="s">
+        <v>71</v>
+      </c>
+      <c r="J90" s="3" t="s">
         <v>60</v>
-      </c>
-      <c r="G90" t="s">
-        <v>75</v>
-      </c>
-      <c r="J90" s="3" t="s">
-        <v>64</v>
       </c>
     </row>
     <row r="91" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A91" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B91" t="s">
-        <v>244</v>
+        <v>210</v>
       </c>
       <c r="C91" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="D91" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="E91" t="s">
         <v>11</v>
       </c>
       <c r="F91" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="G91" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="J91" s="3" t="s">
-        <v>245</v>
+        <v>211</v>
       </c>
     </row>
     <row r="92" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A92" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B92" t="s">
-        <v>246</v>
+        <v>212</v>
       </c>
       <c r="C92" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="D92" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="E92" t="s">
         <v>11</v>
       </c>
       <c r="F92" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
       <c r="G92" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="H92" t="s">
-        <v>247</v>
+        <v>213</v>
       </c>
       <c r="J92" s="3" t="s">
-        <v>245</v>
+        <v>211</v>
       </c>
     </row>
     <row r="93" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A93" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B93" t="s">
-        <v>248</v>
+        <v>214</v>
       </c>
       <c r="C93" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="D93" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="E93" t="s">
         <v>11</v>
       </c>
       <c r="F93" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
       <c r="G93" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="H93" t="s">
-        <v>247</v>
+        <v>213</v>
       </c>
       <c r="J93" s="3" t="s">
-        <v>245</v>
+        <v>211</v>
       </c>
     </row>
     <row r="94" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A94" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B94" t="s">
-        <v>249</v>
+        <v>215</v>
       </c>
       <c r="C94" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="D94" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="E94" t="s">
         <v>11</v>
       </c>
       <c r="F94" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
       <c r="G94" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="J94" s="3" t="s">
-        <v>245</v>
+        <v>211</v>
       </c>
     </row>
     <row r="95" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A95" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B95" t="s">
-        <v>250</v>
+        <v>216</v>
       </c>
       <c r="C95" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="D95" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="E95" t="s">
         <v>11</v>
       </c>
       <c r="F95" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
       <c r="G95" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="H95" t="s">
-        <v>247</v>
+        <v>213</v>
       </c>
       <c r="J95" s="3" t="s">
-        <v>245</v>
+        <v>211</v>
       </c>
     </row>
     <row r="96" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A96" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B96" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C96" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="D96" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="E96" t="s">
         <v>11</v>
       </c>
       <c r="F96" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="G96" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="J96" s="3" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
     </row>
     <row r="97" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A97" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B97" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C97" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="D97" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="E97" t="s">
         <v>11</v>
       </c>
       <c r="F97" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="G97" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="J97" s="3" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
     </row>
     <row r="98" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A98" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B98" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C98" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="D98" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="E98" t="s">
         <v>11</v>
       </c>
       <c r="F98" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="G98" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="J98" s="3" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
     </row>
     <row r="99" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A99" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B99" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C99" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="D99" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="E99" t="s">
         <v>11</v>
       </c>
       <c r="F99" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="G99" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="J99" s="3" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
     </row>
     <row r="100" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A100" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="B100" t="s">
-        <v>103</v>
+        <v>98</v>
       </c>
       <c r="C100" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="D100" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="E100" t="s">
         <v>11</v>
       </c>
       <c r="F100" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
       <c r="G100" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="J100" s="3" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
     </row>
     <row r="101" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A101" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="B101" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="C101" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="D101" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="E101" t="s">
         <v>11</v>
       </c>
       <c r="F101" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="G101" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="J101" s="3" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
     </row>
     <row r="102" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A102" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="B102" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="C102" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="D102" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="E102" t="s">
         <v>11</v>
       </c>
       <c r="F102" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="G102" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="J102" s="3" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
     </row>
     <row r="103" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A103" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="B103" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="C103" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="D103" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="E103" t="s">
         <v>11</v>
       </c>
       <c r="F103" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="G103" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="J103" s="3" t="s">
-        <v>66</v>
+        <v>62</v>
       </c>
     </row>
     <row r="104" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A104" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B104" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="C104" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="D104" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="E104" t="s">
         <v>11</v>
       </c>
       <c r="F104" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="G104" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="J104" s="3" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
     </row>
     <row r="105" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A105" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B105" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C105" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="D105" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="E105" t="s">
         <v>11</v>
       </c>
       <c r="F105" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="G105" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="I105" s="3">
         <v>14</v>
       </c>
       <c r="J105" s="3" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
     </row>
     <row r="106" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A106" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B106" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C106" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="D106" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="E106" t="s">
         <v>11</v>
       </c>
       <c r="F106" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="G106" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="I106" s="3">
         <v>14</v>
       </c>
       <c r="J106" s="3" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
     </row>
     <row r="107" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A107" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="B107" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="C107" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="D107" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="E107" t="s">
         <v>11</v>
       </c>
       <c r="F107" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="G107" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="J107" s="3" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
     </row>
     <row r="108" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A108" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="B108" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="C108" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="D108" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="E108" t="s">
         <v>11</v>
       </c>
       <c r="F108" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="G108" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="J108" s="3" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
     </row>
     <row r="109" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A109" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="B109" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="C109" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="D109" t="s">
+        <v>54</v>
+      </c>
+      <c r="E109" t="s">
+        <v>11</v>
+      </c>
+      <c r="F109" t="s">
+        <v>61</v>
+      </c>
+      <c r="G109" t="s">
         <v>58</v>
       </c>
-      <c r="E109" t="s">
-        <v>11</v>
-      </c>
-      <c r="F109" t="s">
-        <v>65</v>
-      </c>
-      <c r="G109" t="s">
-        <v>62</v>
-      </c>
       <c r="J109" s="3" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
     </row>
     <row r="110" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A110" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="B110" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="C110" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="D110" t="s">
+        <v>54</v>
+      </c>
+      <c r="E110" t="s">
+        <v>11</v>
+      </c>
+      <c r="F110" t="s">
+        <v>61</v>
+      </c>
+      <c r="G110" t="s">
         <v>58</v>
       </c>
-      <c r="E110" t="s">
-        <v>11</v>
-      </c>
-      <c r="F110" t="s">
-        <v>65</v>
-      </c>
-      <c r="G110" t="s">
-        <v>62</v>
-      </c>
       <c r="J110" s="3" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
     </row>
     <row r="111" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A111" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="B111" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="C111" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="D111" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="E111" t="s">
         <v>11</v>
       </c>
       <c r="F111" t="s">
-        <v>102</v>
+        <v>97</v>
       </c>
       <c r="G111" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="J111" s="3" t="s">
-        <v>99</v>
+        <v>94</v>
       </c>
     </row>
     <row r="112" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A112" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="B112" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="C112" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="D112" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="E112" t="s">
         <v>11</v>
       </c>
       <c r="F112" t="s">
-        <v>102</v>
+        <v>97</v>
       </c>
       <c r="G112" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="J112" s="3" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
     </row>
     <row r="113" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A113" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="B113" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="C113" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="D113" t="s">
+        <v>54</v>
+      </c>
+      <c r="E113" t="s">
+        <v>11</v>
+      </c>
+      <c r="F113" t="s">
+        <v>14</v>
+      </c>
+      <c r="G113" t="s">
         <v>58</v>
       </c>
-      <c r="E113" t="s">
-        <v>11</v>
-      </c>
-      <c r="F113" t="s">
-        <v>15</v>
-      </c>
-      <c r="G113" t="s">
-        <v>62</v>
-      </c>
       <c r="J113" s="3" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
     </row>
     <row r="114" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A114" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="B114" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="C114" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="D114" t="s">
+        <v>54</v>
+      </c>
+      <c r="E114" t="s">
+        <v>11</v>
+      </c>
+      <c r="F114" t="s">
+        <v>56</v>
+      </c>
+      <c r="G114" t="s">
         <v>58</v>
       </c>
-      <c r="E114" t="s">
-        <v>11</v>
-      </c>
-      <c r="F114" t="s">
-        <v>60</v>
-      </c>
-      <c r="G114" t="s">
-        <v>62</v>
-      </c>
       <c r="J114" s="3" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
     </row>
     <row r="115" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A115" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="B115" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="C115" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="D115" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="E115" t="s">
         <v>11</v>
       </c>
       <c r="F115" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="G115" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="J115" s="3" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
     </row>
     <row r="116" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A116" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="B116" t="s">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="C116" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="D116" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="E116" t="s">
         <v>11</v>
       </c>
       <c r="F116" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="G116" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="J116" s="3" t="s">
-        <v>54</v>
+        <v>50</v>
       </c>
     </row>
     <row r="117" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A117" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="B117" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="C117" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="D117" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="E117" t="s">
         <v>11</v>
       </c>
       <c r="F117" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="G117" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="J117" s="3" t="s">
-        <v>97</v>
+        <v>93</v>
       </c>
     </row>
     <row r="118" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A118" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="B118" t="s">
-        <v>95</v>
+        <v>91</v>
       </c>
       <c r="C118" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="D118" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="E118" t="s">
         <v>11</v>
       </c>
       <c r="F118" t="s">
+        <v>46</v>
+      </c>
+      <c r="G118" t="s">
+        <v>58</v>
+      </c>
+      <c r="J118" s="3" t="s">
         <v>50</v>
-      </c>
-      <c r="G118" t="s">
-        <v>62</v>
-      </c>
-      <c r="J118" s="3" t="s">
-        <v>54</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualização diaria de Aniversariantes e cargas
</commit_message>
<xml_diff>
--- a/scripts/cargas.xlsx
+++ b/scripts/cargas.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projetos\tr.alienigenaV5-main\scripts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B9BC6202-462C-40D9-9DDA-5E6030BF438D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{A6D289F3-ED23-4377-A366-8066841AFA23}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" tabRatio="551" xr2:uid="{9E8F4E85-D2FF-4383-A72B-5CAFDCCC5644}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Planilha1!$A$1:$J$118</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Planilha1!$A$1:$J$122</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="997" uniqueCount="234">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1033" uniqueCount="227">
   <si>
     <t>Origem</t>
   </si>
@@ -134,18 +134,12 @@
     <t>Corumbá - MS</t>
   </si>
   <si>
-    <t>MILHO</t>
-  </si>
-  <si>
     <t>São Gonçalo do Amarante - CE</t>
   </si>
   <si>
     <t>Sobral - CE</t>
   </si>
   <si>
-    <t>Carreta LS, Rodotrem</t>
-  </si>
-  <si>
     <t>Laranjeiras - SE</t>
   </si>
   <si>
@@ -161,21 +155,12 @@
     <t>Grade Baixa</t>
   </si>
   <si>
-    <t>PARA CARREGAMENTO, NECESSÁRIO CHAPA E TER PALLETS, CINTA, LONA E EPI. Possíveis destinos disponíveis:Região dos Lagos (Araruama/RJ com Saquarema/RJ na mesma rota e Cabo Frio/RJ com Arraial do Cabo/RJ na mesma rota)</t>
-  </si>
-  <si>
     <t>Rio de Janeiro - RJ</t>
   </si>
   <si>
-    <t>PARA CARREGAMENTO, NECESSÁRIO CHAPA E TER PALLETS, CINTA, LONA E EPI. Possíveis destinos disponíveis CD Santa Cruz: Rio de Janeiro-RJ, Itaguaí -RJ, Seropédica-RJ, Itatiaia-RJ.</t>
-  </si>
-  <si>
     <t>CIMENTO ENSACADO</t>
   </si>
   <si>
-    <t>PARA CARREGAMENTO, NECESSÁRIO CHAPA E TER PALLETS, CINTA, LONA E EPI. Possíveis destinos disponíveis CD RIO: Rio de Janeiro-RJ, Nova Iguaçu-RJ, Duque de Caxias-RJ, Mesquita-RJ )</t>
-  </si>
-  <si>
     <t>Campinas - SP</t>
   </si>
   <si>
@@ -185,9 +170,6 @@
     <t>Toco, Truck, Bitruck</t>
   </si>
   <si>
-    <t>PARA CARREGAMENTO, NECESSÁRIO CHAPA E TER PALLETS, CINTA, LONA E EPI- VEICULOS TOCO APENAS 10 TON</t>
-  </si>
-  <si>
     <t>Serra Negra - SP</t>
   </si>
   <si>
@@ -203,9 +185,6 @@
     <t>Guarulhos - SP</t>
   </si>
   <si>
-    <t>PARA CARREGAMENTO, NECESSÁRIO CHAPA E TER PALLETS, CINTA, LONA E EPI - POSSIVEIS DESTINOS DISPONIVEIS: Guarulhos/SP, São Paulo/SP (Zona Leste), Região do Alto Tietê/SP</t>
-  </si>
-  <si>
     <t>Saco</t>
   </si>
   <si>
@@ -245,18 +224,9 @@
     <t>Truck, Carreta LS</t>
   </si>
   <si>
-    <t>PARA CARREGAMENTO, NECESSÁRIO CHAPA E TER PALLETS, CINTA, LONA E EPI - DESTINOS DISPONIVEIS: CASTELO DO PIAUI/PI, SÃO MIGUEL DO TAPUI/PI, PARNAIBA/PI, BARRAS/PI, CAJUEIRO DA PRAIA/PI, SÃO JOÃO DA FRONTEIRA/PI, ILHA GRANDE/PI, COCAL/PI, LAGOA ALEGRE/PI, MIGUEL ALVES/PI, ALTOS/PI, SÃO JOÃO DA SERRA/PI, CAMPO MAIOR/PI, BENEDITINOS/PI, LUZILANDIA/PI, MADEIRO/PI, MATIAS OLIMPIO/PI, TUTOIA/MA.</t>
-  </si>
-  <si>
-    <t>DESTINOS DISPONIVEIS: No Extremo Sul do Estado do PI - PARA CARREGAMENTO, NECESSÁRIO CHAPA E TER PALLETS, CINTA, LONA E EPI</t>
-  </si>
-  <si>
     <t>Petrolina - PE</t>
   </si>
   <si>
-    <t>PARA CARREGAMENTO, NECESSÁRIO CHAPA E TER PALLETS, CINTA, LONA E EPI / DESTINOS: regiões Metropolitana , PB e RN</t>
-  </si>
-  <si>
     <t>Graneleiro, Grade Baixa</t>
   </si>
   <si>
@@ -266,9 +236,6 @@
     <t>Nobres - MT</t>
   </si>
   <si>
-    <t>DESTINO INTRA MUNICIPAL / PARA CARREGAMENTO, NECESSÁRIO CHAPA E TER PALLETS, CINTA, LONA E EPI</t>
-  </si>
-  <si>
     <t>Brasília - DF</t>
   </si>
   <si>
@@ -284,9 +251,6 @@
     <t>Luís Eduardo Magalhães - BA</t>
   </si>
   <si>
-    <t>PARA CARREGAMENTO, NECESSÁRIO CHAPA E TER PALLETS, CINTA, LONA E EPI - Possiveis Destinos Disponíveis: Cocos/BA, Serra Dourada/BA, São Félix do Coribe/BA, Tabocas do Brejo Velho/BA, Correntina/BA, Mansidão/BA, Formosa do Rio Preto/BA, Santa Rita de Cassia/BA, Barreiras/BA e Morpará/BA</t>
-  </si>
-  <si>
     <t>Camaçari - BA</t>
   </si>
   <si>
@@ -305,36 +269,18 @@
     <t>Sider, Grade Baixa, Prancha</t>
   </si>
   <si>
-    <t>PARA CARREGAMENTO, NECESSÁRIO CHAPA E TER PALLETS, CINTA, LONA E EPI - DESTINOS DISPONIVEIS: Simões Filho/BA, Lauro de Freitas/BA, Salvador/BA. - Não trabalhamos com motoristas passantes, prioridade em atuação local com disponibilidade para operar nas regiões mencionadas acima</t>
-  </si>
-  <si>
     <t>Feira de Santana - BA</t>
   </si>
   <si>
-    <t>PARA CARREGAMENTO, NECESSÁRIO CHAPA E TER PALLETS, CINTA, LONA E EPI / DESTINOS DISPONIVEIS: TANHACU, CHAPADA, BRUMADO, JAGUAQUARA - JACOBINA</t>
-  </si>
-  <si>
-    <t>PARA CARREGAMENTO, NECESSÁRIO CHAPA E TER PALLETS, CINTA, LONA E EPI. Veiculos Aceitos: TRUCK E CARRETA TOCO (28 TON)</t>
-  </si>
-  <si>
     <t>Itabuna - BA</t>
   </si>
   <si>
     <t>Vitória da Conquista - BA</t>
   </si>
   <si>
-    <t>PARA CARREGAMENTO, NECESSÁRIO CHAPA E TER PALLETS, CINTA, LONA E EPI - POSSIVEIS DESTINOS DISPONIVEIS: Região de Gargalo, Vitória da Conquista e Ipiau</t>
-  </si>
-  <si>
-    <t>PARA CARREGAMENTO, NECESSÁRIO CHAPA E TER PALLETS, CINTA, LONA E EPI / Tem cargas todos os dias e não agregamos passantes.</t>
-  </si>
-  <si>
     <t>50,00</t>
   </si>
   <si>
-    <t>APENAS MOTORISTAS CATIVOS - PARA CARREGAMENTO, NECESSÁRIO CHAPA E TER PALLETS, CINTA, LONA E EPI - DESTINOS DISPONIVEIS: Região do Litoral Norte de Camaçari, Catu/Ba Pojuca/Ba, Maragojipe/BA, Candeias/BA, São Francisco/BA, São Félix/BA, Cachoeira/BA - Não trabalhamos com motoristas passantes, prioridade em atuação local com disponibilidade para operar nas regiões mencionadas acima</t>
-  </si>
-  <si>
     <t>Toco</t>
   </si>
   <si>
@@ -467,15 +413,6 @@
     <t>168,00</t>
   </si>
   <si>
-    <t>Buriti Alegre - GO</t>
-  </si>
-  <si>
-    <t>CALCÁRIO</t>
-  </si>
-  <si>
-    <t>170,00</t>
-  </si>
-  <si>
     <t>Barro Alto - GO</t>
   </si>
   <si>
@@ -530,33 +467,6 @@
     <t>calcario/ clínquer</t>
   </si>
   <si>
-    <t>Mineiros - GO</t>
-  </si>
-  <si>
-    <t>Chapadão do Céu - GO</t>
-  </si>
-  <si>
-    <t>milho</t>
-  </si>
-  <si>
-    <t>Hidrolândia - GO</t>
-  </si>
-  <si>
-    <t>Jataí - GO</t>
-  </si>
-  <si>
-    <t>Rio Verde - GO</t>
-  </si>
-  <si>
-    <t>Quirinópolis - GO</t>
-  </si>
-  <si>
-    <t>85,00</t>
-  </si>
-  <si>
-    <t>Montividiu - GO</t>
-  </si>
-  <si>
     <t>80,00</t>
   </si>
   <si>
@@ -590,18 +500,9 @@
     <t>Primavera - PA</t>
   </si>
   <si>
-    <t>PARA MOTORISTAS CATIVOS NA REGIÃO - PARA CARREGAMENTO, NECESSÁRIO CHAPA E TER PALLETS, CINTA, LONA E EPI</t>
-  </si>
-  <si>
     <t>Toco, Truck</t>
   </si>
   <si>
-    <t>Marzagão - GO</t>
-  </si>
-  <si>
-    <t>70,00</t>
-  </si>
-  <si>
     <t>Rio Branco do Sul - PR</t>
   </si>
   <si>
@@ -620,33 +521,9 @@
     <t>Vidal Ramos - SC</t>
   </si>
   <si>
-    <t>150,00</t>
-  </si>
-  <si>
     <t>650,00</t>
   </si>
   <si>
-    <t>São Pedro - SP</t>
-  </si>
-  <si>
-    <t>Cajamar - SP</t>
-  </si>
-  <si>
-    <t>Areia</t>
-  </si>
-  <si>
-    <t>115,00</t>
-  </si>
-  <si>
-    <t>Castro - PR</t>
-  </si>
-  <si>
-    <t>Chapadão do Sul - MS</t>
-  </si>
-  <si>
-    <t>57,00</t>
-  </si>
-  <si>
     <t>Santa Filomena - PI</t>
   </si>
   <si>
@@ -659,21 +536,6 @@
     <t>só aceita rodocaçambas com lona fácil. Caso não tenham, o veículo não passa na vistoria dos guardas</t>
   </si>
   <si>
-    <t>Goiatuba - GO</t>
-  </si>
-  <si>
-    <t>73,00</t>
-  </si>
-  <si>
-    <t>Itaberaí - GO</t>
-  </si>
-  <si>
-    <t>87,00</t>
-  </si>
-  <si>
-    <t>35,00</t>
-  </si>
-  <si>
     <t>Alfenas - MG</t>
   </si>
   <si>
@@ -707,18 +569,12 @@
     <t>190,00</t>
   </si>
   <si>
-    <t>Carreta LS, Carreta 4º eixo</t>
-  </si>
-  <si>
     <t>Carreta LS, Bitrem 7 eixos, Carreta 4º eixo</t>
   </si>
   <si>
     <t>Itápolis - SP</t>
   </si>
   <si>
-    <t>Carreta, Carreta LS</t>
-  </si>
-  <si>
     <t>Vanderléia, Carreta 4º eixo</t>
   </si>
   <si>
@@ -737,13 +593,136 @@
     <t>70,71</t>
   </si>
   <si>
-    <t>Bariri - SP</t>
-  </si>
-  <si>
-    <t>40,00</t>
-  </si>
-  <si>
     <t>Caruaru - PE</t>
+  </si>
+  <si>
+    <t>Joinville - SC</t>
+  </si>
+  <si>
+    <t>Tubos e Conexões</t>
+  </si>
+  <si>
+    <t>Tubo</t>
+  </si>
+  <si>
+    <t>Truck, Carreta, Carreta LS, Vanderléia, Carreta 4º eixo</t>
+  </si>
+  <si>
+    <t>Sider, Baú, Grade Baixa</t>
+  </si>
+  <si>
+    <t>Vanderléia</t>
+  </si>
+  <si>
+    <t>155,00</t>
+  </si>
+  <si>
+    <t>Poço Fundo - MG</t>
+  </si>
+  <si>
+    <t>Big Bag</t>
+  </si>
+  <si>
+    <t>Graneleiro, Sider, Grade Baixa</t>
+  </si>
+  <si>
+    <t>195,00</t>
+  </si>
+  <si>
+    <t>Carreta 4º eixo</t>
+  </si>
+  <si>
+    <t>Carreta</t>
+  </si>
+  <si>
+    <t>Primavera do Leste - MT</t>
+  </si>
+  <si>
+    <t>São João da Barra - RJ</t>
+  </si>
+  <si>
+    <t>Milho</t>
+  </si>
+  <si>
+    <t>510,00</t>
+  </si>
+  <si>
+    <t>Santos - SP</t>
+  </si>
+  <si>
+    <t>180,00</t>
+  </si>
+  <si>
+    <t>Nova Ponte - MG</t>
+  </si>
+  <si>
+    <t>Ponte Nova - MG</t>
+  </si>
+  <si>
+    <t>Brasilândia de Minas - MG</t>
+  </si>
+  <si>
+    <t>Penápolis - SP</t>
+  </si>
+  <si>
+    <t>Ureia granel</t>
+  </si>
+  <si>
+    <t>PARA CARREGAMENTO, NECESSÁRIO CHAPA (AJUDANTE) E TER PALLETS, CINTA, LONA E EPI - DESTINOS DISPONIVEIS: CASTELO DO PIAUI/PI, SÃO MIGUEL DO TAPUI/PI, PARNAIBA/PI, BARRAS/PI, CAJUEIRO DA PRAIA/PI, SÃO JOÃO DA FRONTEIRA/PI, ILHA GRANDE/PI, COCAL/PI, LAGOA ALEGRE/PI, MIGUEL ALVES/PI, ALTOS/PI, SÃO JOÃO DA SERRA/PI, CAMPO MAIOR/PI, BENEDITINOS/PI, LUZILANDIA/PI, MADEIRO/PI, MATIAS OLIMPIO/PI, TUTOIA/MA.</t>
+  </si>
+  <si>
+    <t>PARA CARREGAMENTO, NECESSÁRIO CHAPA (AJUDANTE) E TER PALLETS, CINTA, LONA E EPI</t>
+  </si>
+  <si>
+    <t>DESTINOS DISPONIVEIS: No Extremo Sul do Estado do PI - PARA CARREGAMENTO, NECESSÁRIO CHAPA (AJUDANTE) E TER PALLETS, CINTA, LONA E EPI</t>
+  </si>
+  <si>
+    <t>PARA CARREGAMENTO, NECESSÁRIO CHAPA (AJUDANTE) E TER PALLETS, CINTA, LONA E EPI- VEICULOS TOCO APENAS 10 TON</t>
+  </si>
+  <si>
+    <t>PARA CARREGAMENTO, NECESSÁRIO CHAPA (AJUDANTE) E TER PALLETS, CINTA, LONA E EPI - POSSIVEIS DESTINOS DISPONIVEIS: Guarulhos/SP, São Paulo/SP (Zona Leste), Região do Alto Tietê/SP</t>
+  </si>
+  <si>
+    <t>PARA CARREGAMENTO, NECESSÁRIO CHAPA (AJUDANTE) E TER PALLETS, CINTA, LONA E EPI. Possíveis destinos disponíveis:Região dos Lagos (Araruama/RJ com Saquarema/RJ na mesma rota e Cabo Frio/RJ com Arraial do Cabo/RJ na mesma rota)</t>
+  </si>
+  <si>
+    <t>PARA CARREGAMENTO, NECESSÁRIO CHAPA (AJUDANTE) E TER PALLETS, CINTA, LONA E EPI. Possíveis destinos disponíveis CD Santa Cruz: Rio de Janeiro-RJ, Itaguaí -RJ, Seropédica-RJ, Itatiaia-RJ.</t>
+  </si>
+  <si>
+    <t>PARA CARREGAMENTO, NECESSÁRIO CHAPA (AJUDANTE) E TER PALLETS, CINTA, LONA E EPI. Possíveis destinos disponíveis CD RIO: Rio de Janeiro-RJ, Nova Iguaçu-RJ, Duque de Caxias-RJ, Mesquita-RJ )</t>
+  </si>
+  <si>
+    <t>PARA MOTORISTAS CATIVOS NA REGIÃO - PARA CARREGAMENTO, NECESSÁRIO CHAPA (AJUDANTE) E TER PALLETS, CINTA, LONA E EPI</t>
+  </si>
+  <si>
+    <t>PARA CARREGAMENTO, NECESSÁRIO CHAPA (AJUDANTE) E TER PALLETS, CINTA, LONA E EPI / DESTINOS: regiões Metropolitana , PB e RN</t>
+  </si>
+  <si>
+    <t>DESTINO INTRA MUNICIPAL / PARA CARREGAMENTO, NECESSÁRIO CHAPA (AJUDANTE) E TER PALLETS, CINTA, LONA E EPI</t>
+  </si>
+  <si>
+    <t>PARA CARREGAMENTO, NECESSÁRIO CHAPA (AJUDANTE) E TER PALLETS, CINTA, LONA E EPI - Possiveis Destinos Disponíveis: Cocos/BA, Serra Dourada/BA, São Félix do Coribe/BA, Tabocas do Brejo Velho/BA, Correntina/BA, Mansidão/BA, Formosa do Rio Preto/BA, Santa Rita de Cassia/BA, Barreiras/BA e Morpará/BA</t>
+  </si>
+  <si>
+    <t>APENAS MOTORISTAS CATIVOS - PARA CARREGAMENTO, NECESSÁRIO CHAPA (AJUDANTE) E TER PALLETS, CINTA, LONA E EPI - DESTINOS DISPONIVEIS: Região do Litoral Norte de Camaçari, Catu/Ba Pojuca/Ba, Maragojipe/BA, Candeias/BA, São Francisco/BA, São Félix/BA, Cachoeira/BA - Não trabalhamos com motoristas passantes, prioridade em atuação local com disponibilidade para operar nas regiões mencionadas acima</t>
+  </si>
+  <si>
+    <t>PARA CARREGAMENTO, NECESSÁRIO CHAPA (AJUDANTE) E TER PALLETS, CINTA, LONA E EPI / Tem cargas todos os dias e não agregamos passantes.</t>
+  </si>
+  <si>
+    <t>PARA CARREGAMENTO, NECESSÁRIO CHAPA (AJUDANTE) E TER PALLETS, CINTA, LONA E EPI - DESTINOS DISPONIVEIS: Simões Filho/BA, Lauro de Freitas/BA, Salvador/BA. - Não trabalhamos com motoristas passantes, prioridade em atuação local com disponibilidade para operar nas regiões mencionadas acima</t>
+  </si>
+  <si>
+    <t>PARA CARREGAMENTO, NECESSÁRIO CHAPA (AJUDANTE) E TER PALLETS, CINTA, LONA E EPI / DESTINOS DISPONIVEIS: TANHACU, CHAPADA, BRUMADO, JAGUAQUARA - JACOBINA</t>
+  </si>
+  <si>
+    <t>PARA CARREGAMENTO, NECESSÁRIO CHAPA (AJUDANTE) E TER PALLETS, CINTA, LONA E EPI. Veiculos Aceitos: TRUCK E CARRETA TOCO (28 TON)</t>
+  </si>
+  <si>
+    <t>PARA CARREGAMENTO, NECESSÁRIO CHAPA (AJUDANTE) E TER PALLETS, CINTA, LONA E EPI - POSSIVEIS DESTINOS DISPONIVEIS: Região de Gargalo, Vitória da Conquista e Ipiau</t>
+  </si>
+  <si>
+    <t>Ureia Granel</t>
   </si>
 </sst>
 </file>
@@ -1143,15 +1122,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EAF16D4A-DA29-4FF0-AC3B-589258931E62}">
-  <dimension ref="A1:J118"/>
+  <dimension ref="A1:J122"/>
   <sheetFormatPr defaultColWidth="12.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="25.5546875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="25.6640625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="18.44140625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="9.6640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="19.77734375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="35.109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="16.88671875" customWidth="1"/>
+    <col min="6" max="6" width="44.88671875" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="27.77734375" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="8.88671875" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="11.44140625" style="3" bestFit="1" customWidth="1"/>
@@ -1192,39 +1171,39 @@
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>144</v>
+        <v>184</v>
       </c>
       <c r="B2" t="s">
-        <v>217</v>
+        <v>184</v>
       </c>
       <c r="C2" t="s">
-        <v>145</v>
+        <v>185</v>
       </c>
       <c r="D2" t="s">
-        <v>10</v>
+        <v>186</v>
       </c>
       <c r="E2" t="s">
         <v>11</v>
       </c>
       <c r="F2" t="s">
-        <v>19</v>
+        <v>187</v>
       </c>
       <c r="G2" t="s">
-        <v>13</v>
-      </c>
-      <c r="H2" t="s">
-        <v>218</v>
+        <v>188</v>
+      </c>
+      <c r="I2" s="3">
+        <v>14</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>124</v>
+        <v>118</v>
       </c>
       <c r="B3" t="s">
-        <v>25</v>
+        <v>173</v>
       </c>
       <c r="C3" t="s">
-        <v>161</v>
+        <v>85</v>
       </c>
       <c r="D3" t="s">
         <v>10</v>
@@ -1233,27 +1212,27 @@
         <v>11</v>
       </c>
       <c r="F3" t="s">
-        <v>27</v>
+        <v>19</v>
       </c>
       <c r="G3" t="s">
         <v>13</v>
       </c>
       <c r="H3" t="s">
-        <v>95</v>
+        <v>174</v>
       </c>
       <c r="J3" s="3" t="s">
-        <v>125</v>
+        <v>20</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>136</v>
+        <v>118</v>
       </c>
       <c r="B4" t="s">
-        <v>219</v>
+        <v>160</v>
       </c>
       <c r="C4" t="s">
-        <v>103</v>
+        <v>85</v>
       </c>
       <c r="D4" t="s">
         <v>10</v>
@@ -1268,7 +1247,7 @@
         <v>13</v>
       </c>
       <c r="H4" t="s">
-        <v>220</v>
+        <v>161</v>
       </c>
       <c r="J4" s="3" t="s">
         <v>20</v>
@@ -1276,13 +1255,13 @@
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>136</v>
+        <v>147</v>
       </c>
       <c r="B5" t="s">
-        <v>201</v>
+        <v>158</v>
       </c>
       <c r="C5" t="s">
-        <v>103</v>
+        <v>119</v>
       </c>
       <c r="D5" t="s">
         <v>10</v>
@@ -1291,42 +1270,42 @@
         <v>11</v>
       </c>
       <c r="F5" t="s">
-        <v>19</v>
+        <v>189</v>
       </c>
       <c r="G5" t="s">
         <v>13</v>
       </c>
       <c r="H5" t="s">
-        <v>202</v>
+        <v>190</v>
       </c>
       <c r="J5" s="3" t="s">
-        <v>20</v>
+        <v>92</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
+        <v>83</v>
+      </c>
+      <c r="B6" t="s">
+        <v>191</v>
+      </c>
+      <c r="C6" t="s">
+        <v>85</v>
+      </c>
+      <c r="D6" t="s">
+        <v>192</v>
+      </c>
+      <c r="E6" t="s">
+        <v>11</v>
+      </c>
+      <c r="F6" t="s">
+        <v>21</v>
+      </c>
+      <c r="G6" t="s">
+        <v>193</v>
+      </c>
+      <c r="H6" t="s">
         <v>194</v>
-      </c>
-      <c r="B6" t="s">
-        <v>195</v>
-      </c>
-      <c r="C6" t="s">
-        <v>196</v>
-      </c>
-      <c r="D6" t="s">
-        <v>10</v>
-      </c>
-      <c r="E6" t="s">
-        <v>11</v>
-      </c>
-      <c r="F6" t="s">
-        <v>16</v>
-      </c>
-      <c r="G6" t="s">
-        <v>13</v>
-      </c>
-      <c r="H6" t="s">
-        <v>197</v>
       </c>
       <c r="J6" s="3" t="s">
         <v>20</v>
@@ -1334,13 +1313,13 @@
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>177</v>
+        <v>147</v>
       </c>
       <c r="B7" t="s">
-        <v>191</v>
+        <v>158</v>
       </c>
       <c r="C7" t="s">
-        <v>137</v>
+        <v>119</v>
       </c>
       <c r="D7" t="s">
         <v>10</v>
@@ -1349,27 +1328,27 @@
         <v>11</v>
       </c>
       <c r="F7" t="s">
-        <v>221</v>
+        <v>175</v>
       </c>
       <c r="G7" t="s">
         <v>13</v>
       </c>
       <c r="H7" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="J7" s="3" t="s">
-        <v>110</v>
+        <v>92</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>177</v>
+        <v>147</v>
       </c>
       <c r="B8" t="s">
-        <v>191</v>
+        <v>153</v>
       </c>
       <c r="C8" t="s">
-        <v>137</v>
+        <v>119</v>
       </c>
       <c r="D8" t="s">
         <v>10</v>
@@ -1378,27 +1357,27 @@
         <v>11</v>
       </c>
       <c r="F8" t="s">
-        <v>187</v>
+        <v>154</v>
       </c>
       <c r="G8" t="s">
         <v>13</v>
       </c>
       <c r="H8" t="s">
-        <v>192</v>
+        <v>155</v>
       </c>
       <c r="J8" s="3" t="s">
-        <v>110</v>
+        <v>92</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>177</v>
+        <v>147</v>
       </c>
       <c r="B9" t="s">
-        <v>186</v>
+        <v>153</v>
       </c>
       <c r="C9" t="s">
-        <v>137</v>
+        <v>119</v>
       </c>
       <c r="D9" t="s">
         <v>10</v>
@@ -1407,27 +1386,27 @@
         <v>11</v>
       </c>
       <c r="F9" t="s">
-        <v>187</v>
+        <v>81</v>
       </c>
       <c r="G9" t="s">
         <v>13</v>
       </c>
       <c r="H9" t="s">
-        <v>188</v>
+        <v>155</v>
       </c>
       <c r="J9" s="3" t="s">
-        <v>110</v>
+        <v>92</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>177</v>
+        <v>147</v>
       </c>
       <c r="B10" t="s">
-        <v>186</v>
+        <v>156</v>
       </c>
       <c r="C10" t="s">
-        <v>137</v>
+        <v>119</v>
       </c>
       <c r="D10" t="s">
         <v>10</v>
@@ -1436,27 +1415,27 @@
         <v>11</v>
       </c>
       <c r="F10" t="s">
-        <v>222</v>
+        <v>175</v>
       </c>
       <c r="G10" t="s">
         <v>13</v>
       </c>
       <c r="H10" t="s">
-        <v>188</v>
+        <v>155</v>
       </c>
       <c r="J10" s="3" t="s">
-        <v>110</v>
+        <v>92</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>177</v>
+        <v>83</v>
       </c>
       <c r="B11" t="s">
-        <v>189</v>
+        <v>176</v>
       </c>
       <c r="C11" t="s">
-        <v>137</v>
+        <v>85</v>
       </c>
       <c r="D11" t="s">
         <v>10</v>
@@ -1465,27 +1444,27 @@
         <v>11</v>
       </c>
       <c r="F11" t="s">
-        <v>55</v>
+        <v>14</v>
       </c>
       <c r="G11" t="s">
         <v>13</v>
       </c>
       <c r="H11" t="s">
-        <v>188</v>
+        <v>157</v>
       </c>
       <c r="J11" s="3" t="s">
-        <v>110</v>
+        <v>20</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>101</v>
+        <v>83</v>
       </c>
       <c r="B12" t="s">
-        <v>223</v>
+        <v>149</v>
       </c>
       <c r="C12" t="s">
-        <v>103</v>
+        <v>85</v>
       </c>
       <c r="D12" t="s">
         <v>10</v>
@@ -1494,13 +1473,13 @@
         <v>11</v>
       </c>
       <c r="F12" t="s">
-        <v>27</v>
+        <v>14</v>
       </c>
       <c r="G12" t="s">
         <v>13</v>
       </c>
       <c r="H12" t="s">
-        <v>190</v>
+        <v>141</v>
       </c>
       <c r="J12" s="3" t="s">
         <v>20</v>
@@ -1508,13 +1487,13 @@
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>101</v>
+        <v>83</v>
       </c>
       <c r="B13" t="s">
-        <v>179</v>
+        <v>84</v>
       </c>
       <c r="C13" t="s">
-        <v>103</v>
+        <v>85</v>
       </c>
       <c r="D13" t="s">
         <v>10</v>
@@ -1523,13 +1502,13 @@
         <v>11</v>
       </c>
       <c r="F13" t="s">
-        <v>27</v>
+        <v>14</v>
       </c>
       <c r="G13" t="s">
         <v>13</v>
       </c>
       <c r="H13" t="s">
-        <v>171</v>
+        <v>86</v>
       </c>
       <c r="J13" s="3" t="s">
         <v>20</v>
@@ -1537,13 +1516,13 @@
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>101</v>
+        <v>32</v>
       </c>
       <c r="B14" t="s">
-        <v>102</v>
+        <v>25</v>
       </c>
       <c r="C14" t="s">
-        <v>103</v>
+        <v>23</v>
       </c>
       <c r="D14" t="s">
         <v>10</v>
@@ -1552,13 +1531,13 @@
         <v>11</v>
       </c>
       <c r="F14" t="s">
-        <v>27</v>
+        <v>48</v>
       </c>
       <c r="G14" t="s">
         <v>13</v>
       </c>
       <c r="H14" t="s">
-        <v>104</v>
+        <v>87</v>
       </c>
       <c r="J14" s="3" t="s">
         <v>20</v>
@@ -1566,13 +1545,13 @@
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>34</v>
+        <v>88</v>
       </c>
       <c r="B15" t="s">
-        <v>25</v>
+        <v>89</v>
       </c>
       <c r="C15" t="s">
-        <v>23</v>
+        <v>90</v>
       </c>
       <c r="D15" t="s">
         <v>10</v>
@@ -1581,27 +1560,27 @@
         <v>11</v>
       </c>
       <c r="F15" t="s">
-        <v>55</v>
+        <v>19</v>
       </c>
       <c r="G15" t="s">
         <v>13</v>
       </c>
       <c r="H15" t="s">
-        <v>105</v>
+        <v>91</v>
       </c>
       <c r="J15" s="3" t="s">
-        <v>20</v>
+        <v>92</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>106</v>
+        <v>93</v>
       </c>
       <c r="B16" t="s">
-        <v>107</v>
+        <v>94</v>
       </c>
       <c r="C16" t="s">
-        <v>108</v>
+        <v>95</v>
       </c>
       <c r="D16" t="s">
         <v>10</v>
@@ -1610,27 +1589,27 @@
         <v>11</v>
       </c>
       <c r="F16" t="s">
-        <v>33</v>
+        <v>19</v>
       </c>
       <c r="G16" t="s">
         <v>13</v>
       </c>
       <c r="H16" t="s">
-        <v>109</v>
+        <v>96</v>
       </c>
       <c r="J16" s="3" t="s">
-        <v>110</v>
+        <v>92</v>
       </c>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>111</v>
+        <v>88</v>
       </c>
       <c r="B17" t="s">
-        <v>112</v>
+        <v>89</v>
       </c>
       <c r="C17" t="s">
-        <v>113</v>
+        <v>90</v>
       </c>
       <c r="D17" t="s">
         <v>10</v>
@@ -1639,27 +1618,27 @@
         <v>11</v>
       </c>
       <c r="F17" t="s">
-        <v>33</v>
+        <v>21</v>
       </c>
       <c r="G17" t="s">
         <v>13</v>
       </c>
       <c r="H17" t="s">
-        <v>114</v>
+        <v>97</v>
       </c>
       <c r="J17" s="3" t="s">
-        <v>110</v>
+        <v>92</v>
       </c>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>106</v>
+        <v>98</v>
       </c>
       <c r="B18" t="s">
-        <v>107</v>
+        <v>99</v>
       </c>
       <c r="C18" t="s">
-        <v>108</v>
+        <v>22</v>
       </c>
       <c r="D18" t="s">
         <v>10</v>
@@ -1668,24 +1647,27 @@
         <v>11</v>
       </c>
       <c r="F18" t="s">
-        <v>55</v>
+        <v>195</v>
       </c>
       <c r="G18" t="s">
         <v>13</v>
       </c>
       <c r="H18" t="s">
-        <v>115</v>
+        <v>129</v>
+      </c>
+      <c r="I18" s="3">
+        <v>28000</v>
       </c>
       <c r="J18" s="3" t="s">
-        <v>110</v>
+        <v>100</v>
       </c>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>116</v>
+        <v>98</v>
       </c>
       <c r="B19" t="s">
-        <v>117</v>
+        <v>82</v>
       </c>
       <c r="C19" t="s">
         <v>22</v>
@@ -1697,27 +1679,27 @@
         <v>11</v>
       </c>
       <c r="F19" t="s">
-        <v>221</v>
+        <v>195</v>
       </c>
       <c r="G19" t="s">
         <v>13</v>
       </c>
       <c r="H19" t="s">
-        <v>150</v>
+        <v>129</v>
       </c>
       <c r="I19" s="3">
         <v>28000</v>
       </c>
       <c r="J19" s="3" t="s">
-        <v>118</v>
+        <v>100</v>
       </c>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>116</v>
+        <v>98</v>
       </c>
       <c r="B20" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C20" t="s">
         <v>22</v>
@@ -1729,27 +1711,27 @@
         <v>11</v>
       </c>
       <c r="F20" t="s">
-        <v>221</v>
+        <v>19</v>
       </c>
       <c r="G20" t="s">
         <v>13</v>
       </c>
       <c r="H20" t="s">
-        <v>150</v>
+        <v>130</v>
       </c>
       <c r="I20" s="3">
         <v>28000</v>
       </c>
       <c r="J20" s="3" t="s">
-        <v>118</v>
+        <v>100</v>
       </c>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>116</v>
+        <v>98</v>
       </c>
       <c r="B21" t="s">
-        <v>117</v>
+        <v>99</v>
       </c>
       <c r="C21" t="s">
         <v>22</v>
@@ -1761,27 +1743,27 @@
         <v>11</v>
       </c>
       <c r="F21" t="s">
-        <v>33</v>
+        <v>21</v>
       </c>
       <c r="G21" t="s">
         <v>13</v>
       </c>
       <c r="H21" t="s">
-        <v>151</v>
+        <v>129</v>
       </c>
       <c r="I21" s="3">
         <v>28000</v>
       </c>
       <c r="J21" s="3" t="s">
-        <v>118</v>
+        <v>100</v>
       </c>
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>116</v>
+        <v>98</v>
       </c>
       <c r="B22" t="s">
-        <v>117</v>
+        <v>82</v>
       </c>
       <c r="C22" t="s">
         <v>22</v>
@@ -1793,27 +1775,27 @@
         <v>11</v>
       </c>
       <c r="F22" t="s">
-        <v>55</v>
+        <v>19</v>
       </c>
       <c r="G22" t="s">
         <v>13</v>
       </c>
       <c r="H22" t="s">
-        <v>150</v>
+        <v>130</v>
       </c>
       <c r="I22" s="3">
         <v>28000</v>
       </c>
       <c r="J22" s="3" t="s">
-        <v>118</v>
+        <v>100</v>
       </c>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>116</v>
+        <v>98</v>
       </c>
       <c r="B23" t="s">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="C23" t="s">
         <v>22</v>
@@ -1825,30 +1807,30 @@
         <v>11</v>
       </c>
       <c r="F23" t="s">
-        <v>33</v>
+        <v>21</v>
       </c>
       <c r="G23" t="s">
         <v>13</v>
       </c>
       <c r="H23" t="s">
-        <v>151</v>
+        <v>129</v>
       </c>
       <c r="I23" s="3">
         <v>28000</v>
       </c>
       <c r="J23" s="3" t="s">
-        <v>118</v>
+        <v>100</v>
       </c>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>116</v>
+        <v>153</v>
       </c>
       <c r="B24" t="s">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="C24" t="s">
-        <v>22</v>
+        <v>113</v>
       </c>
       <c r="D24" t="s">
         <v>10</v>
@@ -1857,30 +1839,27 @@
         <v>11</v>
       </c>
       <c r="F24" t="s">
-        <v>55</v>
+        <v>27</v>
       </c>
       <c r="G24" t="s">
         <v>13</v>
       </c>
       <c r="H24" t="s">
-        <v>150</v>
-      </c>
-      <c r="I24" s="3">
-        <v>28000</v>
+        <v>87</v>
       </c>
       <c r="J24" s="3" t="s">
-        <v>118</v>
+        <v>20</v>
       </c>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>119</v>
+        <v>101</v>
       </c>
       <c r="B25" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C25" t="s">
-        <v>120</v>
+        <v>102</v>
       </c>
       <c r="D25" t="s">
         <v>10</v>
@@ -1889,13 +1868,13 @@
         <v>11</v>
       </c>
       <c r="F25" t="s">
-        <v>33</v>
+        <v>19</v>
       </c>
       <c r="G25" t="s">
         <v>13</v>
       </c>
       <c r="H25" t="s">
-        <v>152</v>
+        <v>131</v>
       </c>
       <c r="J25" s="3" t="s">
         <v>20</v>
@@ -1903,13 +1882,13 @@
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>119</v>
+        <v>101</v>
       </c>
       <c r="B26" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C26" t="s">
-        <v>120</v>
+        <v>102</v>
       </c>
       <c r="D26" t="s">
         <v>10</v>
@@ -1918,13 +1897,13 @@
         <v>11</v>
       </c>
       <c r="F26" t="s">
-        <v>221</v>
+        <v>195</v>
       </c>
       <c r="G26" t="s">
         <v>13</v>
       </c>
       <c r="H26" t="s">
-        <v>153</v>
+        <v>132</v>
       </c>
       <c r="J26" s="3" t="s">
         <v>20</v>
@@ -1932,13 +1911,13 @@
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>119</v>
+        <v>101</v>
       </c>
       <c r="B27" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C27" t="s">
-        <v>120</v>
+        <v>102</v>
       </c>
       <c r="D27" t="s">
         <v>10</v>
@@ -1947,13 +1926,13 @@
         <v>11</v>
       </c>
       <c r="F27" t="s">
-        <v>55</v>
+        <v>21</v>
       </c>
       <c r="G27" t="s">
         <v>13</v>
       </c>
       <c r="H27" t="s">
-        <v>153</v>
+        <v>132</v>
       </c>
       <c r="J27" s="3" t="s">
         <v>20</v>
@@ -1961,13 +1940,13 @@
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>119</v>
+        <v>101</v>
       </c>
       <c r="B28" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C28" t="s">
-        <v>120</v>
+        <v>102</v>
       </c>
       <c r="D28" t="s">
         <v>10</v>
@@ -1976,13 +1955,13 @@
         <v>11</v>
       </c>
       <c r="F28" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="G28" t="s">
         <v>13</v>
       </c>
       <c r="H28" t="s">
-        <v>154</v>
+        <v>133</v>
       </c>
       <c r="J28" s="3" t="s">
         <v>20</v>
@@ -1990,13 +1969,13 @@
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>119</v>
+        <v>101</v>
       </c>
       <c r="B29" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C29" t="s">
-        <v>120</v>
+        <v>102</v>
       </c>
       <c r="D29" t="s">
         <v>10</v>
@@ -2011,7 +1990,7 @@
         <v>13</v>
       </c>
       <c r="H29" t="s">
-        <v>154</v>
+        <v>133</v>
       </c>
       <c r="J29" s="3" t="s">
         <v>20</v>
@@ -2019,13 +1998,13 @@
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>119</v>
+        <v>101</v>
       </c>
       <c r="B30" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C30" t="s">
-        <v>120</v>
+        <v>102</v>
       </c>
       <c r="D30" t="s">
         <v>10</v>
@@ -2034,27 +2013,27 @@
         <v>11</v>
       </c>
       <c r="F30" t="s">
-        <v>224</v>
+        <v>196</v>
       </c>
       <c r="G30" t="s">
         <v>13</v>
       </c>
       <c r="H30" t="s">
-        <v>155</v>
+        <v>134</v>
       </c>
       <c r="J30" s="3" t="s">
-        <v>156</v>
+        <v>135</v>
       </c>
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>119</v>
+        <v>101</v>
       </c>
       <c r="B31" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C31" t="s">
-        <v>120</v>
+        <v>102</v>
       </c>
       <c r="D31" t="s">
         <v>10</v>
@@ -2063,13 +2042,13 @@
         <v>11</v>
       </c>
       <c r="F31" t="s">
-        <v>33</v>
+        <v>19</v>
       </c>
       <c r="G31" t="s">
         <v>13</v>
       </c>
       <c r="H31" t="s">
-        <v>157</v>
+        <v>136</v>
       </c>
       <c r="J31" s="3" t="s">
         <v>20</v>
@@ -2077,13 +2056,13 @@
     </row>
     <row r="32" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>119</v>
+        <v>101</v>
       </c>
       <c r="B32" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C32" t="s">
-        <v>120</v>
+        <v>102</v>
       </c>
       <c r="D32" t="s">
         <v>10</v>
@@ -2092,13 +2071,13 @@
         <v>11</v>
       </c>
       <c r="F32" t="s">
-        <v>221</v>
+        <v>195</v>
       </c>
       <c r="G32" t="s">
         <v>13</v>
       </c>
       <c r="H32" t="s">
-        <v>158</v>
+        <v>137</v>
       </c>
       <c r="J32" s="3" t="s">
         <v>20</v>
@@ -2106,13 +2085,13 @@
     </row>
     <row r="33" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
-        <v>119</v>
+        <v>101</v>
       </c>
       <c r="B33" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C33" t="s">
-        <v>120</v>
+        <v>102</v>
       </c>
       <c r="D33" t="s">
         <v>10</v>
@@ -2121,13 +2100,13 @@
         <v>11</v>
       </c>
       <c r="F33" t="s">
-        <v>55</v>
+        <v>21</v>
       </c>
       <c r="G33" t="s">
         <v>13</v>
       </c>
       <c r="H33" t="s">
-        <v>158</v>
+        <v>137</v>
       </c>
       <c r="J33" s="3" t="s">
         <v>20</v>
@@ -2135,13 +2114,13 @@
     </row>
     <row r="34" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>119</v>
+        <v>101</v>
       </c>
       <c r="B34" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C34" t="s">
-        <v>120</v>
+        <v>102</v>
       </c>
       <c r="D34" t="s">
         <v>10</v>
@@ -2150,13 +2129,13 @@
         <v>11</v>
       </c>
       <c r="F34" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="G34" t="s">
         <v>13</v>
       </c>
       <c r="H34" t="s">
-        <v>159</v>
+        <v>138</v>
       </c>
       <c r="J34" s="3" t="s">
         <v>20</v>
@@ -2164,13 +2143,13 @@
     </row>
     <row r="35" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
-        <v>119</v>
+        <v>101</v>
       </c>
       <c r="B35" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C35" t="s">
-        <v>120</v>
+        <v>102</v>
       </c>
       <c r="D35" t="s">
         <v>10</v>
@@ -2185,7 +2164,7 @@
         <v>13</v>
       </c>
       <c r="H35" t="s">
-        <v>159</v>
+        <v>138</v>
       </c>
       <c r="J35" s="3" t="s">
         <v>20</v>
@@ -2193,13 +2172,13 @@
     </row>
     <row r="36" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>119</v>
+        <v>101</v>
       </c>
       <c r="B36" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C36" t="s">
-        <v>120</v>
+        <v>102</v>
       </c>
       <c r="D36" t="s">
         <v>10</v>
@@ -2208,27 +2187,27 @@
         <v>11</v>
       </c>
       <c r="F36" t="s">
-        <v>224</v>
+        <v>196</v>
       </c>
       <c r="G36" t="s">
         <v>13</v>
       </c>
       <c r="H36" t="s">
-        <v>160</v>
+        <v>139</v>
       </c>
       <c r="J36" s="3" t="s">
-        <v>156</v>
+        <v>135</v>
       </c>
     </row>
     <row r="37" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>121</v>
+        <v>103</v>
       </c>
       <c r="B37" t="s">
         <v>25</v>
       </c>
       <c r="C37" t="s">
-        <v>122</v>
+        <v>104</v>
       </c>
       <c r="D37" t="s">
         <v>10</v>
@@ -2237,13 +2216,13 @@
         <v>11</v>
       </c>
       <c r="F37" t="s">
-        <v>27</v>
+        <v>14</v>
       </c>
       <c r="G37" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="H37" t="s">
-        <v>123</v>
+        <v>105</v>
       </c>
       <c r="J37" s="3" t="s">
         <v>20</v>
@@ -2251,13 +2230,13 @@
     </row>
     <row r="38" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>121</v>
+        <v>103</v>
       </c>
       <c r="B38" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C38" t="s">
-        <v>122</v>
+        <v>104</v>
       </c>
       <c r="D38" t="s">
         <v>10</v>
@@ -2266,13 +2245,13 @@
         <v>11</v>
       </c>
       <c r="F38" t="s">
-        <v>27</v>
+        <v>14</v>
       </c>
       <c r="G38" t="s">
         <v>13</v>
       </c>
       <c r="H38" t="s">
-        <v>123</v>
+        <v>105</v>
       </c>
       <c r="I38" s="3">
         <v>52</v>
@@ -2283,13 +2262,13 @@
     </row>
     <row r="39" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>126</v>
+        <v>106</v>
       </c>
       <c r="B39" t="s">
-        <v>127</v>
+        <v>25</v>
       </c>
       <c r="C39" t="s">
-        <v>128</v>
+        <v>140</v>
       </c>
       <c r="D39" t="s">
         <v>10</v>
@@ -2298,27 +2277,27 @@
         <v>11</v>
       </c>
       <c r="F39" t="s">
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="G39" t="s">
         <v>13</v>
       </c>
       <c r="H39" t="s">
-        <v>193</v>
+        <v>78</v>
       </c>
       <c r="J39" s="3" t="s">
-        <v>129</v>
+        <v>107</v>
       </c>
     </row>
     <row r="40" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>28</v>
+        <v>197</v>
       </c>
       <c r="B40" t="s">
-        <v>130</v>
+        <v>198</v>
       </c>
       <c r="C40" t="s">
-        <v>131</v>
+        <v>199</v>
       </c>
       <c r="D40" t="s">
         <v>10</v>
@@ -2327,27 +2306,27 @@
         <v>11</v>
       </c>
       <c r="F40" t="s">
-        <v>33</v>
+        <v>148</v>
       </c>
       <c r="G40" t="s">
         <v>13</v>
       </c>
       <c r="H40" t="s">
-        <v>132</v>
+        <v>200</v>
       </c>
       <c r="J40" s="3" t="s">
-        <v>129</v>
+        <v>107</v>
       </c>
     </row>
     <row r="41" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
-        <v>227</v>
+        <v>108</v>
       </c>
       <c r="B41" t="s">
-        <v>228</v>
+        <v>109</v>
       </c>
       <c r="C41" t="s">
-        <v>134</v>
+        <v>110</v>
       </c>
       <c r="D41" t="s">
         <v>10</v>
@@ -2356,27 +2335,27 @@
         <v>11</v>
       </c>
       <c r="F41" t="s">
-        <v>27</v>
+        <v>19</v>
       </c>
       <c r="G41" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H41" t="s">
-        <v>229</v>
+        <v>159</v>
       </c>
       <c r="J41" s="3" t="s">
-        <v>125</v>
+        <v>111</v>
       </c>
     </row>
     <row r="42" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
-        <v>227</v>
+        <v>28</v>
       </c>
       <c r="B42" t="s">
-        <v>228</v>
+        <v>112</v>
       </c>
       <c r="C42" t="s">
-        <v>134</v>
+        <v>113</v>
       </c>
       <c r="D42" t="s">
         <v>10</v>
@@ -2385,27 +2364,27 @@
         <v>11</v>
       </c>
       <c r="F42" t="s">
-        <v>225</v>
+        <v>19</v>
       </c>
       <c r="G42" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H42" t="s">
-        <v>229</v>
+        <v>114</v>
       </c>
       <c r="J42" s="3" t="s">
-        <v>125</v>
+        <v>111</v>
       </c>
     </row>
     <row r="43" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
-        <v>133</v>
+        <v>115</v>
       </c>
       <c r="B43" t="s">
-        <v>228</v>
+        <v>201</v>
       </c>
       <c r="C43" t="s">
-        <v>134</v>
+        <v>116</v>
       </c>
       <c r="D43" t="s">
         <v>10</v>
@@ -2414,27 +2393,27 @@
         <v>11</v>
       </c>
       <c r="F43" t="s">
-        <v>225</v>
+        <v>27</v>
       </c>
       <c r="G43" t="s">
         <v>12</v>
       </c>
       <c r="H43" t="s">
-        <v>226</v>
+        <v>202</v>
       </c>
       <c r="J43" s="3" t="s">
-        <v>125</v>
+        <v>107</v>
       </c>
     </row>
     <row r="44" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
-        <v>133</v>
+        <v>115</v>
       </c>
       <c r="B44" t="s">
-        <v>228</v>
+        <v>201</v>
       </c>
       <c r="C44" t="s">
-        <v>134</v>
+        <v>116</v>
       </c>
       <c r="D44" t="s">
         <v>10</v>
@@ -2443,27 +2422,27 @@
         <v>11</v>
       </c>
       <c r="F44" t="s">
-        <v>27</v>
+        <v>177</v>
       </c>
       <c r="G44" t="s">
         <v>12</v>
       </c>
       <c r="H44" t="s">
-        <v>226</v>
+        <v>202</v>
       </c>
       <c r="J44" s="3" t="s">
-        <v>125</v>
+        <v>107</v>
       </c>
     </row>
     <row r="45" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
-        <v>174</v>
+        <v>115</v>
       </c>
       <c r="B45" t="s">
-        <v>175</v>
+        <v>204</v>
       </c>
       <c r="C45" t="s">
-        <v>134</v>
+        <v>116</v>
       </c>
       <c r="D45" t="s">
         <v>10</v>
@@ -2478,21 +2457,21 @@
         <v>12</v>
       </c>
       <c r="H45" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="J45" s="3" t="s">
-        <v>125</v>
+        <v>107</v>
       </c>
     </row>
     <row r="46" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
-        <v>174</v>
+        <v>115</v>
       </c>
       <c r="B46" t="s">
-        <v>175</v>
+        <v>203</v>
       </c>
       <c r="C46" t="s">
-        <v>134</v>
+        <v>116</v>
       </c>
       <c r="D46" t="s">
         <v>10</v>
@@ -2501,27 +2480,27 @@
         <v>11</v>
       </c>
       <c r="F46" t="s">
-        <v>225</v>
+        <v>177</v>
       </c>
       <c r="G46" t="s">
         <v>12</v>
       </c>
       <c r="H46" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="J46" s="3" t="s">
-        <v>125</v>
+        <v>107</v>
       </c>
     </row>
     <row r="47" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
-        <v>133</v>
+        <v>205</v>
       </c>
       <c r="B47" t="s">
-        <v>172</v>
+        <v>145</v>
       </c>
       <c r="C47" t="s">
-        <v>134</v>
+        <v>116</v>
       </c>
       <c r="D47" t="s">
         <v>10</v>
@@ -2530,27 +2509,27 @@
         <v>11</v>
       </c>
       <c r="F47" t="s">
-        <v>225</v>
+        <v>27</v>
       </c>
       <c r="G47" t="s">
         <v>12</v>
       </c>
       <c r="H47" t="s">
-        <v>173</v>
+        <v>146</v>
       </c>
       <c r="J47" s="3" t="s">
-        <v>125</v>
+        <v>107</v>
       </c>
     </row>
     <row r="48" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
-        <v>133</v>
+        <v>205</v>
       </c>
       <c r="B48" t="s">
-        <v>172</v>
+        <v>145</v>
       </c>
       <c r="C48" t="s">
-        <v>134</v>
+        <v>116</v>
       </c>
       <c r="D48" t="s">
         <v>10</v>
@@ -2559,114 +2538,114 @@
         <v>11</v>
       </c>
       <c r="F48" t="s">
-        <v>27</v>
+        <v>177</v>
       </c>
       <c r="G48" t="s">
         <v>12</v>
       </c>
       <c r="H48" t="s">
-        <v>173</v>
+        <v>146</v>
       </c>
       <c r="J48" s="3" t="s">
-        <v>125</v>
+        <v>107</v>
       </c>
     </row>
     <row r="49" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
-        <v>139</v>
+        <v>179</v>
       </c>
       <c r="B49" t="s">
-        <v>136</v>
+        <v>180</v>
       </c>
       <c r="C49" t="s">
-        <v>22</v>
+        <v>116</v>
       </c>
       <c r="D49" t="s">
-        <v>138</v>
+        <v>10</v>
       </c>
       <c r="E49" t="s">
         <v>11</v>
       </c>
       <c r="F49" t="s">
-        <v>19</v>
+        <v>27</v>
       </c>
       <c r="G49" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="H49" t="s">
-        <v>171</v>
-      </c>
-      <c r="I49" s="3">
-        <v>49</v>
+        <v>181</v>
+      </c>
+      <c r="J49" s="3" t="s">
+        <v>107</v>
       </c>
     </row>
     <row r="50" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
-        <v>135</v>
+        <v>179</v>
       </c>
       <c r="B50" t="s">
-        <v>136</v>
+        <v>180</v>
       </c>
       <c r="C50" t="s">
-        <v>137</v>
+        <v>116</v>
       </c>
       <c r="D50" t="s">
-        <v>138</v>
+        <v>10</v>
       </c>
       <c r="E50" t="s">
         <v>11</v>
       </c>
       <c r="F50" t="s">
-        <v>19</v>
+        <v>177</v>
       </c>
       <c r="G50" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="H50" t="s">
-        <v>180</v>
-      </c>
-      <c r="I50" s="3">
-        <v>49</v>
+        <v>181</v>
+      </c>
+      <c r="J50" s="3" t="s">
+        <v>107</v>
       </c>
     </row>
     <row r="51" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
-        <v>139</v>
+        <v>115</v>
       </c>
       <c r="B51" t="s">
-        <v>26</v>
+        <v>180</v>
       </c>
       <c r="C51" t="s">
-        <v>22</v>
+        <v>116</v>
       </c>
       <c r="D51" t="s">
-        <v>138</v>
+        <v>10</v>
       </c>
       <c r="E51" t="s">
         <v>11</v>
       </c>
       <c r="F51" t="s">
-        <v>27</v>
+        <v>177</v>
       </c>
       <c r="G51" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="H51" t="s">
-        <v>140</v>
-      </c>
-      <c r="I51" s="3">
-        <v>49</v>
+        <v>178</v>
+      </c>
+      <c r="J51" s="3" t="s">
+        <v>107</v>
       </c>
     </row>
     <row r="52" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
-        <v>144</v>
+        <v>115</v>
       </c>
       <c r="B52" t="s">
-        <v>100</v>
+        <v>180</v>
       </c>
       <c r="C52" t="s">
-        <v>145</v>
+        <v>116</v>
       </c>
       <c r="D52" t="s">
         <v>10</v>
@@ -2675,13 +2654,16 @@
         <v>11</v>
       </c>
       <c r="F52" t="s">
-        <v>19</v>
+        <v>27</v>
       </c>
       <c r="G52" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="H52" t="s">
-        <v>146</v>
+        <v>178</v>
+      </c>
+      <c r="J52" s="3" t="s">
+        <v>107</v>
       </c>
     </row>
     <row r="53" spans="1:10" x14ac:dyDescent="0.3">
@@ -2689,10 +2671,10 @@
         <v>144</v>
       </c>
       <c r="B53" t="s">
-        <v>100</v>
+        <v>145</v>
       </c>
       <c r="C53" t="s">
-        <v>145</v>
+        <v>116</v>
       </c>
       <c r="D53" t="s">
         <v>10</v>
@@ -2701,27 +2683,27 @@
         <v>11</v>
       </c>
       <c r="F53" t="s">
-        <v>147</v>
+        <v>27</v>
       </c>
       <c r="G53" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="H53" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="J53" s="3" t="s">
-        <v>149</v>
+        <v>107</v>
       </c>
     </row>
     <row r="54" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
-        <v>31</v>
+        <v>144</v>
       </c>
       <c r="B54" t="s">
-        <v>32</v>
+        <v>145</v>
       </c>
       <c r="C54" t="s">
-        <v>22</v>
+        <v>116</v>
       </c>
       <c r="D54" t="s">
         <v>10</v>
@@ -2730,27 +2712,27 @@
         <v>11</v>
       </c>
       <c r="F54" t="s">
-        <v>19</v>
+        <v>177</v>
       </c>
       <c r="G54" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="H54" t="s">
-        <v>230</v>
+        <v>146</v>
       </c>
       <c r="J54" s="3" t="s">
-        <v>204</v>
+        <v>107</v>
       </c>
     </row>
     <row r="55" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
-        <v>31</v>
+        <v>115</v>
       </c>
       <c r="B55" t="s">
-        <v>26</v>
+        <v>142</v>
       </c>
       <c r="C55" t="s">
-        <v>22</v>
+        <v>116</v>
       </c>
       <c r="D55" t="s">
         <v>10</v>
@@ -2759,27 +2741,27 @@
         <v>11</v>
       </c>
       <c r="F55" t="s">
-        <v>19</v>
+        <v>177</v>
       </c>
       <c r="G55" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="H55" t="s">
-        <v>203</v>
+        <v>143</v>
       </c>
       <c r="J55" s="3" t="s">
-        <v>204</v>
+        <v>107</v>
       </c>
     </row>
     <row r="56" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
-        <v>198</v>
+        <v>115</v>
       </c>
       <c r="B56" t="s">
-        <v>199</v>
+        <v>142</v>
       </c>
       <c r="C56" t="s">
-        <v>142</v>
+        <v>116</v>
       </c>
       <c r="D56" t="s">
         <v>10</v>
@@ -2788,24 +2770,30 @@
         <v>11</v>
       </c>
       <c r="F56" t="s">
-        <v>19</v>
+        <v>27</v>
       </c>
       <c r="G56" t="s">
-        <v>13</v>
+        <v>12</v>
+      </c>
+      <c r="H56" t="s">
+        <v>143</v>
+      </c>
+      <c r="J56" s="3" t="s">
+        <v>107</v>
       </c>
     </row>
     <row r="57" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
-        <v>199</v>
+        <v>121</v>
       </c>
       <c r="B57" t="s">
-        <v>231</v>
+        <v>118</v>
       </c>
       <c r="C57" t="s">
-        <v>30</v>
+        <v>22</v>
       </c>
       <c r="D57" t="s">
-        <v>10</v>
+        <v>120</v>
       </c>
       <c r="E57" t="s">
         <v>11</v>
@@ -2817,70 +2805,79 @@
         <v>13</v>
       </c>
       <c r="H57" t="s">
-        <v>143</v>
+        <v>141</v>
+      </c>
+      <c r="I57" s="3">
+        <v>49</v>
       </c>
     </row>
     <row r="58" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
-        <v>170</v>
+        <v>117</v>
       </c>
       <c r="B58" t="s">
-        <v>207</v>
+        <v>118</v>
       </c>
       <c r="C58" t="s">
-        <v>30</v>
+        <v>119</v>
       </c>
       <c r="D58" t="s">
-        <v>10</v>
+        <v>120</v>
       </c>
       <c r="E58" t="s">
         <v>11</v>
       </c>
       <c r="F58" t="s">
-        <v>27</v>
+        <v>19</v>
       </c>
       <c r="G58" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H58" t="s">
-        <v>208</v>
+        <v>150</v>
+      </c>
+      <c r="I58" s="3">
+        <v>49</v>
       </c>
     </row>
     <row r="59" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
-        <v>170</v>
+        <v>121</v>
       </c>
       <c r="B59" t="s">
-        <v>167</v>
+        <v>26</v>
       </c>
       <c r="C59" t="s">
-        <v>30</v>
+        <v>22</v>
       </c>
       <c r="D59" t="s">
-        <v>10</v>
+        <v>120</v>
       </c>
       <c r="E59" t="s">
         <v>11</v>
       </c>
       <c r="F59" t="s">
-        <v>19</v>
+        <v>27</v>
       </c>
       <c r="G59" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H59" t="s">
-        <v>209</v>
+        <v>122</v>
+      </c>
+      <c r="I59" s="3">
+        <v>49</v>
       </c>
     </row>
     <row r="60" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
-        <v>162</v>
+        <v>123</v>
       </c>
       <c r="B60" t="s">
-        <v>163</v>
+        <v>171</v>
       </c>
       <c r="C60" t="s">
-        <v>164</v>
+        <v>124</v>
       </c>
       <c r="D60" t="s">
         <v>10</v>
@@ -2889,24 +2886,24 @@
         <v>11</v>
       </c>
       <c r="F60" t="s">
-        <v>27</v>
+        <v>19</v>
       </c>
       <c r="G60" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H60" t="s">
-        <v>200</v>
+        <v>172</v>
       </c>
     </row>
     <row r="61" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
-        <v>184</v>
+        <v>123</v>
       </c>
       <c r="B61" t="s">
-        <v>165</v>
+        <v>82</v>
       </c>
       <c r="C61" t="s">
-        <v>164</v>
+        <v>124</v>
       </c>
       <c r="D61" t="s">
         <v>10</v>
@@ -2915,24 +2912,24 @@
         <v>11</v>
       </c>
       <c r="F61" t="s">
-        <v>27</v>
+        <v>19</v>
       </c>
       <c r="G61" t="s">
         <v>13</v>
       </c>
       <c r="H61" t="s">
-        <v>185</v>
+        <v>125</v>
       </c>
     </row>
     <row r="62" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
-        <v>166</v>
+        <v>123</v>
       </c>
       <c r="B62" t="s">
-        <v>167</v>
+        <v>82</v>
       </c>
       <c r="C62" t="s">
-        <v>164</v>
+        <v>124</v>
       </c>
       <c r="D62" t="s">
         <v>10</v>
@@ -2941,24 +2938,27 @@
         <v>11</v>
       </c>
       <c r="F62" t="s">
-        <v>27</v>
+        <v>126</v>
       </c>
       <c r="G62" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H62" t="s">
-        <v>232</v>
+        <v>127</v>
+      </c>
+      <c r="J62" s="3" t="s">
+        <v>128</v>
       </c>
     </row>
     <row r="63" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
-        <v>205</v>
+        <v>30</v>
       </c>
       <c r="B63" t="s">
-        <v>168</v>
+        <v>31</v>
       </c>
       <c r="C63" t="s">
-        <v>30</v>
+        <v>22</v>
       </c>
       <c r="D63" t="s">
         <v>10</v>
@@ -2967,24 +2967,27 @@
         <v>11</v>
       </c>
       <c r="F63" t="s">
-        <v>27</v>
+        <v>19</v>
       </c>
       <c r="G63" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H63" t="s">
-        <v>206</v>
+        <v>182</v>
+      </c>
+      <c r="J63" s="3" t="s">
+        <v>163</v>
       </c>
     </row>
     <row r="64" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
-        <v>141</v>
+        <v>30</v>
       </c>
       <c r="B64" t="s">
-        <v>168</v>
+        <v>26</v>
       </c>
       <c r="C64" t="s">
-        <v>30</v>
+        <v>22</v>
       </c>
       <c r="D64" t="s">
         <v>10</v>
@@ -2993,417 +2996,414 @@
         <v>11</v>
       </c>
       <c r="F64" t="s">
-        <v>27</v>
+        <v>19</v>
       </c>
       <c r="G64" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H64" t="s">
-        <v>169</v>
+        <v>162</v>
+      </c>
+      <c r="J64" s="3" t="s">
+        <v>163</v>
       </c>
     </row>
     <row r="65" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
-        <v>64</v>
+        <v>69</v>
       </c>
       <c r="B65" t="s">
-        <v>65</v>
+        <v>206</v>
       </c>
       <c r="C65" t="s">
-        <v>36</v>
+        <v>207</v>
       </c>
       <c r="D65" t="s">
-        <v>37</v>
+        <v>10</v>
       </c>
       <c r="E65" t="s">
         <v>11</v>
       </c>
       <c r="F65" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="G65" t="s">
-        <v>58</v>
-      </c>
-      <c r="J65" s="3" t="s">
-        <v>50</v>
+        <v>12</v>
       </c>
     </row>
     <row r="66" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
-        <v>64</v>
+        <v>32</v>
       </c>
       <c r="B66" t="s">
-        <v>64</v>
+        <v>206</v>
       </c>
       <c r="C66" t="s">
-        <v>36</v>
+        <v>207</v>
       </c>
       <c r="D66" t="s">
-        <v>37</v>
+        <v>10</v>
       </c>
       <c r="E66" t="s">
         <v>11</v>
       </c>
       <c r="F66" t="s">
-        <v>66</v>
+        <v>19</v>
       </c>
       <c r="G66" t="s">
-        <v>63</v>
-      </c>
-      <c r="J66" s="3" t="s">
-        <v>67</v>
+        <v>12</v>
       </c>
     </row>
     <row r="67" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="B67" t="s">
-        <v>64</v>
+        <v>58</v>
       </c>
       <c r="C67" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="D67" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="E67" t="s">
         <v>11</v>
       </c>
       <c r="F67" t="s">
-        <v>61</v>
+        <v>17</v>
       </c>
       <c r="G67" t="s">
-        <v>58</v>
+        <v>51</v>
       </c>
       <c r="J67" s="3" t="s">
-        <v>50</v>
+        <v>44</v>
       </c>
     </row>
     <row r="68" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="B68" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="C68" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="D68" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="E68" t="s">
         <v>11</v>
       </c>
       <c r="F68" t="s">
-        <v>14</v>
+        <v>59</v>
       </c>
       <c r="G68" t="s">
-        <v>63</v>
+        <v>56</v>
       </c>
       <c r="J68" s="3" t="s">
-        <v>68</v>
+        <v>208</v>
       </c>
     </row>
     <row r="69" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
-        <v>44</v>
+        <v>57</v>
       </c>
       <c r="B69" t="s">
-        <v>45</v>
+        <v>57</v>
       </c>
       <c r="C69" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="D69" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="E69" t="s">
         <v>11</v>
       </c>
       <c r="F69" t="s">
-        <v>46</v>
+        <v>54</v>
       </c>
       <c r="G69" t="s">
-        <v>38</v>
+        <v>51</v>
       </c>
       <c r="J69" s="3" t="s">
-        <v>47</v>
+        <v>209</v>
       </c>
     </row>
     <row r="70" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
-        <v>44</v>
+        <v>57</v>
       </c>
       <c r="B70" t="s">
-        <v>48</v>
+        <v>57</v>
       </c>
       <c r="C70" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="D70" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="E70" t="s">
         <v>11</v>
       </c>
       <c r="F70" t="s">
-        <v>46</v>
+        <v>14</v>
       </c>
       <c r="G70" t="s">
-        <v>38</v>
+        <v>56</v>
       </c>
       <c r="J70" s="3" t="s">
-        <v>47</v>
+        <v>210</v>
       </c>
     </row>
     <row r="71" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="B71" t="s">
-        <v>49</v>
+        <v>40</v>
       </c>
       <c r="C71" t="s">
+        <v>34</v>
+      </c>
+      <c r="D71" t="s">
+        <v>35</v>
+      </c>
+      <c r="E71" t="s">
+        <v>11</v>
+      </c>
+      <c r="F71" t="s">
+        <v>41</v>
+      </c>
+      <c r="G71" t="s">
         <v>36</v>
       </c>
-      <c r="D71" t="s">
-        <v>37</v>
-      </c>
-      <c r="E71" t="s">
-        <v>11</v>
-      </c>
-      <c r="F71" t="s">
-        <v>46</v>
-      </c>
-      <c r="G71" t="s">
-        <v>38</v>
-      </c>
       <c r="J71" s="3" t="s">
-        <v>47</v>
+        <v>211</v>
       </c>
     </row>
     <row r="72" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="B72" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="C72" t="s">
+        <v>34</v>
+      </c>
+      <c r="D72" t="s">
+        <v>35</v>
+      </c>
+      <c r="E72" t="s">
+        <v>11</v>
+      </c>
+      <c r="F72" t="s">
+        <v>41</v>
+      </c>
+      <c r="G72" t="s">
         <v>36</v>
       </c>
-      <c r="D72" t="s">
-        <v>37</v>
-      </c>
-      <c r="E72" t="s">
-        <v>11</v>
-      </c>
-      <c r="F72" t="s">
-        <v>46</v>
-      </c>
-      <c r="G72" t="s">
-        <v>38</v>
-      </c>
       <c r="J72" s="3" t="s">
-        <v>47</v>
+        <v>211</v>
       </c>
     </row>
     <row r="73" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
-        <v>51</v>
+        <v>39</v>
       </c>
       <c r="B73" t="s">
-        <v>51</v>
+        <v>43</v>
       </c>
       <c r="C73" t="s">
+        <v>34</v>
+      </c>
+      <c r="D73" t="s">
+        <v>35</v>
+      </c>
+      <c r="E73" t="s">
+        <v>11</v>
+      </c>
+      <c r="F73" t="s">
+        <v>41</v>
+      </c>
+      <c r="G73" t="s">
         <v>36</v>
       </c>
-      <c r="D73" t="s">
-        <v>37</v>
-      </c>
-      <c r="E73" t="s">
-        <v>11</v>
-      </c>
-      <c r="F73" t="s">
-        <v>46</v>
-      </c>
-      <c r="G73" t="s">
-        <v>38</v>
-      </c>
       <c r="J73" s="3" t="s">
-        <v>50</v>
+        <v>211</v>
       </c>
     </row>
     <row r="74" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
-        <v>52</v>
+        <v>39</v>
       </c>
       <c r="B74" t="s">
-        <v>52</v>
+        <v>39</v>
       </c>
       <c r="C74" t="s">
+        <v>34</v>
+      </c>
+      <c r="D74" t="s">
+        <v>35</v>
+      </c>
+      <c r="E74" t="s">
+        <v>11</v>
+      </c>
+      <c r="F74" t="s">
+        <v>41</v>
+      </c>
+      <c r="G74" t="s">
         <v>36</v>
       </c>
-      <c r="D74" t="s">
-        <v>37</v>
-      </c>
-      <c r="E74" t="s">
-        <v>11</v>
-      </c>
-      <c r="F74" t="s">
-        <v>46</v>
-      </c>
-      <c r="G74" t="s">
-        <v>58</v>
-      </c>
       <c r="J74" s="3" t="s">
-        <v>53</v>
+        <v>211</v>
       </c>
     </row>
     <row r="75" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
-        <v>34</v>
+        <v>45</v>
       </c>
       <c r="B75" t="s">
-        <v>34</v>
+        <v>45</v>
       </c>
       <c r="C75" t="s">
+        <v>34</v>
+      </c>
+      <c r="D75" t="s">
+        <v>35</v>
+      </c>
+      <c r="E75" t="s">
+        <v>11</v>
+      </c>
+      <c r="F75" t="s">
+        <v>41</v>
+      </c>
+      <c r="G75" t="s">
         <v>36</v>
       </c>
-      <c r="D75" t="s">
-        <v>54</v>
-      </c>
-      <c r="E75" t="s">
-        <v>11</v>
-      </c>
-      <c r="F75" t="s">
-        <v>55</v>
-      </c>
-      <c r="G75" t="s">
-        <v>38</v>
-      </c>
       <c r="J75" s="3" t="s">
-        <v>50</v>
+        <v>209</v>
       </c>
     </row>
     <row r="76" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A76" t="s">
-        <v>34</v>
+        <v>46</v>
       </c>
       <c r="B76" t="s">
-        <v>34</v>
+        <v>46</v>
       </c>
       <c r="C76" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="D76" t="s">
-        <v>54</v>
+        <v>35</v>
       </c>
       <c r="E76" t="s">
         <v>11</v>
       </c>
       <c r="F76" t="s">
-        <v>56</v>
+        <v>41</v>
       </c>
       <c r="G76" t="s">
-        <v>38</v>
+        <v>51</v>
       </c>
       <c r="J76" s="3" t="s">
-        <v>50</v>
+        <v>212</v>
       </c>
     </row>
     <row r="77" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A77" t="s">
-        <v>57</v>
+        <v>32</v>
       </c>
       <c r="B77" t="s">
-        <v>57</v>
+        <v>32</v>
       </c>
       <c r="C77" t="s">
+        <v>34</v>
+      </c>
+      <c r="D77" t="s">
+        <v>47</v>
+      </c>
+      <c r="E77" t="s">
+        <v>11</v>
+      </c>
+      <c r="F77" t="s">
+        <v>48</v>
+      </c>
+      <c r="G77" t="s">
         <v>36</v>
       </c>
-      <c r="D77" t="s">
-        <v>37</v>
-      </c>
-      <c r="E77" t="s">
-        <v>11</v>
-      </c>
-      <c r="F77" t="s">
-        <v>56</v>
-      </c>
-      <c r="G77" t="s">
-        <v>58</v>
-      </c>
       <c r="J77" s="3" t="s">
-        <v>59</v>
+        <v>209</v>
       </c>
     </row>
     <row r="78" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A78" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="B78" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="C78" t="s">
+        <v>34</v>
+      </c>
+      <c r="D78" t="s">
+        <v>47</v>
+      </c>
+      <c r="E78" t="s">
+        <v>11</v>
+      </c>
+      <c r="F78" t="s">
+        <v>49</v>
+      </c>
+      <c r="G78" t="s">
         <v>36</v>
       </c>
-      <c r="D78" t="s">
-        <v>37</v>
-      </c>
-      <c r="E78" t="s">
-        <v>11</v>
-      </c>
-      <c r="F78" t="s">
-        <v>17</v>
-      </c>
-      <c r="G78" t="s">
-        <v>38</v>
-      </c>
       <c r="J78" s="3" t="s">
-        <v>39</v>
+        <v>209</v>
       </c>
     </row>
     <row r="79" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A79" t="s">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="B79" t="s">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="C79" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="D79" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="E79" t="s">
         <v>11</v>
       </c>
       <c r="F79" t="s">
-        <v>17</v>
+        <v>49</v>
       </c>
       <c r="G79" t="s">
-        <v>38</v>
+        <v>51</v>
       </c>
       <c r="J79" s="3" t="s">
-        <v>41</v>
+        <v>52</v>
       </c>
     </row>
     <row r="80" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A80" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="B80" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="C80" t="s">
-        <v>42</v>
+        <v>34</v>
       </c>
       <c r="D80" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="E80" t="s">
         <v>11</v>
@@ -3412,180 +3412,180 @@
         <v>17</v>
       </c>
       <c r="G80" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="J80" s="3" t="s">
-        <v>43</v>
+        <v>213</v>
       </c>
     </row>
     <row r="81" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A81" t="s">
-        <v>181</v>
+        <v>37</v>
       </c>
       <c r="B81" t="s">
-        <v>181</v>
+        <v>37</v>
       </c>
       <c r="C81" t="s">
+        <v>34</v>
+      </c>
+      <c r="D81" t="s">
+        <v>35</v>
+      </c>
+      <c r="E81" t="s">
+        <v>11</v>
+      </c>
+      <c r="F81" t="s">
+        <v>17</v>
+      </c>
+      <c r="G81" t="s">
         <v>36</v>
       </c>
-      <c r="D81" t="s">
-        <v>37</v>
-      </c>
-      <c r="E81" t="s">
-        <v>11</v>
-      </c>
-      <c r="F81" t="s">
-        <v>178</v>
-      </c>
-      <c r="G81" t="s">
-        <v>38</v>
-      </c>
       <c r="J81" s="3" t="s">
-        <v>182</v>
+        <v>214</v>
       </c>
     </row>
     <row r="82" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A82" t="s">
-        <v>69</v>
+        <v>37</v>
       </c>
       <c r="B82" t="s">
-        <v>69</v>
+        <v>37</v>
       </c>
       <c r="C82" t="s">
+        <v>38</v>
+      </c>
+      <c r="D82" t="s">
+        <v>35</v>
+      </c>
+      <c r="E82" t="s">
+        <v>11</v>
+      </c>
+      <c r="F82" t="s">
+        <v>17</v>
+      </c>
+      <c r="G82" t="s">
         <v>36</v>
       </c>
-      <c r="D82" t="s">
-        <v>37</v>
-      </c>
-      <c r="E82" t="s">
-        <v>11</v>
-      </c>
-      <c r="F82" t="s">
-        <v>183</v>
-      </c>
-      <c r="G82" t="s">
-        <v>63</v>
-      </c>
       <c r="J82" s="3" t="s">
-        <v>50</v>
+        <v>215</v>
       </c>
     </row>
     <row r="83" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A83" t="s">
-        <v>25</v>
+        <v>151</v>
       </c>
       <c r="B83" t="s">
-        <v>25</v>
+        <v>151</v>
       </c>
       <c r="C83" t="s">
+        <v>34</v>
+      </c>
+      <c r="D83" t="s">
+        <v>35</v>
+      </c>
+      <c r="E83" t="s">
+        <v>11</v>
+      </c>
+      <c r="F83" t="s">
+        <v>148</v>
+      </c>
+      <c r="G83" t="s">
         <v>36</v>
       </c>
-      <c r="D83" t="s">
-        <v>37</v>
-      </c>
-      <c r="E83" t="s">
-        <v>11</v>
-      </c>
-      <c r="F83" t="s">
-        <v>61</v>
-      </c>
-      <c r="G83" t="s">
-        <v>58</v>
-      </c>
       <c r="J83" s="3" t="s">
-        <v>70</v>
+        <v>216</v>
       </c>
     </row>
     <row r="84" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A84" t="s">
-        <v>233</v>
+        <v>60</v>
       </c>
       <c r="B84" t="s">
-        <v>233</v>
+        <v>60</v>
       </c>
       <c r="C84" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="D84" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="E84" t="s">
         <v>11</v>
       </c>
       <c r="F84" t="s">
-        <v>61</v>
+        <v>152</v>
       </c>
       <c r="G84" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="J84" s="3" t="s">
-        <v>50</v>
+        <v>209</v>
       </c>
     </row>
     <row r="85" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A85" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="B85" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="C85" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="D85" t="s">
+        <v>35</v>
+      </c>
+      <c r="E85" t="s">
+        <v>11</v>
+      </c>
+      <c r="F85" t="s">
         <v>54</v>
       </c>
-      <c r="E85" t="s">
-        <v>11</v>
-      </c>
-      <c r="F85" t="s">
-        <v>14</v>
-      </c>
       <c r="G85" t="s">
-        <v>71</v>
+        <v>51</v>
       </c>
       <c r="J85" s="3" t="s">
-        <v>72</v>
+        <v>217</v>
       </c>
     </row>
     <row r="86" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A86" t="s">
-        <v>28</v>
+        <v>183</v>
       </c>
       <c r="B86" t="s">
-        <v>28</v>
+        <v>183</v>
       </c>
       <c r="C86" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="D86" t="s">
+        <v>35</v>
+      </c>
+      <c r="E86" t="s">
+        <v>11</v>
+      </c>
+      <c r="F86" t="s">
         <v>54</v>
       </c>
-      <c r="E86" t="s">
-        <v>11</v>
-      </c>
-      <c r="F86" t="s">
-        <v>16</v>
-      </c>
       <c r="G86" t="s">
-        <v>71</v>
+        <v>51</v>
       </c>
       <c r="J86" s="3" t="s">
-        <v>72</v>
+        <v>209</v>
       </c>
     </row>
     <row r="87" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A87" t="s">
-        <v>73</v>
+        <v>28</v>
       </c>
       <c r="B87" t="s">
-        <v>73</v>
+        <v>28</v>
       </c>
       <c r="C87" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="D87" t="s">
-        <v>54</v>
+        <v>47</v>
       </c>
       <c r="E87" t="s">
         <v>11</v>
@@ -3594,62 +3594,62 @@
         <v>14</v>
       </c>
       <c r="G87" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="J87" s="3" t="s">
-        <v>72</v>
+        <v>62</v>
       </c>
     </row>
     <row r="88" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A88" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B88" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C88" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="D88" t="s">
-        <v>54</v>
+        <v>47</v>
       </c>
       <c r="E88" t="s">
         <v>11</v>
       </c>
       <c r="F88" t="s">
-        <v>178</v>
+        <v>16</v>
       </c>
       <c r="G88" t="s">
-        <v>71</v>
+        <v>61</v>
       </c>
       <c r="J88" s="3" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
     </row>
     <row r="89" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A89" t="s">
-        <v>29</v>
+        <v>63</v>
       </c>
       <c r="B89" t="s">
-        <v>29</v>
+        <v>63</v>
       </c>
       <c r="C89" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="D89" t="s">
-        <v>54</v>
+        <v>47</v>
       </c>
       <c r="E89" t="s">
         <v>11</v>
       </c>
       <c r="F89" t="s">
-        <v>187</v>
+        <v>14</v>
       </c>
       <c r="G89" t="s">
-        <v>71</v>
+        <v>56</v>
       </c>
       <c r="J89" s="3" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
     </row>
     <row r="90" spans="1:10" x14ac:dyDescent="0.3">
@@ -3660,77 +3660,74 @@
         <v>29</v>
       </c>
       <c r="C90" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="D90" t="s">
-        <v>54</v>
+        <v>47</v>
       </c>
       <c r="E90" t="s">
         <v>11</v>
       </c>
       <c r="F90" t="s">
-        <v>56</v>
+        <v>148</v>
       </c>
       <c r="G90" t="s">
-        <v>71</v>
+        <v>61</v>
       </c>
       <c r="J90" s="3" t="s">
-        <v>60</v>
+        <v>53</v>
       </c>
     </row>
     <row r="91" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A91" t="s">
-        <v>18</v>
+        <v>29</v>
       </c>
       <c r="B91" t="s">
-        <v>210</v>
+        <v>29</v>
       </c>
       <c r="C91" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="D91" t="s">
-        <v>37</v>
+        <v>47</v>
       </c>
       <c r="E91" t="s">
         <v>11</v>
       </c>
       <c r="F91" t="s">
-        <v>24</v>
+        <v>154</v>
       </c>
       <c r="G91" t="s">
-        <v>38</v>
+        <v>61</v>
       </c>
       <c r="J91" s="3" t="s">
-        <v>211</v>
+        <v>53</v>
       </c>
     </row>
     <row r="92" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A92" t="s">
-        <v>18</v>
+        <v>29</v>
       </c>
       <c r="B92" t="s">
-        <v>212</v>
+        <v>29</v>
       </c>
       <c r="C92" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="D92" t="s">
-        <v>37</v>
+        <v>47</v>
       </c>
       <c r="E92" t="s">
         <v>11</v>
       </c>
       <c r="F92" t="s">
-        <v>99</v>
+        <v>49</v>
       </c>
       <c r="G92" t="s">
-        <v>38</v>
-      </c>
-      <c r="H92" t="s">
-        <v>213</v>
+        <v>61</v>
       </c>
       <c r="J92" s="3" t="s">
-        <v>211</v>
+        <v>53</v>
       </c>
     </row>
     <row r="93" spans="1:10" x14ac:dyDescent="0.3">
@@ -3738,28 +3735,25 @@
         <v>18</v>
       </c>
       <c r="B93" t="s">
-        <v>214</v>
+        <v>164</v>
       </c>
       <c r="C93" t="s">
+        <v>34</v>
+      </c>
+      <c r="D93" t="s">
+        <v>35</v>
+      </c>
+      <c r="E93" t="s">
+        <v>11</v>
+      </c>
+      <c r="F93" t="s">
+        <v>24</v>
+      </c>
+      <c r="G93" t="s">
         <v>36</v>
       </c>
-      <c r="D93" t="s">
-        <v>37</v>
-      </c>
-      <c r="E93" t="s">
-        <v>11</v>
-      </c>
-      <c r="F93" t="s">
-        <v>99</v>
-      </c>
-      <c r="G93" t="s">
-        <v>38</v>
-      </c>
-      <c r="H93" t="s">
-        <v>213</v>
-      </c>
       <c r="J93" s="3" t="s">
-        <v>211</v>
+        <v>165</v>
       </c>
     </row>
     <row r="94" spans="1:10" x14ac:dyDescent="0.3">
@@ -3767,25 +3761,28 @@
         <v>18</v>
       </c>
       <c r="B94" t="s">
-        <v>215</v>
+        <v>166</v>
       </c>
       <c r="C94" t="s">
+        <v>34</v>
+      </c>
+      <c r="D94" t="s">
+        <v>35</v>
+      </c>
+      <c r="E94" t="s">
+        <v>11</v>
+      </c>
+      <c r="F94" t="s">
+        <v>81</v>
+      </c>
+      <c r="G94" t="s">
         <v>36</v>
       </c>
-      <c r="D94" t="s">
-        <v>37</v>
-      </c>
-      <c r="E94" t="s">
-        <v>11</v>
-      </c>
-      <c r="F94" t="s">
-        <v>99</v>
-      </c>
-      <c r="G94" t="s">
-        <v>38</v>
+      <c r="H94" t="s">
+        <v>167</v>
       </c>
       <c r="J94" s="3" t="s">
-        <v>211</v>
+        <v>165</v>
       </c>
     </row>
     <row r="95" spans="1:10" x14ac:dyDescent="0.3">
@@ -3793,28 +3790,28 @@
         <v>18</v>
       </c>
       <c r="B95" t="s">
-        <v>216</v>
+        <v>168</v>
       </c>
       <c r="C95" t="s">
+        <v>34</v>
+      </c>
+      <c r="D95" t="s">
+        <v>35</v>
+      </c>
+      <c r="E95" t="s">
+        <v>11</v>
+      </c>
+      <c r="F95" t="s">
+        <v>81</v>
+      </c>
+      <c r="G95" t="s">
         <v>36</v>
       </c>
-      <c r="D95" t="s">
-        <v>37</v>
-      </c>
-      <c r="E95" t="s">
-        <v>11</v>
-      </c>
-      <c r="F95" t="s">
-        <v>99</v>
-      </c>
-      <c r="G95" t="s">
-        <v>38</v>
-      </c>
       <c r="H95" t="s">
-        <v>213</v>
+        <v>167</v>
       </c>
       <c r="J95" s="3" t="s">
-        <v>211</v>
+        <v>165</v>
       </c>
     </row>
     <row r="96" spans="1:10" x14ac:dyDescent="0.3">
@@ -3822,25 +3819,25 @@
         <v>18</v>
       </c>
       <c r="B96" t="s">
-        <v>18</v>
+        <v>169</v>
       </c>
       <c r="C96" t="s">
+        <v>34</v>
+      </c>
+      <c r="D96" t="s">
+        <v>35</v>
+      </c>
+      <c r="E96" t="s">
+        <v>11</v>
+      </c>
+      <c r="F96" t="s">
+        <v>81</v>
+      </c>
+      <c r="G96" t="s">
         <v>36</v>
       </c>
-      <c r="D96" t="s">
-        <v>37</v>
-      </c>
-      <c r="E96" t="s">
-        <v>11</v>
-      </c>
-      <c r="F96" t="s">
-        <v>14</v>
-      </c>
-      <c r="G96" t="s">
-        <v>63</v>
-      </c>
       <c r="J96" s="3" t="s">
-        <v>60</v>
+        <v>165</v>
       </c>
     </row>
     <row r="97" spans="1:10" x14ac:dyDescent="0.3">
@@ -3848,581 +3845,688 @@
         <v>18</v>
       </c>
       <c r="B97" t="s">
-        <v>18</v>
+        <v>170</v>
       </c>
       <c r="C97" t="s">
+        <v>34</v>
+      </c>
+      <c r="D97" t="s">
+        <v>35</v>
+      </c>
+      <c r="E97" t="s">
+        <v>11</v>
+      </c>
+      <c r="F97" t="s">
+        <v>81</v>
+      </c>
+      <c r="G97" t="s">
         <v>36</v>
       </c>
-      <c r="D97" t="s">
-        <v>37</v>
-      </c>
-      <c r="E97" t="s">
-        <v>11</v>
-      </c>
-      <c r="F97" t="s">
-        <v>61</v>
-      </c>
-      <c r="G97" t="s">
-        <v>63</v>
+      <c r="H97" t="s">
+        <v>167</v>
       </c>
       <c r="J97" s="3" t="s">
-        <v>60</v>
+        <v>165</v>
       </c>
     </row>
     <row r="98" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A98" t="s">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="B98" t="s">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="C98" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="D98" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="E98" t="s">
         <v>11</v>
       </c>
       <c r="F98" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="G98" t="s">
-        <v>63</v>
+        <v>56</v>
       </c>
       <c r="J98" s="3" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
     </row>
     <row r="99" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A99" t="s">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="B99" t="s">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="C99" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="D99" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="E99" t="s">
         <v>11</v>
       </c>
       <c r="F99" t="s">
-        <v>46</v>
+        <v>54</v>
       </c>
       <c r="G99" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="J99" s="3" t="s">
-        <v>74</v>
+        <v>53</v>
       </c>
     </row>
     <row r="100" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A100" t="s">
-        <v>75</v>
+        <v>26</v>
       </c>
       <c r="B100" t="s">
-        <v>98</v>
+        <v>26</v>
       </c>
       <c r="C100" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="D100" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="E100" t="s">
         <v>11</v>
       </c>
       <c r="F100" t="s">
-        <v>99</v>
+        <v>19</v>
       </c>
       <c r="G100" t="s">
-        <v>38</v>
+        <v>56</v>
       </c>
       <c r="J100" s="3" t="s">
-        <v>62</v>
+        <v>218</v>
       </c>
     </row>
     <row r="101" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A101" t="s">
-        <v>75</v>
+        <v>26</v>
       </c>
       <c r="B101" t="s">
-        <v>76</v>
+        <v>26</v>
       </c>
       <c r="C101" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="D101" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="E101" t="s">
         <v>11</v>
       </c>
       <c r="F101" t="s">
-        <v>21</v>
+        <v>41</v>
       </c>
       <c r="G101" t="s">
-        <v>38</v>
+        <v>51</v>
       </c>
       <c r="J101" s="3" t="s">
-        <v>62</v>
+        <v>218</v>
       </c>
     </row>
     <row r="102" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A102" t="s">
-        <v>75</v>
+        <v>64</v>
       </c>
       <c r="B102" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="C102" t="s">
+        <v>34</v>
+      </c>
+      <c r="D102" t="s">
+        <v>35</v>
+      </c>
+      <c r="E102" t="s">
+        <v>11</v>
+      </c>
+      <c r="F102" t="s">
+        <v>81</v>
+      </c>
+      <c r="G102" t="s">
         <v>36</v>
       </c>
-      <c r="D102" t="s">
-        <v>37</v>
-      </c>
-      <c r="E102" t="s">
-        <v>11</v>
-      </c>
-      <c r="F102" t="s">
-        <v>21</v>
-      </c>
-      <c r="G102" t="s">
-        <v>38</v>
-      </c>
       <c r="J102" s="3" t="s">
-        <v>62</v>
+        <v>55</v>
       </c>
     </row>
     <row r="103" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A103" t="s">
-        <v>75</v>
+        <v>64</v>
       </c>
       <c r="B103" t="s">
-        <v>75</v>
+        <v>65</v>
       </c>
       <c r="C103" t="s">
+        <v>34</v>
+      </c>
+      <c r="D103" t="s">
+        <v>35</v>
+      </c>
+      <c r="E103" t="s">
+        <v>11</v>
+      </c>
+      <c r="F103" t="s">
+        <v>21</v>
+      </c>
+      <c r="G103" t="s">
         <v>36</v>
       </c>
-      <c r="D103" t="s">
-        <v>37</v>
-      </c>
-      <c r="E103" t="s">
-        <v>11</v>
-      </c>
-      <c r="F103" t="s">
-        <v>61</v>
-      </c>
-      <c r="G103" t="s">
-        <v>38</v>
-      </c>
       <c r="J103" s="3" t="s">
-        <v>62</v>
+        <v>55</v>
       </c>
     </row>
     <row r="104" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A104" t="s">
-        <v>32</v>
+        <v>64</v>
       </c>
       <c r="B104" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="C104" t="s">
+        <v>34</v>
+      </c>
+      <c r="D104" t="s">
+        <v>35</v>
+      </c>
+      <c r="E104" t="s">
+        <v>11</v>
+      </c>
+      <c r="F104" t="s">
+        <v>21</v>
+      </c>
+      <c r="G104" t="s">
         <v>36</v>
       </c>
-      <c r="D104" t="s">
-        <v>37</v>
-      </c>
-      <c r="E104" t="s">
-        <v>11</v>
-      </c>
-      <c r="F104" t="s">
-        <v>19</v>
-      </c>
-      <c r="G104" t="s">
-        <v>38</v>
-      </c>
       <c r="J104" s="3" t="s">
-        <v>78</v>
+        <v>55</v>
       </c>
     </row>
     <row r="105" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A105" t="s">
-        <v>32</v>
+        <v>64</v>
       </c>
       <c r="B105" t="s">
-        <v>32</v>
+        <v>64</v>
       </c>
       <c r="C105" t="s">
+        <v>34</v>
+      </c>
+      <c r="D105" t="s">
+        <v>35</v>
+      </c>
+      <c r="E105" t="s">
+        <v>11</v>
+      </c>
+      <c r="F105" t="s">
+        <v>54</v>
+      </c>
+      <c r="G105" t="s">
         <v>36</v>
       </c>
-      <c r="D105" t="s">
-        <v>37</v>
-      </c>
-      <c r="E105" t="s">
-        <v>11</v>
-      </c>
-      <c r="F105" t="s">
+      <c r="J105" s="3" t="s">
         <v>55</v>
-      </c>
-      <c r="G105" t="s">
-        <v>58</v>
-      </c>
-      <c r="I105" s="3">
-        <v>14</v>
-      </c>
-      <c r="J105" s="3" t="s">
-        <v>50</v>
       </c>
     </row>
     <row r="106" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A106" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B106" t="s">
-        <v>32</v>
+        <v>57</v>
       </c>
       <c r="C106" t="s">
+        <v>34</v>
+      </c>
+      <c r="D106" t="s">
+        <v>35</v>
+      </c>
+      <c r="E106" t="s">
+        <v>11</v>
+      </c>
+      <c r="F106" t="s">
+        <v>19</v>
+      </c>
+      <c r="G106" t="s">
         <v>36</v>
       </c>
-      <c r="D106" t="s">
-        <v>37</v>
-      </c>
-      <c r="E106" t="s">
-        <v>11</v>
-      </c>
-      <c r="F106" t="s">
-        <v>56</v>
-      </c>
-      <c r="G106" t="s">
-        <v>58</v>
-      </c>
-      <c r="I106" s="3">
-        <v>14</v>
-      </c>
       <c r="J106" s="3" t="s">
-        <v>50</v>
+        <v>67</v>
       </c>
     </row>
     <row r="107" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A107" t="s">
-        <v>79</v>
+        <v>31</v>
       </c>
       <c r="B107" t="s">
-        <v>79</v>
+        <v>31</v>
       </c>
       <c r="C107" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="D107" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="E107" t="s">
         <v>11</v>
       </c>
       <c r="F107" t="s">
-        <v>24</v>
+        <v>48</v>
       </c>
       <c r="G107" t="s">
-        <v>38</v>
+        <v>51</v>
+      </c>
+      <c r="I107" s="3">
+        <v>14</v>
       </c>
       <c r="J107" s="3" t="s">
-        <v>80</v>
+        <v>209</v>
       </c>
     </row>
     <row r="108" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A108" t="s">
-        <v>81</v>
+        <v>31</v>
       </c>
       <c r="B108" t="s">
-        <v>82</v>
+        <v>31</v>
       </c>
       <c r="C108" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="D108" t="s">
-        <v>54</v>
+        <v>35</v>
       </c>
       <c r="E108" t="s">
         <v>11</v>
       </c>
       <c r="F108" t="s">
-        <v>61</v>
+        <v>49</v>
       </c>
       <c r="G108" t="s">
-        <v>83</v>
+        <v>51</v>
+      </c>
+      <c r="I108" s="3">
+        <v>14</v>
       </c>
       <c r="J108" s="3" t="s">
-        <v>50</v>
+        <v>209</v>
       </c>
     </row>
     <row r="109" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A109" t="s">
-        <v>81</v>
+        <v>68</v>
       </c>
       <c r="B109" t="s">
-        <v>82</v>
+        <v>68</v>
       </c>
       <c r="C109" t="s">
+        <v>34</v>
+      </c>
+      <c r="D109" t="s">
+        <v>35</v>
+      </c>
+      <c r="E109" t="s">
+        <v>11</v>
+      </c>
+      <c r="F109" t="s">
+        <v>24</v>
+      </c>
+      <c r="G109" t="s">
         <v>36</v>
       </c>
-      <c r="D109" t="s">
-        <v>54</v>
-      </c>
-      <c r="E109" t="s">
-        <v>11</v>
-      </c>
-      <c r="F109" t="s">
-        <v>61</v>
-      </c>
-      <c r="G109" t="s">
-        <v>58</v>
-      </c>
       <c r="J109" s="3" t="s">
-        <v>50</v>
+        <v>219</v>
       </c>
     </row>
     <row r="110" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A110" t="s">
-        <v>81</v>
+        <v>69</v>
       </c>
       <c r="B110" t="s">
-        <v>81</v>
+        <v>70</v>
       </c>
       <c r="C110" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="D110" t="s">
+        <v>47</v>
+      </c>
+      <c r="E110" t="s">
+        <v>11</v>
+      </c>
+      <c r="F110" t="s">
         <v>54</v>
       </c>
-      <c r="E110" t="s">
-        <v>11</v>
-      </c>
-      <c r="F110" t="s">
-        <v>61</v>
-      </c>
       <c r="G110" t="s">
-        <v>58</v>
+        <v>71</v>
       </c>
       <c r="J110" s="3" t="s">
-        <v>96</v>
+        <v>209</v>
       </c>
     </row>
     <row r="111" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A111" t="s">
-        <v>84</v>
+        <v>69</v>
       </c>
       <c r="B111" t="s">
-        <v>85</v>
+        <v>70</v>
       </c>
       <c r="C111" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="D111" t="s">
+        <v>47</v>
+      </c>
+      <c r="E111" t="s">
+        <v>11</v>
+      </c>
+      <c r="F111" t="s">
         <v>54</v>
       </c>
-      <c r="E111" t="s">
-        <v>11</v>
-      </c>
-      <c r="F111" t="s">
-        <v>97</v>
-      </c>
       <c r="G111" t="s">
-        <v>86</v>
+        <v>51</v>
       </c>
       <c r="J111" s="3" t="s">
-        <v>94</v>
+        <v>44</v>
       </c>
     </row>
     <row r="112" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A112" t="s">
-        <v>84</v>
+        <v>69</v>
       </c>
       <c r="B112" t="s">
-        <v>84</v>
+        <v>69</v>
       </c>
       <c r="C112" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="D112" t="s">
+        <v>47</v>
+      </c>
+      <c r="E112" t="s">
+        <v>11</v>
+      </c>
+      <c r="F112" t="s">
         <v>54</v>
       </c>
-      <c r="E112" t="s">
-        <v>11</v>
-      </c>
-      <c r="F112" t="s">
-        <v>97</v>
-      </c>
       <c r="G112" t="s">
-        <v>86</v>
+        <v>51</v>
       </c>
       <c r="J112" s="3" t="s">
-        <v>87</v>
+        <v>220</v>
       </c>
     </row>
     <row r="113" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A113" t="s">
-        <v>88</v>
+        <v>72</v>
       </c>
       <c r="B113" t="s">
-        <v>88</v>
+        <v>73</v>
       </c>
       <c r="C113" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="D113" t="s">
-        <v>54</v>
+        <v>47</v>
       </c>
       <c r="E113" t="s">
         <v>11</v>
       </c>
       <c r="F113" t="s">
-        <v>14</v>
+        <v>79</v>
       </c>
       <c r="G113" t="s">
-        <v>58</v>
+        <v>74</v>
       </c>
       <c r="J113" s="3" t="s">
-        <v>89</v>
+        <v>221</v>
       </c>
     </row>
     <row r="114" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A114" t="s">
-        <v>88</v>
+        <v>72</v>
       </c>
       <c r="B114" t="s">
-        <v>88</v>
+        <v>72</v>
       </c>
       <c r="C114" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="D114" t="s">
-        <v>54</v>
+        <v>47</v>
       </c>
       <c r="E114" t="s">
         <v>11</v>
       </c>
       <c r="F114" t="s">
-        <v>56</v>
+        <v>79</v>
       </c>
       <c r="G114" t="s">
-        <v>58</v>
+        <v>74</v>
       </c>
       <c r="J114" s="3" t="s">
-        <v>90</v>
+        <v>222</v>
       </c>
     </row>
     <row r="115" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A115" t="s">
-        <v>91</v>
+        <v>75</v>
       </c>
       <c r="B115" t="s">
-        <v>92</v>
+        <v>75</v>
       </c>
       <c r="C115" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="D115" t="s">
-        <v>37</v>
+        <v>47</v>
       </c>
       <c r="E115" t="s">
         <v>11</v>
       </c>
       <c r="F115" t="s">
-        <v>55</v>
+        <v>14</v>
       </c>
       <c r="G115" t="s">
-        <v>58</v>
+        <v>51</v>
       </c>
       <c r="J115" s="3" t="s">
-        <v>50</v>
+        <v>223</v>
       </c>
     </row>
     <row r="116" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A116" t="s">
-        <v>91</v>
+        <v>75</v>
       </c>
       <c r="B116" t="s">
-        <v>92</v>
+        <v>75</v>
       </c>
       <c r="C116" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="D116" t="s">
-        <v>37</v>
+        <v>47</v>
       </c>
       <c r="E116" t="s">
         <v>11</v>
       </c>
       <c r="F116" t="s">
-        <v>56</v>
+        <v>49</v>
       </c>
       <c r="G116" t="s">
-        <v>58</v>
+        <v>51</v>
       </c>
       <c r="J116" s="3" t="s">
-        <v>50</v>
+        <v>224</v>
       </c>
     </row>
     <row r="117" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A117" t="s">
-        <v>91</v>
+        <v>76</v>
       </c>
       <c r="B117" t="s">
-        <v>91</v>
+        <v>77</v>
       </c>
       <c r="C117" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="D117" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="E117" t="s">
         <v>11</v>
       </c>
       <c r="F117" t="s">
-        <v>15</v>
+        <v>48</v>
       </c>
       <c r="G117" t="s">
-        <v>58</v>
+        <v>51</v>
       </c>
       <c r="J117" s="3" t="s">
-        <v>93</v>
+        <v>209</v>
       </c>
     </row>
     <row r="118" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A118" t="s">
-        <v>91</v>
+        <v>76</v>
       </c>
       <c r="B118" t="s">
-        <v>91</v>
+        <v>77</v>
       </c>
       <c r="C118" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="D118" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="E118" t="s">
         <v>11</v>
       </c>
       <c r="F118" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="G118" t="s">
-        <v>58</v>
+        <v>51</v>
       </c>
       <c r="J118" s="3" t="s">
-        <v>50</v>
+        <v>209</v>
+      </c>
+    </row>
+    <row r="119" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A119" t="s">
+        <v>76</v>
+      </c>
+      <c r="B119" t="s">
+        <v>76</v>
+      </c>
+      <c r="C119" t="s">
+        <v>34</v>
+      </c>
+      <c r="D119" t="s">
+        <v>35</v>
+      </c>
+      <c r="E119" t="s">
+        <v>11</v>
+      </c>
+      <c r="F119" t="s">
+        <v>15</v>
+      </c>
+      <c r="G119" t="s">
+        <v>51</v>
+      </c>
+      <c r="J119" s="3" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="120" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A120" t="s">
+        <v>76</v>
+      </c>
+      <c r="B120" t="s">
+        <v>76</v>
+      </c>
+      <c r="C120" t="s">
+        <v>34</v>
+      </c>
+      <c r="D120" t="s">
+        <v>35</v>
+      </c>
+      <c r="E120" t="s">
+        <v>11</v>
+      </c>
+      <c r="F120" t="s">
+        <v>41</v>
+      </c>
+      <c r="G120" t="s">
+        <v>51</v>
+      </c>
+      <c r="J120" s="3" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="121" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A121" t="s">
+        <v>69</v>
+      </c>
+      <c r="B121" t="s">
+        <v>206</v>
+      </c>
+      <c r="C121" t="s">
+        <v>226</v>
+      </c>
+      <c r="D121" t="s">
+        <v>10</v>
+      </c>
+      <c r="E121" t="s">
+        <v>11</v>
+      </c>
+      <c r="F121" t="s">
+        <v>19</v>
+      </c>
+      <c r="G121" t="s">
+        <v>12</v>
+      </c>
+      <c r="I121" s="3">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="122" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A122" t="s">
+        <v>32</v>
+      </c>
+      <c r="B122" t="s">
+        <v>206</v>
+      </c>
+      <c r="C122" t="s">
+        <v>226</v>
+      </c>
+      <c r="D122" t="s">
+        <v>10</v>
+      </c>
+      <c r="E122" t="s">
+        <v>11</v>
+      </c>
+      <c r="F122" t="s">
+        <v>19</v>
+      </c>
+      <c r="G122" t="s">
+        <v>12</v>
+      </c>
+      <c r="I122" s="3">
+        <v>48</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J118" xr:uid="{EAF16D4A-DA29-4FF0-AC3B-589258931E62}"/>
+  <autoFilter ref="A1:J122" xr:uid="{EAF16D4A-DA29-4FF0-AC3B-589258931E62}"/>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
atualizacao diaria fretes e aniversarios
</commit_message>
<xml_diff>
--- a/scripts/cargas.xlsx
+++ b/scripts/cargas.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projetos\tr.alienigenaV5-main\scripts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A6D289F3-ED23-4377-A366-8066841AFA23}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{883037DA-9842-47F7-AF2D-CC8EC2E7B76E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" tabRatio="551" xr2:uid="{9E8F4E85-D2FF-4383-A72B-5CAFDCCC5644}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Planilha1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Planilha1!$A$1:$J$122</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Planilha1!$A$1:$J$115</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1033" uniqueCount="227">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="977" uniqueCount="218">
   <si>
     <t>Origem</t>
   </si>
@@ -143,9 +143,6 @@
     <t>Laranjeiras - SE</t>
   </si>
   <si>
-    <t>São Gonçalo - RJ</t>
-  </si>
-  <si>
     <t>CIMENTO</t>
   </si>
   <si>
@@ -155,12 +152,6 @@
     <t>Grade Baixa</t>
   </si>
   <si>
-    <t>Rio de Janeiro - RJ</t>
-  </si>
-  <si>
-    <t>CIMENTO ENSACADO</t>
-  </si>
-  <si>
     <t>Campinas - SP</t>
   </si>
   <si>
@@ -653,21 +644,9 @@
     <t>180,00</t>
   </si>
   <si>
-    <t>Nova Ponte - MG</t>
-  </si>
-  <si>
-    <t>Ponte Nova - MG</t>
-  </si>
-  <si>
     <t>Brasilândia de Minas - MG</t>
   </si>
   <si>
-    <t>Penápolis - SP</t>
-  </si>
-  <si>
-    <t>Ureia granel</t>
-  </si>
-  <si>
     <t>PARA CARREGAMENTO, NECESSÁRIO CHAPA (AJUDANTE) E TER PALLETS, CINTA, LONA E EPI - DESTINOS DISPONIVEIS: CASTELO DO PIAUI/PI, SÃO MIGUEL DO TAPUI/PI, PARNAIBA/PI, BARRAS/PI, CAJUEIRO DA PRAIA/PI, SÃO JOÃO DA FRONTEIRA/PI, ILHA GRANDE/PI, COCAL/PI, LAGOA ALEGRE/PI, MIGUEL ALVES/PI, ALTOS/PI, SÃO JOÃO DA SERRA/PI, CAMPO MAIOR/PI, BENEDITINOS/PI, LUZILANDIA/PI, MADEIRO/PI, MATIAS OLIMPIO/PI, TUTOIA/MA.</t>
   </si>
   <si>
@@ -683,15 +662,6 @@
     <t>PARA CARREGAMENTO, NECESSÁRIO CHAPA (AJUDANTE) E TER PALLETS, CINTA, LONA E EPI - POSSIVEIS DESTINOS DISPONIVEIS: Guarulhos/SP, São Paulo/SP (Zona Leste), Região do Alto Tietê/SP</t>
   </si>
   <si>
-    <t>PARA CARREGAMENTO, NECESSÁRIO CHAPA (AJUDANTE) E TER PALLETS, CINTA, LONA E EPI. Possíveis destinos disponíveis:Região dos Lagos (Araruama/RJ com Saquarema/RJ na mesma rota e Cabo Frio/RJ com Arraial do Cabo/RJ na mesma rota)</t>
-  </si>
-  <si>
-    <t>PARA CARREGAMENTO, NECESSÁRIO CHAPA (AJUDANTE) E TER PALLETS, CINTA, LONA E EPI. Possíveis destinos disponíveis CD Santa Cruz: Rio de Janeiro-RJ, Itaguaí -RJ, Seropédica-RJ, Itatiaia-RJ.</t>
-  </si>
-  <si>
-    <t>PARA CARREGAMENTO, NECESSÁRIO CHAPA (AJUDANTE) E TER PALLETS, CINTA, LONA E EPI. Possíveis destinos disponíveis CD RIO: Rio de Janeiro-RJ, Nova Iguaçu-RJ, Duque de Caxias-RJ, Mesquita-RJ )</t>
-  </si>
-  <si>
     <t>PARA MOTORISTAS CATIVOS NA REGIÃO - PARA CARREGAMENTO, NECESSÁRIO CHAPA (AJUDANTE) E TER PALLETS, CINTA, LONA E EPI</t>
   </si>
   <si>
@@ -722,7 +692,10 @@
     <t>PARA CARREGAMENTO, NECESSÁRIO CHAPA (AJUDANTE) E TER PALLETS, CINTA, LONA E EPI - POSSIVEIS DESTINOS DISPONIVEIS: Região de Gargalo, Vitória da Conquista e Ipiau</t>
   </si>
   <si>
-    <t>Ureia Granel</t>
+    <t>Diversos</t>
+  </si>
+  <si>
+    <t>Truck, Carreta, Carreta 4º eixo</t>
   </si>
 </sst>
 </file>
@@ -1122,19 +1095,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EAF16D4A-DA29-4FF0-AC3B-589258931E62}">
-  <dimension ref="A1:J122"/>
+  <dimension ref="A1:J115"/>
   <sheetFormatPr defaultColWidth="12.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="25.5546875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="25.6640625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="18.44140625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="9.6640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="16.88671875" customWidth="1"/>
+    <col min="5" max="5" width="19.77734375" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="44.88671875" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="27.77734375" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="8.88671875" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="11.44140625" style="3" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="255.6640625" style="3" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="112" style="3" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.3">
@@ -1171,39 +1144,42 @@
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>184</v>
+        <v>115</v>
       </c>
       <c r="B2" t="s">
-        <v>184</v>
+        <v>170</v>
       </c>
       <c r="C2" t="s">
-        <v>185</v>
+        <v>82</v>
       </c>
       <c r="D2" t="s">
-        <v>186</v>
+        <v>10</v>
       </c>
       <c r="E2" t="s">
         <v>11</v>
       </c>
       <c r="F2" t="s">
-        <v>187</v>
+        <v>19</v>
       </c>
       <c r="G2" t="s">
-        <v>188</v>
-      </c>
-      <c r="I2" s="3">
-        <v>14</v>
+        <v>13</v>
+      </c>
+      <c r="H2" t="s">
+        <v>171</v>
+      </c>
+      <c r="J2" s="3" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="B3" t="s">
-        <v>173</v>
+        <v>157</v>
       </c>
       <c r="C3" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="D3" t="s">
         <v>10</v>
@@ -1218,7 +1194,7 @@
         <v>13</v>
       </c>
       <c r="H3" t="s">
-        <v>174</v>
+        <v>158</v>
       </c>
       <c r="J3" s="3" t="s">
         <v>20</v>
@@ -1226,13 +1202,13 @@
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>118</v>
+        <v>144</v>
       </c>
       <c r="B4" t="s">
-        <v>160</v>
+        <v>155</v>
       </c>
       <c r="C4" t="s">
-        <v>85</v>
+        <v>116</v>
       </c>
       <c r="D4" t="s">
         <v>10</v>
@@ -1241,85 +1217,85 @@
         <v>11</v>
       </c>
       <c r="F4" t="s">
-        <v>19</v>
+        <v>186</v>
       </c>
       <c r="G4" t="s">
         <v>13</v>
       </c>
       <c r="H4" t="s">
-        <v>161</v>
+        <v>187</v>
       </c>
       <c r="J4" s="3" t="s">
-        <v>20</v>
+        <v>89</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>147</v>
+        <v>80</v>
       </c>
       <c r="B5" t="s">
-        <v>158</v>
+        <v>188</v>
       </c>
       <c r="C5" t="s">
-        <v>119</v>
+        <v>82</v>
       </c>
       <c r="D5" t="s">
-        <v>10</v>
+        <v>189</v>
       </c>
       <c r="E5" t="s">
         <v>11</v>
       </c>
       <c r="F5" t="s">
-        <v>189</v>
+        <v>21</v>
       </c>
       <c r="G5" t="s">
-        <v>13</v>
+        <v>190</v>
       </c>
       <c r="H5" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="J5" s="3" t="s">
-        <v>92</v>
+        <v>20</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>83</v>
+        <v>144</v>
       </c>
       <c r="B6" t="s">
-        <v>191</v>
+        <v>155</v>
       </c>
       <c r="C6" t="s">
-        <v>85</v>
+        <v>116</v>
       </c>
       <c r="D6" t="s">
-        <v>192</v>
+        <v>10</v>
       </c>
       <c r="E6" t="s">
         <v>11</v>
       </c>
       <c r="F6" t="s">
-        <v>21</v>
+        <v>172</v>
       </c>
       <c r="G6" t="s">
-        <v>193</v>
+        <v>13</v>
       </c>
       <c r="H6" t="s">
-        <v>194</v>
+        <v>187</v>
       </c>
       <c r="J6" s="3" t="s">
-        <v>20</v>
+        <v>89</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="B7" t="s">
-        <v>158</v>
+        <v>150</v>
       </c>
       <c r="C7" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="D7" t="s">
         <v>10</v>
@@ -1328,27 +1304,27 @@
         <v>11</v>
       </c>
       <c r="F7" t="s">
-        <v>175</v>
+        <v>151</v>
       </c>
       <c r="G7" t="s">
         <v>13</v>
       </c>
       <c r="H7" t="s">
-        <v>190</v>
+        <v>152</v>
       </c>
       <c r="J7" s="3" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="B8" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="C8" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="D8" t="s">
         <v>10</v>
@@ -1357,27 +1333,27 @@
         <v>11</v>
       </c>
       <c r="F8" t="s">
-        <v>154</v>
+        <v>78</v>
       </c>
       <c r="G8" t="s">
         <v>13</v>
       </c>
       <c r="H8" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="J8" s="3" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="B9" t="s">
         <v>153</v>
       </c>
       <c r="C9" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="D9" t="s">
         <v>10</v>
@@ -1386,27 +1362,27 @@
         <v>11</v>
       </c>
       <c r="F9" t="s">
-        <v>81</v>
+        <v>172</v>
       </c>
       <c r="G9" t="s">
         <v>13</v>
       </c>
       <c r="H9" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="J9" s="3" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>147</v>
+        <v>80</v>
       </c>
       <c r="B10" t="s">
-        <v>156</v>
+        <v>173</v>
       </c>
       <c r="C10" t="s">
-        <v>119</v>
+        <v>82</v>
       </c>
       <c r="D10" t="s">
         <v>10</v>
@@ -1415,27 +1391,27 @@
         <v>11</v>
       </c>
       <c r="F10" t="s">
-        <v>175</v>
+        <v>14</v>
       </c>
       <c r="G10" t="s">
         <v>13</v>
       </c>
       <c r="H10" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="J10" s="3" t="s">
-        <v>92</v>
+        <v>20</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="B11" t="s">
-        <v>176</v>
+        <v>146</v>
       </c>
       <c r="C11" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="D11" t="s">
         <v>10</v>
@@ -1450,7 +1426,7 @@
         <v>13</v>
       </c>
       <c r="H11" t="s">
-        <v>157</v>
+        <v>138</v>
       </c>
       <c r="J11" s="3" t="s">
         <v>20</v>
@@ -1458,13 +1434,13 @@
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="B12" t="s">
-        <v>149</v>
+        <v>81</v>
       </c>
       <c r="C12" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="D12" t="s">
         <v>10</v>
@@ -1479,7 +1455,7 @@
         <v>13</v>
       </c>
       <c r="H12" t="s">
-        <v>141</v>
+        <v>83</v>
       </c>
       <c r="J12" s="3" t="s">
         <v>20</v>
@@ -1487,28 +1463,28 @@
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>83</v>
+        <v>32</v>
       </c>
       <c r="B13" t="s">
+        <v>25</v>
+      </c>
+      <c r="C13" t="s">
+        <v>23</v>
+      </c>
+      <c r="D13" t="s">
+        <v>10</v>
+      </c>
+      <c r="E13" t="s">
+        <v>11</v>
+      </c>
+      <c r="F13" t="s">
+        <v>45</v>
+      </c>
+      <c r="G13" t="s">
+        <v>13</v>
+      </c>
+      <c r="H13" t="s">
         <v>84</v>
-      </c>
-      <c r="C13" t="s">
-        <v>85</v>
-      </c>
-      <c r="D13" t="s">
-        <v>10</v>
-      </c>
-      <c r="E13" t="s">
-        <v>11</v>
-      </c>
-      <c r="F13" t="s">
-        <v>14</v>
-      </c>
-      <c r="G13" t="s">
-        <v>13</v>
-      </c>
-      <c r="H13" t="s">
-        <v>86</v>
       </c>
       <c r="J13" s="3" t="s">
         <v>20</v>
@@ -1516,71 +1492,59 @@
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>32</v>
+        <v>181</v>
       </c>
       <c r="B14" t="s">
-        <v>25</v>
+        <v>181</v>
       </c>
       <c r="C14" t="s">
-        <v>23</v>
+        <v>182</v>
       </c>
       <c r="D14" t="s">
-        <v>10</v>
+        <v>216</v>
       </c>
       <c r="E14" t="s">
         <v>11</v>
       </c>
       <c r="F14" t="s">
-        <v>48</v>
+        <v>151</v>
       </c>
       <c r="G14" t="s">
-        <v>13</v>
-      </c>
-      <c r="H14" t="s">
-        <v>87</v>
-      </c>
-      <c r="J14" s="3" t="s">
-        <v>20</v>
+        <v>185</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>88</v>
+        <v>181</v>
       </c>
       <c r="B15" t="s">
-        <v>89</v>
+        <v>181</v>
       </c>
       <c r="C15" t="s">
-        <v>90</v>
+        <v>182</v>
       </c>
       <c r="D15" t="s">
-        <v>10</v>
+        <v>216</v>
       </c>
       <c r="E15" t="s">
         <v>11</v>
       </c>
       <c r="F15" t="s">
-        <v>19</v>
+        <v>217</v>
       </c>
       <c r="G15" t="s">
-        <v>13</v>
-      </c>
-      <c r="H15" t="s">
-        <v>91</v>
-      </c>
-      <c r="J15" s="3" t="s">
-        <v>92</v>
+        <v>185</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>93</v>
+        <v>85</v>
       </c>
       <c r="B16" t="s">
-        <v>94</v>
+        <v>86</v>
       </c>
       <c r="C16" t="s">
-        <v>95</v>
+        <v>87</v>
       </c>
       <c r="D16" t="s">
         <v>10</v>
@@ -1595,50 +1559,50 @@
         <v>13</v>
       </c>
       <c r="H16" t="s">
-        <v>96</v>
+        <v>88</v>
       </c>
       <c r="J16" s="3" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="B17" t="s">
+        <v>91</v>
+      </c>
+      <c r="C17" t="s">
+        <v>92</v>
+      </c>
+      <c r="D17" t="s">
+        <v>10</v>
+      </c>
+      <c r="E17" t="s">
+        <v>11</v>
+      </c>
+      <c r="F17" t="s">
+        <v>19</v>
+      </c>
+      <c r="G17" t="s">
+        <v>13</v>
+      </c>
+      <c r="H17" t="s">
+        <v>93</v>
+      </c>
+      <c r="J17" s="3" t="s">
         <v>89</v>
-      </c>
-      <c r="C17" t="s">
-        <v>90</v>
-      </c>
-      <c r="D17" t="s">
-        <v>10</v>
-      </c>
-      <c r="E17" t="s">
-        <v>11</v>
-      </c>
-      <c r="F17" t="s">
-        <v>21</v>
-      </c>
-      <c r="G17" t="s">
-        <v>13</v>
-      </c>
-      <c r="H17" t="s">
-        <v>97</v>
-      </c>
-      <c r="J17" s="3" t="s">
-        <v>92</v>
       </c>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>98</v>
+        <v>85</v>
       </c>
       <c r="B18" t="s">
-        <v>99</v>
+        <v>86</v>
       </c>
       <c r="C18" t="s">
-        <v>22</v>
+        <v>87</v>
       </c>
       <c r="D18" t="s">
         <v>10</v>
@@ -1647,27 +1611,24 @@
         <v>11</v>
       </c>
       <c r="F18" t="s">
-        <v>195</v>
+        <v>21</v>
       </c>
       <c r="G18" t="s">
         <v>13</v>
       </c>
       <c r="H18" t="s">
-        <v>129</v>
-      </c>
-      <c r="I18" s="3">
-        <v>28000</v>
+        <v>94</v>
       </c>
       <c r="J18" s="3" t="s">
-        <v>100</v>
+        <v>89</v>
       </c>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="B19" t="s">
-        <v>82</v>
+        <v>96</v>
       </c>
       <c r="C19" t="s">
         <v>22</v>
@@ -1679,27 +1640,27 @@
         <v>11</v>
       </c>
       <c r="F19" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="G19" t="s">
         <v>13</v>
       </c>
       <c r="H19" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="I19" s="3">
         <v>28000</v>
       </c>
       <c r="J19" s="3" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="B20" t="s">
-        <v>99</v>
+        <v>79</v>
       </c>
       <c r="C20" t="s">
         <v>22</v>
@@ -1711,27 +1672,27 @@
         <v>11</v>
       </c>
       <c r="F20" t="s">
-        <v>19</v>
+        <v>192</v>
       </c>
       <c r="G20" t="s">
         <v>13</v>
       </c>
       <c r="H20" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="I20" s="3">
         <v>28000</v>
       </c>
       <c r="J20" s="3" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="B21" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="C21" t="s">
         <v>22</v>
@@ -1743,27 +1704,27 @@
         <v>11</v>
       </c>
       <c r="F21" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="G21" t="s">
         <v>13</v>
       </c>
       <c r="H21" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="I21" s="3">
         <v>28000</v>
       </c>
       <c r="J21" s="3" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="B22" t="s">
-        <v>82</v>
+        <v>96</v>
       </c>
       <c r="C22" t="s">
         <v>22</v>
@@ -1775,27 +1736,27 @@
         <v>11</v>
       </c>
       <c r="F22" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="G22" t="s">
         <v>13</v>
       </c>
       <c r="H22" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="I22" s="3">
         <v>28000</v>
       </c>
       <c r="J22" s="3" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="B23" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="C23" t="s">
         <v>22</v>
@@ -1807,30 +1768,30 @@
         <v>11</v>
       </c>
       <c r="F23" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="G23" t="s">
         <v>13</v>
       </c>
       <c r="H23" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="I23" s="3">
         <v>28000</v>
       </c>
       <c r="J23" s="3" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>153</v>
+        <v>95</v>
       </c>
       <c r="B24" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="C24" t="s">
-        <v>113</v>
+        <v>22</v>
       </c>
       <c r="D24" t="s">
         <v>10</v>
@@ -1839,27 +1800,30 @@
         <v>11</v>
       </c>
       <c r="F24" t="s">
-        <v>27</v>
+        <v>21</v>
       </c>
       <c r="G24" t="s">
         <v>13</v>
       </c>
       <c r="H24" t="s">
-        <v>87</v>
+        <v>126</v>
+      </c>
+      <c r="I24" s="3">
+        <v>28000</v>
       </c>
       <c r="J24" s="3" t="s">
-        <v>20</v>
+        <v>97</v>
       </c>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>101</v>
+        <v>150</v>
       </c>
       <c r="B25" t="s">
-        <v>32</v>
+        <v>79</v>
       </c>
       <c r="C25" t="s">
-        <v>102</v>
+        <v>110</v>
       </c>
       <c r="D25" t="s">
         <v>10</v>
@@ -1868,13 +1832,13 @@
         <v>11</v>
       </c>
       <c r="F25" t="s">
-        <v>19</v>
+        <v>27</v>
       </c>
       <c r="G25" t="s">
         <v>13</v>
       </c>
       <c r="H25" t="s">
-        <v>131</v>
+        <v>84</v>
       </c>
       <c r="J25" s="3" t="s">
         <v>20</v>
@@ -1882,13 +1846,13 @@
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="B26" t="s">
         <v>32</v>
       </c>
       <c r="C26" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="D26" t="s">
         <v>10</v>
@@ -1897,13 +1861,13 @@
         <v>11</v>
       </c>
       <c r="F26" t="s">
-        <v>195</v>
+        <v>19</v>
       </c>
       <c r="G26" t="s">
         <v>13</v>
       </c>
       <c r="H26" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="J26" s="3" t="s">
         <v>20</v>
@@ -1911,13 +1875,13 @@
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="B27" t="s">
         <v>32</v>
       </c>
       <c r="C27" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="D27" t="s">
         <v>10</v>
@@ -1926,13 +1890,13 @@
         <v>11</v>
       </c>
       <c r="F27" t="s">
-        <v>21</v>
+        <v>192</v>
       </c>
       <c r="G27" t="s">
         <v>13</v>
       </c>
       <c r="H27" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="J27" s="3" t="s">
         <v>20</v>
@@ -1940,13 +1904,13 @@
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="B28" t="s">
         <v>32</v>
       </c>
       <c r="C28" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="D28" t="s">
         <v>10</v>
@@ -1955,13 +1919,13 @@
         <v>11</v>
       </c>
       <c r="F28" t="s">
-        <v>189</v>
+        <v>21</v>
       </c>
       <c r="G28" t="s">
         <v>13</v>
       </c>
       <c r="H28" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="J28" s="3" t="s">
         <v>20</v>
@@ -1969,13 +1933,13 @@
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="B29" t="s">
         <v>32</v>
       </c>
       <c r="C29" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="D29" t="s">
         <v>10</v>
@@ -1984,13 +1948,13 @@
         <v>11</v>
       </c>
       <c r="F29" t="s">
-        <v>24</v>
+        <v>186</v>
       </c>
       <c r="G29" t="s">
         <v>13</v>
       </c>
       <c r="H29" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="J29" s="3" t="s">
         <v>20</v>
@@ -1998,13 +1962,13 @@
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="B30" t="s">
         <v>32</v>
       </c>
       <c r="C30" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="D30" t="s">
         <v>10</v>
@@ -2013,27 +1977,27 @@
         <v>11</v>
       </c>
       <c r="F30" t="s">
-        <v>196</v>
+        <v>24</v>
       </c>
       <c r="G30" t="s">
         <v>13</v>
       </c>
       <c r="H30" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="J30" s="3" t="s">
-        <v>135</v>
+        <v>20</v>
       </c>
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="B31" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C31" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="D31" t="s">
         <v>10</v>
@@ -2042,27 +2006,27 @@
         <v>11</v>
       </c>
       <c r="F31" t="s">
-        <v>19</v>
+        <v>193</v>
       </c>
       <c r="G31" t="s">
         <v>13</v>
       </c>
       <c r="H31" t="s">
-        <v>136</v>
+        <v>131</v>
       </c>
       <c r="J31" s="3" t="s">
-        <v>20</v>
+        <v>132</v>
       </c>
     </row>
     <row r="32" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="B32" t="s">
         <v>31</v>
       </c>
       <c r="C32" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="D32" t="s">
         <v>10</v>
@@ -2071,13 +2035,13 @@
         <v>11</v>
       </c>
       <c r="F32" t="s">
-        <v>195</v>
+        <v>19</v>
       </c>
       <c r="G32" t="s">
         <v>13</v>
       </c>
       <c r="H32" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
       <c r="J32" s="3" t="s">
         <v>20</v>
@@ -2085,13 +2049,13 @@
     </row>
     <row r="33" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="B33" t="s">
         <v>31</v>
       </c>
       <c r="C33" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="D33" t="s">
         <v>10</v>
@@ -2100,13 +2064,13 @@
         <v>11</v>
       </c>
       <c r="F33" t="s">
-        <v>21</v>
+        <v>192</v>
       </c>
       <c r="G33" t="s">
         <v>13</v>
       </c>
       <c r="H33" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="J33" s="3" t="s">
         <v>20</v>
@@ -2114,13 +2078,13 @@
     </row>
     <row r="34" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="B34" t="s">
         <v>31</v>
       </c>
       <c r="C34" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="D34" t="s">
         <v>10</v>
@@ -2129,13 +2093,13 @@
         <v>11</v>
       </c>
       <c r="F34" t="s">
-        <v>189</v>
+        <v>21</v>
       </c>
       <c r="G34" t="s">
         <v>13</v>
       </c>
       <c r="H34" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="J34" s="3" t="s">
         <v>20</v>
@@ -2143,13 +2107,13 @@
     </row>
     <row r="35" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="B35" t="s">
         <v>31</v>
       </c>
       <c r="C35" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="D35" t="s">
         <v>10</v>
@@ -2158,13 +2122,13 @@
         <v>11</v>
       </c>
       <c r="F35" t="s">
-        <v>24</v>
+        <v>186</v>
       </c>
       <c r="G35" t="s">
         <v>13</v>
       </c>
       <c r="H35" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="J35" s="3" t="s">
         <v>20</v>
@@ -2172,13 +2136,13 @@
     </row>
     <row r="36" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="B36" t="s">
         <v>31</v>
       </c>
       <c r="C36" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="D36" t="s">
         <v>10</v>
@@ -2187,27 +2151,27 @@
         <v>11</v>
       </c>
       <c r="F36" t="s">
-        <v>196</v>
+        <v>24</v>
       </c>
       <c r="G36" t="s">
         <v>13</v>
       </c>
       <c r="H36" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
       <c r="J36" s="3" t="s">
-        <v>135</v>
+        <v>20</v>
       </c>
     </row>
     <row r="37" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>103</v>
+        <v>98</v>
       </c>
       <c r="B37" t="s">
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="C37" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
       <c r="D37" t="s">
         <v>10</v>
@@ -2216,27 +2180,27 @@
         <v>11</v>
       </c>
       <c r="F37" t="s">
-        <v>14</v>
+        <v>193</v>
       </c>
       <c r="G37" t="s">
-        <v>36</v>
+        <v>13</v>
       </c>
       <c r="H37" t="s">
-        <v>105</v>
+        <v>136</v>
       </c>
       <c r="J37" s="3" t="s">
-        <v>20</v>
+        <v>132</v>
       </c>
     </row>
     <row r="38" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="B38" t="s">
-        <v>32</v>
+        <v>25</v>
       </c>
       <c r="C38" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="D38" t="s">
         <v>10</v>
@@ -2248,13 +2212,10 @@
         <v>14</v>
       </c>
       <c r="G38" t="s">
-        <v>13</v>
+        <v>35</v>
       </c>
       <c r="H38" t="s">
-        <v>105</v>
-      </c>
-      <c r="I38" s="3">
-        <v>52</v>
+        <v>102</v>
       </c>
       <c r="J38" s="3" t="s">
         <v>20</v>
@@ -2262,13 +2223,13 @@
     </row>
     <row r="39" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>106</v>
+        <v>100</v>
       </c>
       <c r="B39" t="s">
-        <v>25</v>
+        <v>32</v>
       </c>
       <c r="C39" t="s">
-        <v>140</v>
+        <v>101</v>
       </c>
       <c r="D39" t="s">
         <v>10</v>
@@ -2277,27 +2238,30 @@
         <v>11</v>
       </c>
       <c r="F39" t="s">
-        <v>27</v>
+        <v>14</v>
       </c>
       <c r="G39" t="s">
         <v>13</v>
       </c>
       <c r="H39" t="s">
-        <v>78</v>
+        <v>102</v>
+      </c>
+      <c r="I39" s="3">
+        <v>52</v>
       </c>
       <c r="J39" s="3" t="s">
-        <v>107</v>
+        <v>20</v>
       </c>
     </row>
     <row r="40" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>197</v>
+        <v>103</v>
       </c>
       <c r="B40" t="s">
-        <v>198</v>
+        <v>25</v>
       </c>
       <c r="C40" t="s">
-        <v>199</v>
+        <v>137</v>
       </c>
       <c r="D40" t="s">
         <v>10</v>
@@ -2306,27 +2270,27 @@
         <v>11</v>
       </c>
       <c r="F40" t="s">
-        <v>148</v>
+        <v>27</v>
       </c>
       <c r="G40" t="s">
         <v>13</v>
       </c>
       <c r="H40" t="s">
-        <v>200</v>
+        <v>75</v>
       </c>
       <c r="J40" s="3" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
     </row>
     <row r="41" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
-        <v>108</v>
+        <v>194</v>
       </c>
       <c r="B41" t="s">
-        <v>109</v>
+        <v>195</v>
       </c>
       <c r="C41" t="s">
-        <v>110</v>
+        <v>196</v>
       </c>
       <c r="D41" t="s">
         <v>10</v>
@@ -2335,27 +2299,27 @@
         <v>11</v>
       </c>
       <c r="F41" t="s">
-        <v>19</v>
+        <v>145</v>
       </c>
       <c r="G41" t="s">
         <v>13</v>
       </c>
       <c r="H41" t="s">
-        <v>159</v>
+        <v>197</v>
       </c>
       <c r="J41" s="3" t="s">
-        <v>111</v>
+        <v>104</v>
       </c>
     </row>
     <row r="42" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
-        <v>28</v>
+        <v>105</v>
       </c>
       <c r="B42" t="s">
-        <v>112</v>
+        <v>106</v>
       </c>
       <c r="C42" t="s">
-        <v>113</v>
+        <v>107</v>
       </c>
       <c r="D42" t="s">
         <v>10</v>
@@ -2370,21 +2334,21 @@
         <v>13</v>
       </c>
       <c r="H42" t="s">
-        <v>114</v>
+        <v>156</v>
       </c>
       <c r="J42" s="3" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
     </row>
     <row r="43" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
-        <v>115</v>
+        <v>28</v>
       </c>
       <c r="B43" t="s">
-        <v>201</v>
+        <v>109</v>
       </c>
       <c r="C43" t="s">
-        <v>116</v>
+        <v>110</v>
       </c>
       <c r="D43" t="s">
         <v>10</v>
@@ -2393,27 +2357,27 @@
         <v>11</v>
       </c>
       <c r="F43" t="s">
-        <v>27</v>
+        <v>19</v>
       </c>
       <c r="G43" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H43" t="s">
-        <v>202</v>
+        <v>111</v>
       </c>
       <c r="J43" s="3" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
     </row>
     <row r="44" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="B44" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
       <c r="C44" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="D44" t="s">
         <v>10</v>
@@ -2422,27 +2386,27 @@
         <v>11</v>
       </c>
       <c r="F44" t="s">
-        <v>177</v>
+        <v>27</v>
       </c>
       <c r="G44" t="s">
         <v>12</v>
       </c>
       <c r="H44" t="s">
-        <v>202</v>
+        <v>199</v>
       </c>
       <c r="J44" s="3" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
     </row>
     <row r="45" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="B45" t="s">
-        <v>204</v>
+        <v>198</v>
       </c>
       <c r="C45" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="D45" t="s">
         <v>10</v>
@@ -2451,27 +2415,27 @@
         <v>11</v>
       </c>
       <c r="F45" t="s">
-        <v>27</v>
+        <v>174</v>
       </c>
       <c r="G45" t="s">
         <v>12</v>
       </c>
       <c r="H45" t="s">
-        <v>178</v>
+        <v>199</v>
       </c>
       <c r="J45" s="3" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
     </row>
     <row r="46" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
-        <v>115</v>
+        <v>200</v>
       </c>
       <c r="B46" t="s">
-        <v>203</v>
+        <v>142</v>
       </c>
       <c r="C46" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="D46" t="s">
         <v>10</v>
@@ -2480,27 +2444,27 @@
         <v>11</v>
       </c>
       <c r="F46" t="s">
-        <v>177</v>
+        <v>27</v>
       </c>
       <c r="G46" t="s">
         <v>12</v>
       </c>
       <c r="H46" t="s">
-        <v>178</v>
+        <v>143</v>
       </c>
       <c r="J46" s="3" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
     </row>
     <row r="47" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
-        <v>205</v>
+        <v>200</v>
       </c>
       <c r="B47" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="C47" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="D47" t="s">
         <v>10</v>
@@ -2509,27 +2473,27 @@
         <v>11</v>
       </c>
       <c r="F47" t="s">
-        <v>27</v>
+        <v>174</v>
       </c>
       <c r="G47" t="s">
         <v>12</v>
       </c>
       <c r="H47" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="J47" s="3" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
     </row>
     <row r="48" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
-        <v>205</v>
+        <v>176</v>
       </c>
       <c r="B48" t="s">
-        <v>145</v>
+        <v>177</v>
       </c>
       <c r="C48" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="D48" t="s">
         <v>10</v>
@@ -2538,27 +2502,27 @@
         <v>11</v>
       </c>
       <c r="F48" t="s">
-        <v>177</v>
+        <v>27</v>
       </c>
       <c r="G48" t="s">
         <v>12</v>
       </c>
       <c r="H48" t="s">
-        <v>146</v>
+        <v>178</v>
       </c>
       <c r="J48" s="3" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
     </row>
     <row r="49" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
-        <v>179</v>
+        <v>176</v>
       </c>
       <c r="B49" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
       <c r="C49" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="D49" t="s">
         <v>10</v>
@@ -2567,27 +2531,27 @@
         <v>11</v>
       </c>
       <c r="F49" t="s">
-        <v>27</v>
+        <v>174</v>
       </c>
       <c r="G49" t="s">
         <v>12</v>
       </c>
       <c r="H49" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
       <c r="J49" s="3" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
     </row>
     <row r="50" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
-        <v>179</v>
+        <v>112</v>
       </c>
       <c r="B50" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
       <c r="C50" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="D50" t="s">
         <v>10</v>
@@ -2596,27 +2560,27 @@
         <v>11</v>
       </c>
       <c r="F50" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="G50" t="s">
         <v>12</v>
       </c>
       <c r="H50" t="s">
-        <v>181</v>
+        <v>175</v>
       </c>
       <c r="J50" s="3" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
     </row>
     <row r="51" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="B51" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
       <c r="C51" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="D51" t="s">
         <v>10</v>
@@ -2625,27 +2589,27 @@
         <v>11</v>
       </c>
       <c r="F51" t="s">
-        <v>177</v>
+        <v>27</v>
       </c>
       <c r="G51" t="s">
         <v>12</v>
       </c>
       <c r="H51" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="J51" s="3" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
     </row>
     <row r="52" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
-        <v>115</v>
+        <v>141</v>
       </c>
       <c r="B52" t="s">
-        <v>180</v>
+        <v>142</v>
       </c>
       <c r="C52" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="D52" t="s">
         <v>10</v>
@@ -2660,21 +2624,21 @@
         <v>12</v>
       </c>
       <c r="H52" t="s">
-        <v>178</v>
+        <v>143</v>
       </c>
       <c r="J52" s="3" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
     </row>
     <row r="53" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="B53" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="C53" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="D53" t="s">
         <v>10</v>
@@ -2683,27 +2647,27 @@
         <v>11</v>
       </c>
       <c r="F53" t="s">
-        <v>27</v>
+        <v>174</v>
       </c>
       <c r="G53" t="s">
         <v>12</v>
       </c>
       <c r="H53" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="J53" s="3" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
     </row>
     <row r="54" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
-        <v>144</v>
+        <v>112</v>
       </c>
       <c r="B54" t="s">
-        <v>145</v>
+        <v>139</v>
       </c>
       <c r="C54" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="D54" t="s">
         <v>10</v>
@@ -2712,27 +2676,27 @@
         <v>11</v>
       </c>
       <c r="F54" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="G54" t="s">
         <v>12</v>
       </c>
       <c r="H54" t="s">
-        <v>146</v>
+        <v>140</v>
       </c>
       <c r="J54" s="3" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
     </row>
     <row r="55" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="B55" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="C55" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="D55" t="s">
         <v>10</v>
@@ -2741,59 +2705,59 @@
         <v>11</v>
       </c>
       <c r="F55" t="s">
-        <v>177</v>
+        <v>27</v>
       </c>
       <c r="G55" t="s">
         <v>12</v>
       </c>
       <c r="H55" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="J55" s="3" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
     </row>
     <row r="56" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
+        <v>118</v>
+      </c>
+      <c r="B56" t="s">
         <v>115</v>
       </c>
-      <c r="B56" t="s">
-        <v>142</v>
-      </c>
       <c r="C56" t="s">
-        <v>116</v>
+        <v>22</v>
       </c>
       <c r="D56" t="s">
-        <v>10</v>
+        <v>117</v>
       </c>
       <c r="E56" t="s">
         <v>11</v>
       </c>
       <c r="F56" t="s">
-        <v>27</v>
+        <v>19</v>
       </c>
       <c r="G56" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H56" t="s">
-        <v>143</v>
-      </c>
-      <c r="J56" s="3" t="s">
-        <v>107</v>
+        <v>138</v>
+      </c>
+      <c r="I56" s="3">
+        <v>49</v>
       </c>
     </row>
     <row r="57" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
-        <v>121</v>
+        <v>114</v>
       </c>
       <c r="B57" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="C57" t="s">
-        <v>22</v>
+        <v>116</v>
       </c>
       <c r="D57" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="E57" t="s">
         <v>11</v>
@@ -2805,7 +2769,7 @@
         <v>13</v>
       </c>
       <c r="H57" t="s">
-        <v>141</v>
+        <v>147</v>
       </c>
       <c r="I57" s="3">
         <v>49</v>
@@ -2813,28 +2777,28 @@
     </row>
     <row r="58" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
+        <v>118</v>
+      </c>
+      <c r="B58" t="s">
+        <v>26</v>
+      </c>
+      <c r="C58" t="s">
+        <v>22</v>
+      </c>
+      <c r="D58" t="s">
         <v>117</v>
       </c>
-      <c r="B58" t="s">
-        <v>118</v>
-      </c>
-      <c r="C58" t="s">
+      <c r="E58" t="s">
+        <v>11</v>
+      </c>
+      <c r="F58" t="s">
+        <v>27</v>
+      </c>
+      <c r="G58" t="s">
+        <v>13</v>
+      </c>
+      <c r="H58" t="s">
         <v>119</v>
-      </c>
-      <c r="D58" t="s">
-        <v>120</v>
-      </c>
-      <c r="E58" t="s">
-        <v>11</v>
-      </c>
-      <c r="F58" t="s">
-        <v>19</v>
-      </c>
-      <c r="G58" t="s">
-        <v>13</v>
-      </c>
-      <c r="H58" t="s">
-        <v>150</v>
       </c>
       <c r="I58" s="3">
         <v>49</v>
@@ -2842,42 +2806,39 @@
     </row>
     <row r="59" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
+        <v>120</v>
+      </c>
+      <c r="B59" t="s">
+        <v>168</v>
+      </c>
+      <c r="C59" t="s">
         <v>121</v>
       </c>
-      <c r="B59" t="s">
-        <v>26</v>
-      </c>
-      <c r="C59" t="s">
-        <v>22</v>
-      </c>
       <c r="D59" t="s">
-        <v>120</v>
+        <v>10</v>
       </c>
       <c r="E59" t="s">
         <v>11</v>
       </c>
       <c r="F59" t="s">
-        <v>27</v>
+        <v>19</v>
       </c>
       <c r="G59" t="s">
         <v>13</v>
       </c>
       <c r="H59" t="s">
-        <v>122</v>
-      </c>
-      <c r="I59" s="3">
-        <v>49</v>
+        <v>169</v>
       </c>
     </row>
     <row r="60" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="B60" t="s">
-        <v>171</v>
+        <v>79</v>
       </c>
       <c r="C60" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="D60" t="s">
         <v>10</v>
@@ -2892,44 +2853,47 @@
         <v>13</v>
       </c>
       <c r="H60" t="s">
-        <v>172</v>
+        <v>122</v>
       </c>
     </row>
     <row r="61" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
+        <v>120</v>
+      </c>
+      <c r="B61" t="s">
+        <v>79</v>
+      </c>
+      <c r="C61" t="s">
+        <v>121</v>
+      </c>
+      <c r="D61" t="s">
+        <v>10</v>
+      </c>
+      <c r="E61" t="s">
+        <v>11</v>
+      </c>
+      <c r="F61" t="s">
         <v>123</v>
       </c>
-      <c r="B61" t="s">
-        <v>82</v>
-      </c>
-      <c r="C61" t="s">
+      <c r="G61" t="s">
+        <v>13</v>
+      </c>
+      <c r="H61" t="s">
         <v>124</v>
       </c>
-      <c r="D61" t="s">
-        <v>10</v>
-      </c>
-      <c r="E61" t="s">
-        <v>11</v>
-      </c>
-      <c r="F61" t="s">
-        <v>19</v>
-      </c>
-      <c r="G61" t="s">
-        <v>13</v>
-      </c>
-      <c r="H61" t="s">
+      <c r="J61" s="3" t="s">
         <v>125</v>
       </c>
     </row>
     <row r="62" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
-        <v>123</v>
+        <v>30</v>
       </c>
       <c r="B62" t="s">
-        <v>82</v>
+        <v>31</v>
       </c>
       <c r="C62" t="s">
-        <v>124</v>
+        <v>22</v>
       </c>
       <c r="D62" t="s">
         <v>10</v>
@@ -2938,16 +2902,16 @@
         <v>11</v>
       </c>
       <c r="F62" t="s">
-        <v>126</v>
+        <v>19</v>
       </c>
       <c r="G62" t="s">
         <v>13</v>
       </c>
       <c r="H62" t="s">
-        <v>127</v>
+        <v>179</v>
       </c>
       <c r="J62" s="3" t="s">
-        <v>128</v>
+        <v>160</v>
       </c>
     </row>
     <row r="63" spans="1:10" x14ac:dyDescent="0.3">
@@ -2955,7 +2919,7 @@
         <v>30</v>
       </c>
       <c r="B63" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="C63" t="s">
         <v>22</v>
@@ -2973,761 +2937,773 @@
         <v>13</v>
       </c>
       <c r="H63" t="s">
-        <v>182</v>
+        <v>159</v>
       </c>
       <c r="J63" s="3" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
     </row>
     <row r="64" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
-        <v>30</v>
+        <v>54</v>
       </c>
       <c r="B64" t="s">
-        <v>26</v>
+        <v>55</v>
       </c>
       <c r="C64" t="s">
-        <v>22</v>
+        <v>33</v>
       </c>
       <c r="D64" t="s">
-        <v>10</v>
+        <v>34</v>
       </c>
       <c r="E64" t="s">
         <v>11</v>
       </c>
       <c r="F64" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="G64" t="s">
-        <v>13</v>
-      </c>
-      <c r="H64" t="s">
-        <v>162</v>
+        <v>48</v>
       </c>
       <c r="J64" s="3" t="s">
-        <v>163</v>
+        <v>41</v>
       </c>
     </row>
     <row r="65" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
-        <v>69</v>
+        <v>54</v>
       </c>
       <c r="B65" t="s">
-        <v>206</v>
+        <v>54</v>
       </c>
       <c r="C65" t="s">
-        <v>207</v>
+        <v>33</v>
       </c>
       <c r="D65" t="s">
-        <v>10</v>
+        <v>34</v>
       </c>
       <c r="E65" t="s">
         <v>11</v>
       </c>
       <c r="F65" t="s">
-        <v>19</v>
+        <v>56</v>
       </c>
       <c r="G65" t="s">
-        <v>12</v>
+        <v>53</v>
+      </c>
+      <c r="J65" s="3" t="s">
+        <v>201</v>
       </c>
     </row>
     <row r="66" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
-        <v>32</v>
+        <v>54</v>
       </c>
       <c r="B66" t="s">
-        <v>206</v>
+        <v>54</v>
       </c>
       <c r="C66" t="s">
-        <v>207</v>
+        <v>33</v>
       </c>
       <c r="D66" t="s">
-        <v>10</v>
+        <v>34</v>
       </c>
       <c r="E66" t="s">
         <v>11</v>
       </c>
       <c r="F66" t="s">
-        <v>19</v>
+        <v>51</v>
       </c>
       <c r="G66" t="s">
-        <v>12</v>
+        <v>48</v>
+      </c>
+      <c r="J66" s="3" t="s">
+        <v>202</v>
       </c>
     </row>
     <row r="67" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="B67" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="C67" t="s">
+        <v>33</v>
+      </c>
+      <c r="D67" t="s">
         <v>34</v>
       </c>
-      <c r="D67" t="s">
-        <v>35</v>
-      </c>
       <c r="E67" t="s">
         <v>11</v>
       </c>
       <c r="F67" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="G67" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="J67" s="3" t="s">
-        <v>44</v>
+        <v>203</v>
       </c>
     </row>
     <row r="68" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
-        <v>57</v>
+        <v>36</v>
       </c>
       <c r="B68" t="s">
-        <v>57</v>
+        <v>37</v>
       </c>
       <c r="C68" t="s">
+        <v>33</v>
+      </c>
+      <c r="D68" t="s">
         <v>34</v>
       </c>
-      <c r="D68" t="s">
+      <c r="E68" t="s">
+        <v>11</v>
+      </c>
+      <c r="F68" t="s">
+        <v>38</v>
+      </c>
+      <c r="G68" t="s">
         <v>35</v>
       </c>
-      <c r="E68" t="s">
-        <v>11</v>
-      </c>
-      <c r="F68" t="s">
-        <v>59</v>
-      </c>
-      <c r="G68" t="s">
-        <v>56</v>
-      </c>
       <c r="J68" s="3" t="s">
-        <v>208</v>
+        <v>204</v>
       </c>
     </row>
     <row r="69" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
-        <v>57</v>
+        <v>36</v>
       </c>
       <c r="B69" t="s">
-        <v>57</v>
+        <v>39</v>
       </c>
       <c r="C69" t="s">
+        <v>33</v>
+      </c>
+      <c r="D69" t="s">
         <v>34</v>
       </c>
-      <c r="D69" t="s">
+      <c r="E69" t="s">
+        <v>11</v>
+      </c>
+      <c r="F69" t="s">
+        <v>38</v>
+      </c>
+      <c r="G69" t="s">
         <v>35</v>
       </c>
-      <c r="E69" t="s">
-        <v>11</v>
-      </c>
-      <c r="F69" t="s">
-        <v>54</v>
-      </c>
-      <c r="G69" t="s">
-        <v>51</v>
-      </c>
       <c r="J69" s="3" t="s">
-        <v>209</v>
+        <v>204</v>
       </c>
     </row>
     <row r="70" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
-        <v>57</v>
+        <v>36</v>
       </c>
       <c r="B70" t="s">
-        <v>57</v>
+        <v>40</v>
       </c>
       <c r="C70" t="s">
+        <v>33</v>
+      </c>
+      <c r="D70" t="s">
         <v>34</v>
       </c>
-      <c r="D70" t="s">
+      <c r="E70" t="s">
+        <v>11</v>
+      </c>
+      <c r="F70" t="s">
+        <v>38</v>
+      </c>
+      <c r="G70" t="s">
         <v>35</v>
       </c>
-      <c r="E70" t="s">
-        <v>11</v>
-      </c>
-      <c r="F70" t="s">
-        <v>14</v>
-      </c>
-      <c r="G70" t="s">
-        <v>56</v>
-      </c>
       <c r="J70" s="3" t="s">
-        <v>210</v>
+        <v>204</v>
       </c>
     </row>
     <row r="71" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="B71" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="C71" t="s">
+        <v>33</v>
+      </c>
+      <c r="D71" t="s">
         <v>34</v>
       </c>
-      <c r="D71" t="s">
+      <c r="E71" t="s">
+        <v>11</v>
+      </c>
+      <c r="F71" t="s">
+        <v>38</v>
+      </c>
+      <c r="G71" t="s">
         <v>35</v>
       </c>
-      <c r="E71" t="s">
-        <v>11</v>
-      </c>
-      <c r="F71" t="s">
-        <v>41</v>
-      </c>
-      <c r="G71" t="s">
-        <v>36</v>
-      </c>
       <c r="J71" s="3" t="s">
-        <v>211</v>
+        <v>204</v>
       </c>
     </row>
     <row r="72" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="B72" t="s">
         <v>42</v>
       </c>
       <c r="C72" t="s">
+        <v>33</v>
+      </c>
+      <c r="D72" t="s">
         <v>34</v>
       </c>
-      <c r="D72" t="s">
+      <c r="E72" t="s">
+        <v>11</v>
+      </c>
+      <c r="F72" t="s">
+        <v>38</v>
+      </c>
+      <c r="G72" t="s">
         <v>35</v>
       </c>
-      <c r="E72" t="s">
-        <v>11</v>
-      </c>
-      <c r="F72" t="s">
-        <v>41</v>
-      </c>
-      <c r="G72" t="s">
-        <v>36</v>
-      </c>
       <c r="J72" s="3" t="s">
-        <v>211</v>
+        <v>202</v>
       </c>
     </row>
     <row r="73" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="B73" t="s">
         <v>43</v>
       </c>
       <c r="C73" t="s">
+        <v>33</v>
+      </c>
+      <c r="D73" t="s">
         <v>34</v>
       </c>
-      <c r="D73" t="s">
-        <v>35</v>
-      </c>
       <c r="E73" t="s">
         <v>11</v>
       </c>
       <c r="F73" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="G73" t="s">
-        <v>36</v>
+        <v>48</v>
       </c>
       <c r="J73" s="3" t="s">
-        <v>211</v>
+        <v>205</v>
       </c>
     </row>
     <row r="74" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
-        <v>39</v>
+        <v>32</v>
       </c>
       <c r="B74" t="s">
-        <v>39</v>
+        <v>32</v>
       </c>
       <c r="C74" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D74" t="s">
+        <v>44</v>
+      </c>
+      <c r="E74" t="s">
+        <v>11</v>
+      </c>
+      <c r="F74" t="s">
+        <v>45</v>
+      </c>
+      <c r="G74" t="s">
         <v>35</v>
       </c>
-      <c r="E74" t="s">
-        <v>11</v>
-      </c>
-      <c r="F74" t="s">
-        <v>41</v>
-      </c>
-      <c r="G74" t="s">
-        <v>36</v>
-      </c>
       <c r="J74" s="3" t="s">
-        <v>211</v>
+        <v>202</v>
       </c>
     </row>
     <row r="75" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
-        <v>45</v>
+        <v>32</v>
       </c>
       <c r="B75" t="s">
-        <v>45</v>
+        <v>32</v>
       </c>
       <c r="C75" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D75" t="s">
+        <v>44</v>
+      </c>
+      <c r="E75" t="s">
+        <v>11</v>
+      </c>
+      <c r="F75" t="s">
+        <v>46</v>
+      </c>
+      <c r="G75" t="s">
         <v>35</v>
       </c>
-      <c r="E75" t="s">
-        <v>11</v>
-      </c>
-      <c r="F75" t="s">
-        <v>41</v>
-      </c>
-      <c r="G75" t="s">
-        <v>36</v>
-      </c>
       <c r="J75" s="3" t="s">
-        <v>209</v>
+        <v>202</v>
       </c>
     </row>
     <row r="76" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A76" t="s">
+        <v>47</v>
+      </c>
+      <c r="B76" t="s">
+        <v>47</v>
+      </c>
+      <c r="C76" t="s">
+        <v>33</v>
+      </c>
+      <c r="D76" t="s">
+        <v>34</v>
+      </c>
+      <c r="E76" t="s">
+        <v>11</v>
+      </c>
+      <c r="F76" t="s">
         <v>46</v>
       </c>
-      <c r="B76" t="s">
-        <v>46</v>
-      </c>
-      <c r="C76" t="s">
-        <v>34</v>
-      </c>
-      <c r="D76" t="s">
-        <v>35</v>
-      </c>
-      <c r="E76" t="s">
-        <v>11</v>
-      </c>
-      <c r="F76" t="s">
-        <v>41</v>
-      </c>
       <c r="G76" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="J76" s="3" t="s">
-        <v>212</v>
+        <v>49</v>
       </c>
     </row>
     <row r="77" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A77" t="s">
-        <v>32</v>
+        <v>148</v>
       </c>
       <c r="B77" t="s">
-        <v>32</v>
+        <v>148</v>
       </c>
       <c r="C77" t="s">
+        <v>33</v>
+      </c>
+      <c r="D77" t="s">
         <v>34</v>
       </c>
-      <c r="D77" t="s">
-        <v>47</v>
-      </c>
       <c r="E77" t="s">
         <v>11</v>
       </c>
       <c r="F77" t="s">
-        <v>48</v>
+        <v>145</v>
       </c>
       <c r="G77" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="J77" s="3" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
     </row>
     <row r="78" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A78" t="s">
-        <v>32</v>
+        <v>57</v>
       </c>
       <c r="B78" t="s">
-        <v>32</v>
+        <v>57</v>
       </c>
       <c r="C78" t="s">
+        <v>33</v>
+      </c>
+      <c r="D78" t="s">
         <v>34</v>
       </c>
-      <c r="D78" t="s">
-        <v>47</v>
-      </c>
       <c r="E78" t="s">
         <v>11</v>
       </c>
       <c r="F78" t="s">
-        <v>49</v>
+        <v>149</v>
       </c>
       <c r="G78" t="s">
-        <v>36</v>
+        <v>53</v>
       </c>
       <c r="J78" s="3" t="s">
-        <v>209</v>
+        <v>202</v>
       </c>
     </row>
     <row r="79" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A79" t="s">
-        <v>50</v>
+        <v>25</v>
       </c>
       <c r="B79" t="s">
-        <v>50</v>
+        <v>25</v>
       </c>
       <c r="C79" t="s">
+        <v>33</v>
+      </c>
+      <c r="D79" t="s">
         <v>34</v>
       </c>
-      <c r="D79" t="s">
-        <v>35</v>
-      </c>
       <c r="E79" t="s">
         <v>11</v>
       </c>
       <c r="F79" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="G79" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="J79" s="3" t="s">
-        <v>52</v>
+        <v>207</v>
       </c>
     </row>
     <row r="80" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A80" t="s">
-        <v>33</v>
+        <v>180</v>
       </c>
       <c r="B80" t="s">
-        <v>33</v>
+        <v>180</v>
       </c>
       <c r="C80" t="s">
+        <v>33</v>
+      </c>
+      <c r="D80" t="s">
         <v>34</v>
       </c>
-      <c r="D80" t="s">
-        <v>35</v>
-      </c>
       <c r="E80" t="s">
         <v>11</v>
       </c>
       <c r="F80" t="s">
-        <v>17</v>
+        <v>51</v>
       </c>
       <c r="G80" t="s">
-        <v>36</v>
+        <v>48</v>
       </c>
       <c r="J80" s="3" t="s">
-        <v>213</v>
+        <v>202</v>
       </c>
     </row>
     <row r="81" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A81" t="s">
-        <v>37</v>
+        <v>28</v>
       </c>
       <c r="B81" t="s">
-        <v>37</v>
+        <v>28</v>
       </c>
       <c r="C81" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D81" t="s">
-        <v>35</v>
+        <v>44</v>
       </c>
       <c r="E81" t="s">
         <v>11</v>
       </c>
       <c r="F81" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="G81" t="s">
-        <v>36</v>
+        <v>58</v>
       </c>
       <c r="J81" s="3" t="s">
-        <v>214</v>
+        <v>59</v>
       </c>
     </row>
     <row r="82" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A82" t="s">
-        <v>37</v>
+        <v>28</v>
       </c>
       <c r="B82" t="s">
-        <v>37</v>
+        <v>28</v>
       </c>
       <c r="C82" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="D82" t="s">
-        <v>35</v>
+        <v>44</v>
       </c>
       <c r="E82" t="s">
         <v>11</v>
       </c>
       <c r="F82" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="G82" t="s">
-        <v>36</v>
+        <v>58</v>
       </c>
       <c r="J82" s="3" t="s">
-        <v>215</v>
+        <v>59</v>
       </c>
     </row>
     <row r="83" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A83" t="s">
-        <v>151</v>
+        <v>60</v>
       </c>
       <c r="B83" t="s">
-        <v>151</v>
+        <v>60</v>
       </c>
       <c r="C83" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D83" t="s">
-        <v>35</v>
+        <v>44</v>
       </c>
       <c r="E83" t="s">
         <v>11</v>
       </c>
       <c r="F83" t="s">
-        <v>148</v>
+        <v>14</v>
       </c>
       <c r="G83" t="s">
-        <v>36</v>
+        <v>53</v>
       </c>
       <c r="J83" s="3" t="s">
-        <v>216</v>
+        <v>59</v>
       </c>
     </row>
     <row r="84" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A84" t="s">
-        <v>60</v>
+        <v>29</v>
       </c>
       <c r="B84" t="s">
-        <v>60</v>
+        <v>29</v>
       </c>
       <c r="C84" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D84" t="s">
-        <v>35</v>
+        <v>44</v>
       </c>
       <c r="E84" t="s">
         <v>11</v>
       </c>
       <c r="F84" t="s">
-        <v>152</v>
+        <v>145</v>
       </c>
       <c r="G84" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="J84" s="3" t="s">
-        <v>209</v>
+        <v>50</v>
       </c>
     </row>
     <row r="85" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A85" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="B85" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="C85" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D85" t="s">
-        <v>35</v>
+        <v>44</v>
       </c>
       <c r="E85" t="s">
         <v>11</v>
       </c>
       <c r="F85" t="s">
-        <v>54</v>
+        <v>151</v>
       </c>
       <c r="G85" t="s">
-        <v>51</v>
+        <v>58</v>
       </c>
       <c r="J85" s="3" t="s">
-        <v>217</v>
+        <v>50</v>
       </c>
     </row>
     <row r="86" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A86" t="s">
-        <v>183</v>
+        <v>29</v>
       </c>
       <c r="B86" t="s">
-        <v>183</v>
+        <v>29</v>
       </c>
       <c r="C86" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D86" t="s">
-        <v>35</v>
+        <v>44</v>
       </c>
       <c r="E86" t="s">
         <v>11</v>
       </c>
       <c r="F86" t="s">
-        <v>54</v>
+        <v>46</v>
       </c>
       <c r="G86" t="s">
-        <v>51</v>
+        <v>58</v>
       </c>
       <c r="J86" s="3" t="s">
-        <v>209</v>
+        <v>50</v>
       </c>
     </row>
     <row r="87" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A87" t="s">
-        <v>28</v>
+        <v>18</v>
       </c>
       <c r="B87" t="s">
-        <v>28</v>
+        <v>161</v>
       </c>
       <c r="C87" t="s">
+        <v>33</v>
+      </c>
+      <c r="D87" t="s">
         <v>34</v>
       </c>
-      <c r="D87" t="s">
-        <v>47</v>
-      </c>
       <c r="E87" t="s">
         <v>11</v>
       </c>
       <c r="F87" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="G87" t="s">
-        <v>61</v>
+        <v>35</v>
       </c>
       <c r="J87" s="3" t="s">
-        <v>62</v>
+        <v>162</v>
       </c>
     </row>
     <row r="88" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A88" t="s">
-        <v>28</v>
+        <v>18</v>
       </c>
       <c r="B88" t="s">
-        <v>28</v>
+        <v>163</v>
       </c>
       <c r="C88" t="s">
+        <v>33</v>
+      </c>
+      <c r="D88" t="s">
         <v>34</v>
       </c>
-      <c r="D88" t="s">
-        <v>47</v>
-      </c>
       <c r="E88" t="s">
         <v>11</v>
       </c>
       <c r="F88" t="s">
-        <v>16</v>
+        <v>78</v>
       </c>
       <c r="G88" t="s">
-        <v>61</v>
+        <v>35</v>
+      </c>
+      <c r="H88" t="s">
+        <v>164</v>
       </c>
       <c r="J88" s="3" t="s">
-        <v>62</v>
+        <v>162</v>
       </c>
     </row>
     <row r="89" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A89" t="s">
-        <v>63</v>
+        <v>18</v>
       </c>
       <c r="B89" t="s">
-        <v>63</v>
+        <v>165</v>
       </c>
       <c r="C89" t="s">
+        <v>33</v>
+      </c>
+      <c r="D89" t="s">
         <v>34</v>
       </c>
-      <c r="D89" t="s">
-        <v>47</v>
-      </c>
       <c r="E89" t="s">
         <v>11</v>
       </c>
       <c r="F89" t="s">
-        <v>14</v>
+        <v>78</v>
       </c>
       <c r="G89" t="s">
-        <v>56</v>
+        <v>35</v>
+      </c>
+      <c r="H89" t="s">
+        <v>164</v>
       </c>
       <c r="J89" s="3" t="s">
-        <v>62</v>
+        <v>162</v>
       </c>
     </row>
     <row r="90" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A90" t="s">
-        <v>29</v>
+        <v>18</v>
       </c>
       <c r="B90" t="s">
-        <v>29</v>
+        <v>166</v>
       </c>
       <c r="C90" t="s">
+        <v>33</v>
+      </c>
+      <c r="D90" t="s">
         <v>34</v>
       </c>
-      <c r="D90" t="s">
-        <v>47</v>
-      </c>
       <c r="E90" t="s">
         <v>11</v>
       </c>
       <c r="F90" t="s">
-        <v>148</v>
+        <v>78</v>
       </c>
       <c r="G90" t="s">
-        <v>61</v>
+        <v>35</v>
       </c>
       <c r="J90" s="3" t="s">
-        <v>53</v>
+        <v>162</v>
       </c>
     </row>
     <row r="91" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A91" t="s">
-        <v>29</v>
+        <v>18</v>
       </c>
       <c r="B91" t="s">
-        <v>29</v>
+        <v>167</v>
       </c>
       <c r="C91" t="s">
+        <v>33</v>
+      </c>
+      <c r="D91" t="s">
         <v>34</v>
       </c>
-      <c r="D91" t="s">
-        <v>47</v>
-      </c>
       <c r="E91" t="s">
         <v>11</v>
       </c>
       <c r="F91" t="s">
-        <v>154</v>
+        <v>78</v>
       </c>
       <c r="G91" t="s">
-        <v>61</v>
+        <v>35</v>
+      </c>
+      <c r="H91" t="s">
+        <v>164</v>
       </c>
       <c r="J91" s="3" t="s">
-        <v>53</v>
+        <v>162</v>
       </c>
     </row>
     <row r="92" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A92" t="s">
-        <v>29</v>
+        <v>18</v>
       </c>
       <c r="B92" t="s">
-        <v>29</v>
+        <v>18</v>
       </c>
       <c r="C92" t="s">
+        <v>33</v>
+      </c>
+      <c r="D92" t="s">
         <v>34</v>
       </c>
-      <c r="D92" t="s">
-        <v>47</v>
-      </c>
       <c r="E92" t="s">
         <v>11</v>
       </c>
       <c r="F92" t="s">
-        <v>49</v>
+        <v>14</v>
       </c>
       <c r="G92" t="s">
-        <v>61</v>
+        <v>53</v>
       </c>
       <c r="J92" s="3" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
     </row>
     <row r="93" spans="1:10" x14ac:dyDescent="0.3">
@@ -3735,204 +3711,195 @@
         <v>18</v>
       </c>
       <c r="B93" t="s">
-        <v>164</v>
+        <v>18</v>
       </c>
       <c r="C93" t="s">
+        <v>33</v>
+      </c>
+      <c r="D93" t="s">
         <v>34</v>
       </c>
-      <c r="D93" t="s">
-        <v>35</v>
-      </c>
       <c r="E93" t="s">
         <v>11</v>
       </c>
       <c r="F93" t="s">
-        <v>24</v>
+        <v>51</v>
       </c>
       <c r="G93" t="s">
-        <v>36</v>
+        <v>53</v>
       </c>
       <c r="J93" s="3" t="s">
-        <v>165</v>
+        <v>50</v>
       </c>
     </row>
     <row r="94" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A94" t="s">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="B94" t="s">
-        <v>166</v>
+        <v>26</v>
       </c>
       <c r="C94" t="s">
+        <v>33</v>
+      </c>
+      <c r="D94" t="s">
         <v>34</v>
       </c>
-      <c r="D94" t="s">
-        <v>35</v>
-      </c>
       <c r="E94" t="s">
         <v>11</v>
       </c>
       <c r="F94" t="s">
-        <v>81</v>
+        <v>19</v>
       </c>
       <c r="G94" t="s">
-        <v>36</v>
-      </c>
-      <c r="H94" t="s">
-        <v>167</v>
+        <v>53</v>
       </c>
       <c r="J94" s="3" t="s">
-        <v>165</v>
+        <v>208</v>
       </c>
     </row>
     <row r="95" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A95" t="s">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="B95" t="s">
-        <v>168</v>
+        <v>26</v>
       </c>
       <c r="C95" t="s">
+        <v>33</v>
+      </c>
+      <c r="D95" t="s">
         <v>34</v>
       </c>
-      <c r="D95" t="s">
-        <v>35</v>
-      </c>
       <c r="E95" t="s">
         <v>11</v>
       </c>
       <c r="F95" t="s">
-        <v>81</v>
+        <v>38</v>
       </c>
       <c r="G95" t="s">
-        <v>36</v>
-      </c>
-      <c r="H95" t="s">
-        <v>167</v>
+        <v>48</v>
       </c>
       <c r="J95" s="3" t="s">
-        <v>165</v>
+        <v>208</v>
       </c>
     </row>
     <row r="96" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A96" t="s">
-        <v>18</v>
+        <v>61</v>
       </c>
       <c r="B96" t="s">
-        <v>169</v>
+        <v>77</v>
       </c>
       <c r="C96" t="s">
+        <v>33</v>
+      </c>
+      <c r="D96" t="s">
         <v>34</v>
       </c>
-      <c r="D96" t="s">
+      <c r="E96" t="s">
+        <v>11</v>
+      </c>
+      <c r="F96" t="s">
+        <v>78</v>
+      </c>
+      <c r="G96" t="s">
         <v>35</v>
       </c>
-      <c r="E96" t="s">
-        <v>11</v>
-      </c>
-      <c r="F96" t="s">
-        <v>81</v>
-      </c>
-      <c r="G96" t="s">
-        <v>36</v>
-      </c>
       <c r="J96" s="3" t="s">
-        <v>165</v>
+        <v>52</v>
       </c>
     </row>
     <row r="97" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A97" t="s">
-        <v>18</v>
+        <v>61</v>
       </c>
       <c r="B97" t="s">
-        <v>170</v>
+        <v>62</v>
       </c>
       <c r="C97" t="s">
+        <v>33</v>
+      </c>
+      <c r="D97" t="s">
         <v>34</v>
       </c>
-      <c r="D97" t="s">
+      <c r="E97" t="s">
+        <v>11</v>
+      </c>
+      <c r="F97" t="s">
+        <v>21</v>
+      </c>
+      <c r="G97" t="s">
         <v>35</v>
       </c>
-      <c r="E97" t="s">
-        <v>11</v>
-      </c>
-      <c r="F97" t="s">
-        <v>81</v>
-      </c>
-      <c r="G97" t="s">
-        <v>36</v>
-      </c>
-      <c r="H97" t="s">
-        <v>167</v>
-      </c>
       <c r="J97" s="3" t="s">
-        <v>165</v>
+        <v>52</v>
       </c>
     </row>
     <row r="98" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A98" t="s">
-        <v>18</v>
+        <v>61</v>
       </c>
       <c r="B98" t="s">
-        <v>18</v>
+        <v>63</v>
       </c>
       <c r="C98" t="s">
+        <v>33</v>
+      </c>
+      <c r="D98" t="s">
         <v>34</v>
       </c>
-      <c r="D98" t="s">
+      <c r="E98" t="s">
+        <v>11</v>
+      </c>
+      <c r="F98" t="s">
+        <v>21</v>
+      </c>
+      <c r="G98" t="s">
         <v>35</v>
       </c>
-      <c r="E98" t="s">
-        <v>11</v>
-      </c>
-      <c r="F98" t="s">
-        <v>14</v>
-      </c>
-      <c r="G98" t="s">
-        <v>56</v>
-      </c>
       <c r="J98" s="3" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="99" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A99" t="s">
-        <v>18</v>
+        <v>61</v>
       </c>
       <c r="B99" t="s">
-        <v>18</v>
+        <v>61</v>
       </c>
       <c r="C99" t="s">
+        <v>33</v>
+      </c>
+      <c r="D99" t="s">
         <v>34</v>
       </c>
-      <c r="D99" t="s">
+      <c r="E99" t="s">
+        <v>11</v>
+      </c>
+      <c r="F99" t="s">
+        <v>51</v>
+      </c>
+      <c r="G99" t="s">
         <v>35</v>
       </c>
-      <c r="E99" t="s">
-        <v>11</v>
-      </c>
-      <c r="F99" t="s">
-        <v>54</v>
-      </c>
-      <c r="G99" t="s">
-        <v>56</v>
-      </c>
       <c r="J99" s="3" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="100" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A100" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="B100" t="s">
-        <v>26</v>
+        <v>54</v>
       </c>
       <c r="C100" t="s">
+        <v>33</v>
+      </c>
+      <c r="D100" t="s">
         <v>34</v>
-      </c>
-      <c r="D100" t="s">
-        <v>35</v>
       </c>
       <c r="E100" t="s">
         <v>11</v>
@@ -3941,592 +3908,410 @@
         <v>19</v>
       </c>
       <c r="G100" t="s">
-        <v>56</v>
+        <v>35</v>
       </c>
       <c r="J100" s="3" t="s">
-        <v>218</v>
+        <v>64</v>
       </c>
     </row>
     <row r="101" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A101" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="B101" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="C101" t="s">
+        <v>33</v>
+      </c>
+      <c r="D101" t="s">
         <v>34</v>
       </c>
-      <c r="D101" t="s">
-        <v>35</v>
-      </c>
       <c r="E101" t="s">
         <v>11</v>
       </c>
       <c r="F101" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="G101" t="s">
-        <v>51</v>
+        <v>48</v>
+      </c>
+      <c r="I101" s="3">
+        <v>14</v>
       </c>
       <c r="J101" s="3" t="s">
-        <v>218</v>
+        <v>202</v>
       </c>
     </row>
     <row r="102" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A102" t="s">
-        <v>64</v>
+        <v>31</v>
       </c>
       <c r="B102" t="s">
-        <v>80</v>
+        <v>31</v>
       </c>
       <c r="C102" t="s">
+        <v>33</v>
+      </c>
+      <c r="D102" t="s">
         <v>34</v>
       </c>
-      <c r="D102" t="s">
-        <v>35</v>
-      </c>
       <c r="E102" t="s">
         <v>11</v>
       </c>
       <c r="F102" t="s">
-        <v>81</v>
+        <v>46</v>
       </c>
       <c r="G102" t="s">
-        <v>36</v>
+        <v>48</v>
+      </c>
+      <c r="I102" s="3">
+        <v>14</v>
       </c>
       <c r="J102" s="3" t="s">
-        <v>55</v>
+        <v>202</v>
       </c>
     </row>
     <row r="103" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A103" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B103" t="s">
         <v>65</v>
       </c>
       <c r="C103" t="s">
+        <v>33</v>
+      </c>
+      <c r="D103" t="s">
         <v>34</v>
       </c>
-      <c r="D103" t="s">
+      <c r="E103" t="s">
+        <v>11</v>
+      </c>
+      <c r="F103" t="s">
+        <v>24</v>
+      </c>
+      <c r="G103" t="s">
         <v>35</v>
       </c>
-      <c r="E103" t="s">
-        <v>11</v>
-      </c>
-      <c r="F103" t="s">
-        <v>21</v>
-      </c>
-      <c r="G103" t="s">
-        <v>36</v>
-      </c>
       <c r="J103" s="3" t="s">
-        <v>55</v>
+        <v>209</v>
       </c>
     </row>
     <row r="104" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A104" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="B104" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C104" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D104" t="s">
-        <v>35</v>
+        <v>44</v>
       </c>
       <c r="E104" t="s">
         <v>11</v>
       </c>
       <c r="F104" t="s">
-        <v>21</v>
+        <v>51</v>
       </c>
       <c r="G104" t="s">
-        <v>36</v>
+        <v>68</v>
       </c>
       <c r="J104" s="3" t="s">
-        <v>55</v>
+        <v>202</v>
       </c>
     </row>
     <row r="105" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A105" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="B105" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="C105" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D105" t="s">
-        <v>35</v>
+        <v>44</v>
       </c>
       <c r="E105" t="s">
         <v>11</v>
       </c>
       <c r="F105" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="G105" t="s">
-        <v>36</v>
+        <v>48</v>
       </c>
       <c r="J105" s="3" t="s">
-        <v>55</v>
+        <v>41</v>
       </c>
     </row>
     <row r="106" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A106" t="s">
-        <v>31</v>
+        <v>66</v>
       </c>
       <c r="B106" t="s">
-        <v>57</v>
+        <v>66</v>
       </c>
       <c r="C106" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D106" t="s">
-        <v>35</v>
+        <v>44</v>
       </c>
       <c r="E106" t="s">
         <v>11</v>
       </c>
       <c r="F106" t="s">
-        <v>19</v>
+        <v>51</v>
       </c>
       <c r="G106" t="s">
-        <v>36</v>
+        <v>48</v>
       </c>
       <c r="J106" s="3" t="s">
-        <v>67</v>
+        <v>210</v>
       </c>
     </row>
     <row r="107" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A107" t="s">
-        <v>31</v>
+        <v>69</v>
       </c>
       <c r="B107" t="s">
-        <v>31</v>
+        <v>70</v>
       </c>
       <c r="C107" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D107" t="s">
-        <v>35</v>
+        <v>44</v>
       </c>
       <c r="E107" t="s">
         <v>11</v>
       </c>
       <c r="F107" t="s">
-        <v>48</v>
+        <v>76</v>
       </c>
       <c r="G107" t="s">
-        <v>51</v>
-      </c>
-      <c r="I107" s="3">
-        <v>14</v>
+        <v>71</v>
       </c>
       <c r="J107" s="3" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
     </row>
     <row r="108" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A108" t="s">
-        <v>31</v>
+        <v>69</v>
       </c>
       <c r="B108" t="s">
-        <v>31</v>
+        <v>69</v>
       </c>
       <c r="C108" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D108" t="s">
-        <v>35</v>
+        <v>44</v>
       </c>
       <c r="E108" t="s">
         <v>11</v>
       </c>
       <c r="F108" t="s">
-        <v>49</v>
+        <v>76</v>
       </c>
       <c r="G108" t="s">
-        <v>51</v>
-      </c>
-      <c r="I108" s="3">
-        <v>14</v>
+        <v>71</v>
       </c>
       <c r="J108" s="3" t="s">
-        <v>209</v>
+        <v>212</v>
       </c>
     </row>
     <row r="109" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A109" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="B109" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="C109" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D109" t="s">
-        <v>35</v>
+        <v>44</v>
       </c>
       <c r="E109" t="s">
         <v>11</v>
       </c>
       <c r="F109" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="G109" t="s">
-        <v>36</v>
+        <v>48</v>
       </c>
       <c r="J109" s="3" t="s">
-        <v>219</v>
+        <v>213</v>
       </c>
     </row>
     <row r="110" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A110" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="B110" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="C110" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D110" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="E110" t="s">
         <v>11</v>
       </c>
       <c r="F110" t="s">
-        <v>54</v>
+        <v>46</v>
       </c>
       <c r="G110" t="s">
-        <v>71</v>
+        <v>48</v>
       </c>
       <c r="J110" s="3" t="s">
-        <v>209</v>
+        <v>214</v>
       </c>
     </row>
     <row r="111" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A111" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="B111" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="C111" t="s">
+        <v>33</v>
+      </c>
+      <c r="D111" t="s">
         <v>34</v>
       </c>
-      <c r="D111" t="s">
-        <v>47</v>
-      </c>
       <c r="E111" t="s">
         <v>11</v>
       </c>
       <c r="F111" t="s">
-        <v>54</v>
+        <v>45</v>
       </c>
       <c r="G111" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="J111" s="3" t="s">
-        <v>44</v>
+        <v>202</v>
       </c>
     </row>
     <row r="112" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A112" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="B112" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="C112" t="s">
+        <v>33</v>
+      </c>
+      <c r="D112" t="s">
         <v>34</v>
       </c>
-      <c r="D112" t="s">
-        <v>47</v>
-      </c>
       <c r="E112" t="s">
         <v>11</v>
       </c>
       <c r="F112" t="s">
-        <v>54</v>
+        <v>46</v>
       </c>
       <c r="G112" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="J112" s="3" t="s">
-        <v>220</v>
+        <v>202</v>
       </c>
     </row>
     <row r="113" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A113" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B113" t="s">
         <v>73</v>
       </c>
       <c r="C113" t="s">
+        <v>33</v>
+      </c>
+      <c r="D113" t="s">
         <v>34</v>
       </c>
-      <c r="D113" t="s">
-        <v>47</v>
-      </c>
       <c r="E113" t="s">
         <v>11</v>
       </c>
       <c r="F113" t="s">
-        <v>79</v>
+        <v>15</v>
       </c>
       <c r="G113" t="s">
-        <v>74</v>
+        <v>48</v>
       </c>
       <c r="J113" s="3" t="s">
-        <v>221</v>
+        <v>215</v>
       </c>
     </row>
     <row r="114" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A114" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B114" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C114" t="s">
+        <v>33</v>
+      </c>
+      <c r="D114" t="s">
         <v>34</v>
       </c>
-      <c r="D114" t="s">
-        <v>47</v>
-      </c>
       <c r="E114" t="s">
         <v>11</v>
       </c>
       <c r="F114" t="s">
-        <v>79</v>
+        <v>38</v>
       </c>
       <c r="G114" t="s">
-        <v>74</v>
+        <v>48</v>
       </c>
       <c r="J114" s="3" t="s">
-        <v>222</v>
+        <v>202</v>
       </c>
     </row>
     <row r="115" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A115" t="s">
-        <v>75</v>
+        <v>181</v>
       </c>
       <c r="B115" t="s">
-        <v>75</v>
+        <v>181</v>
       </c>
       <c r="C115" t="s">
-        <v>34</v>
+        <v>182</v>
       </c>
       <c r="D115" t="s">
-        <v>47</v>
+        <v>183</v>
       </c>
       <c r="E115" t="s">
         <v>11</v>
       </c>
       <c r="F115" t="s">
+        <v>184</v>
+      </c>
+      <c r="G115" t="s">
+        <v>185</v>
+      </c>
+      <c r="I115" s="3">
         <v>14</v>
       </c>
-      <c r="G115" t="s">
-        <v>51</v>
-      </c>
-      <c r="J115" s="3" t="s">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="116" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A116" t="s">
-        <v>75</v>
-      </c>
-      <c r="B116" t="s">
-        <v>75</v>
-      </c>
-      <c r="C116" t="s">
-        <v>34</v>
-      </c>
-      <c r="D116" t="s">
-        <v>47</v>
-      </c>
-      <c r="E116" t="s">
-        <v>11</v>
-      </c>
-      <c r="F116" t="s">
-        <v>49</v>
-      </c>
-      <c r="G116" t="s">
-        <v>51</v>
-      </c>
-      <c r="J116" s="3" t="s">
-        <v>224</v>
-      </c>
-    </row>
-    <row r="117" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A117" t="s">
-        <v>76</v>
-      </c>
-      <c r="B117" t="s">
-        <v>77</v>
-      </c>
-      <c r="C117" t="s">
-        <v>34</v>
-      </c>
-      <c r="D117" t="s">
-        <v>35</v>
-      </c>
-      <c r="E117" t="s">
-        <v>11</v>
-      </c>
-      <c r="F117" t="s">
-        <v>48</v>
-      </c>
-      <c r="G117" t="s">
-        <v>51</v>
-      </c>
-      <c r="J117" s="3" t="s">
-        <v>209</v>
-      </c>
-    </row>
-    <row r="118" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A118" t="s">
-        <v>76</v>
-      </c>
-      <c r="B118" t="s">
-        <v>77</v>
-      </c>
-      <c r="C118" t="s">
-        <v>34</v>
-      </c>
-      <c r="D118" t="s">
-        <v>35</v>
-      </c>
-      <c r="E118" t="s">
-        <v>11</v>
-      </c>
-      <c r="F118" t="s">
-        <v>49</v>
-      </c>
-      <c r="G118" t="s">
-        <v>51</v>
-      </c>
-      <c r="J118" s="3" t="s">
-        <v>209</v>
-      </c>
-    </row>
-    <row r="119" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A119" t="s">
-        <v>76</v>
-      </c>
-      <c r="B119" t="s">
-        <v>76</v>
-      </c>
-      <c r="C119" t="s">
-        <v>34</v>
-      </c>
-      <c r="D119" t="s">
-        <v>35</v>
-      </c>
-      <c r="E119" t="s">
-        <v>11</v>
-      </c>
-      <c r="F119" t="s">
-        <v>15</v>
-      </c>
-      <c r="G119" t="s">
-        <v>51</v>
-      </c>
-      <c r="J119" s="3" t="s">
-        <v>225</v>
-      </c>
-    </row>
-    <row r="120" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A120" t="s">
-        <v>76</v>
-      </c>
-      <c r="B120" t="s">
-        <v>76</v>
-      </c>
-      <c r="C120" t="s">
-        <v>34</v>
-      </c>
-      <c r="D120" t="s">
-        <v>35</v>
-      </c>
-      <c r="E120" t="s">
-        <v>11</v>
-      </c>
-      <c r="F120" t="s">
-        <v>41</v>
-      </c>
-      <c r="G120" t="s">
-        <v>51</v>
-      </c>
-      <c r="J120" s="3" t="s">
-        <v>209</v>
-      </c>
-    </row>
-    <row r="121" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A121" t="s">
-        <v>69</v>
-      </c>
-      <c r="B121" t="s">
-        <v>206</v>
-      </c>
-      <c r="C121" t="s">
-        <v>226</v>
-      </c>
-      <c r="D121" t="s">
-        <v>10</v>
-      </c>
-      <c r="E121" t="s">
-        <v>11</v>
-      </c>
-      <c r="F121" t="s">
-        <v>19</v>
-      </c>
-      <c r="G121" t="s">
-        <v>12</v>
-      </c>
-      <c r="I121" s="3">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="122" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A122" t="s">
-        <v>32</v>
-      </c>
-      <c r="B122" t="s">
-        <v>206</v>
-      </c>
-      <c r="C122" t="s">
-        <v>226</v>
-      </c>
-      <c r="D122" t="s">
-        <v>10</v>
-      </c>
-      <c r="E122" t="s">
-        <v>11</v>
-      </c>
-      <c r="F122" t="s">
-        <v>19</v>
-      </c>
-      <c r="G122" t="s">
-        <v>12</v>
-      </c>
-      <c r="I122" s="3">
-        <v>48</v>
-      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J122" xr:uid="{EAF16D4A-DA29-4FF0-AC3B-589258931E62}"/>
+  <autoFilter ref="A1:J115" xr:uid="{EAF16D4A-DA29-4FF0-AC3B-589258931E62}"/>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>
 </file>
</xml_diff>